<commit_message>
Update Market Lens paper agent results
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="52" min="1" max="1"/>
@@ -881,7 +881,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
@@ -2463,259 +2462,1473 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="str"/>
-      <c r="B17" s="13" t="str"/>
-      <c r="C17" s="13" t="str"/>
-      <c r="D17" s="13" t="str"/>
-      <c r="E17" s="13" t="str"/>
-      <c r="F17" s="13" t="str"/>
-      <c r="G17" s="13" t="str"/>
-      <c r="H17" s="13" t="str"/>
-      <c r="I17" s="13" t="str"/>
-      <c r="J17" s="13" t="str"/>
-      <c r="K17" s="13" t="str"/>
-      <c r="L17" s="13" t="str"/>
-      <c r="M17" s="13" t="str"/>
-      <c r="N17" s="13" t="str"/>
-      <c r="O17" s="13" t="str"/>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>416.67</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>414.17</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>427.06</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>407.73</v>
+      </c>
+      <c r="I17" s="13" t="n">
+        <v>446.38</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>444.49</v>
+      </c>
+      <c r="K17" s="13" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Price (416.67) retesting broken resistance (427.06) as support. Breakout on 2026-05-29 with 2.3× avg volume. Volume confirmed breakout. Entry at 416.67, stop at 407.73.</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>Existing simulated position remains open.</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>MSFT
+Breakout + Retest
+0.47
+score
+Price
+416.67
+R/R
+3.32x
+Grade
+A
+Quality
+79%
+Buy Zone
+414.17 - 427.06
+Stop
+407.73
+Targets
+446.38 / 444.49
+High-quality watchlist candidate
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Close above 436.15 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 407.73 or setup support fails.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (416.67) retesting broken resistance (427.06) as support. Breakout on 2026-05-29 with 2.3× avg volume. Volume confirmed breakout. Entry at 416.67, stop at 407.73.
+Fib 61.8
+412.14
+Fib Zone
+408.92 - 415.36
+Swing Low
+400.01
+Swing High
+431.76
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="str"/>
-      <c r="B18" s="13" t="str"/>
-      <c r="C18" s="13" t="str"/>
-      <c r="D18" s="13" t="str"/>
-      <c r="E18" s="13" t="str"/>
-      <c r="F18" s="13" t="str"/>
-      <c r="G18" s="13" t="str"/>
-      <c r="H18" s="13" t="str"/>
-      <c r="I18" s="13" t="str"/>
-      <c r="J18" s="13" t="str"/>
-      <c r="K18" s="13" t="str"/>
-      <c r="L18" s="13" t="str"/>
-      <c r="M18" s="13" t="str"/>
-      <c r="N18" s="13" t="str"/>
-      <c r="O18" s="13" t="str"/>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>185.66</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>183.96</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>193.56</v>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>179.16</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>207.96</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>195.18</v>
+      </c>
+      <c r="K18" s="13" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>Price (185.66) retesting broken resistance (193.56) as support. Breakout on 2026-06-01 with 2.0× avg volume. Volume confirmed breakout. Entry at 185.66, stop at 179.16.</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>Existing simulated position remains open.</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>CRM
+Breakout + Retest
+0.41
+score
+Price
+185.66
+R/R
+3.43x
+Grade
+A
+Quality
+78%
+Buy Zone
+183.96 - 193.56
+Stop
+179.16
+Targets
+207.96 / 195.18
+High-quality watchlist candidate
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+Trigger
+Close above 198.09 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 179.16 or setup support fails.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (185.66) retesting broken resistance (193.56) as support. Breakout on 2026-06-01 with 2.0× avg volume. Volume confirmed breakout. Entry at 185.66, stop at 179.16.
+Fib 61.8
+173.16
+Fib Zone
+170.76 - 175.56
+Swing Low
+164.33
+Swing High
+187.44
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="str"/>
-      <c r="B19" s="13" t="str"/>
-      <c r="C19" s="13" t="str"/>
-      <c r="D19" s="13" t="str"/>
-      <c r="E19" s="13" t="str"/>
-      <c r="F19" s="13" t="str"/>
-      <c r="G19" s="13" t="str"/>
-      <c r="H19" s="13" t="str"/>
-      <c r="I19" s="13" t="str"/>
-      <c r="J19" s="13" t="str"/>
-      <c r="K19" s="13" t="str"/>
-      <c r="L19" s="13" t="str"/>
-      <c r="M19" s="13" t="str"/>
-      <c r="N19" s="13" t="str"/>
-      <c r="O19" s="13" t="str"/>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>251.44</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>248.89</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>259.44</v>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>243.61</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>275.27</v>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>265.09</v>
+      </c>
+      <c r="K19" s="13" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>Price (251.44) retesting broken resistance (259.44) as support. Breakout on 2026-06-01 with 1.8× avg volume. Volume confirmed breakout. Entry at 251.44, stop at 243.61.</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>Existing simulated position remains open.</t>
+        </is>
+      </c>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>ADBE
+Breakout + Retest
+0.27
+score
+Price
+251.44
+R/R
+3.04x
+Grade
+C
+Quality
+59%
+Buy Zone
+248.89 - 259.44
+Stop
+243.61
+Targets
+275.27 / 265.09
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+73%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Close above 265.94 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 243.61 or setup support fails.
+Earnings are close; reduce size or wait.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (251.44) retesting broken resistance (259.44) as support. Breakout on 2026-06-01 with 1.8× avg volume. Volume confirmed breakout. Entry at 251.44, stop at 243.61.
+Fib 61.8
+244.48
+Fib Zone
+241.84 - 247.12
+Swing Low
+231.74
+Swing High
+265.09
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="str"/>
-      <c r="B20" s="13" t="str"/>
-      <c r="C20" s="13" t="str"/>
-      <c r="D20" s="13" t="str"/>
-      <c r="E20" s="13" t="str"/>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>307.34</v>
+      </c>
       <c r="F20" s="13" t="str"/>
       <c r="G20" s="13" t="str"/>
-      <c r="H20" s="13" t="str"/>
+      <c r="H20" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I20" s="13" t="str"/>
       <c r="J20" s="13" t="str"/>
-      <c r="K20" s="13" t="str"/>
-      <c r="L20" s="13" t="str"/>
-      <c r="M20" s="13" t="str"/>
-      <c r="N20" s="13" t="str"/>
-      <c r="O20" s="13" t="str"/>
+      <c r="K20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>AAPL
+No Trade
+0.00
+score
+Price
+307.34
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+257.26
+Fib Zone
+255.75 - 258.78
+Swing Low
+242.97
+Swing High
+280.39
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="str"/>
-      <c r="B21" s="13" t="str"/>
-      <c r="C21" s="13" t="str"/>
-      <c r="D21" s="13" t="str"/>
-      <c r="E21" s="13" t="str"/>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>205.1</v>
+      </c>
       <c r="F21" s="13" t="str"/>
       <c r="G21" s="13" t="str"/>
-      <c r="H21" s="13" t="str"/>
+      <c r="H21" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I21" s="13" t="str"/>
       <c r="J21" s="13" t="str"/>
-      <c r="K21" s="13" t="str"/>
-      <c r="L21" s="13" t="str"/>
-      <c r="M21" s="13" t="str"/>
-      <c r="N21" s="13" t="str"/>
-      <c r="O21" s="13" t="str"/>
+      <c r="K21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>NVDA
+No Trade
+0.00
+score
+Price
+205.10
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+210.46
+Fib Zone
+208.33 - 212.59
+Swing Low
+194.51
+Swing High
+236.26
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="str"/>
-      <c r="B22" s="13" t="str"/>
-      <c r="C22" s="13" t="str"/>
-      <c r="D22" s="13" t="str"/>
-      <c r="E22" s="13" t="str"/>
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>385.73</v>
+      </c>
       <c r="F22" s="13" t="str"/>
       <c r="G22" s="13" t="str"/>
-      <c r="H22" s="13" t="str"/>
+      <c r="H22" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I22" s="13" t="str"/>
       <c r="J22" s="13" t="str"/>
-      <c r="K22" s="13" t="str"/>
-      <c r="L22" s="13" t="str"/>
-      <c r="M22" s="13" t="str"/>
-      <c r="N22" s="13" t="str"/>
-      <c r="O22" s="13" t="str"/>
+      <c r="K22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t>AVGO
+No Trade
+0.00
+score
+Price
+385.73
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+28%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+343.19
+Fib Zone
+337.54 - 348.85
+Swing Low
+289.96
+Swing High
+429.31
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="str"/>
-      <c r="B23" s="13" t="str"/>
-      <c r="C23" s="13" t="str"/>
-      <c r="D23" s="13" t="str"/>
-      <c r="E23" s="13" t="str"/>
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>213.68</v>
+      </c>
       <c r="F23" s="13" t="str"/>
       <c r="G23" s="13" t="str"/>
-      <c r="H23" s="13" t="str"/>
+      <c r="H23" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I23" s="13" t="str"/>
       <c r="J23" s="13" t="str"/>
-      <c r="K23" s="13" t="str"/>
-      <c r="L23" s="13" t="str"/>
-      <c r="M23" s="13" t="str"/>
-      <c r="N23" s="13" t="str"/>
-      <c r="O23" s="13" t="str"/>
+      <c r="K23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>ORCL
+No Trade
+0.00
+score
+Price
+213.68
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+175.76
+Fib Zone
+172.62 - 178.89
+Swing Low
+160.33
+Swing High
+200.71
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="str"/>
-      <c r="B24" s="13" t="str"/>
-      <c r="C24" s="13" t="str"/>
-      <c r="D24" s="13" t="str"/>
-      <c r="E24" s="13" t="str"/>
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>112.45</v>
+      </c>
       <c r="F24" s="13" t="str"/>
       <c r="G24" s="13" t="str"/>
-      <c r="H24" s="13" t="str"/>
+      <c r="H24" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I24" s="13" t="str"/>
       <c r="J24" s="13" t="str"/>
-      <c r="K24" s="13" t="str"/>
-      <c r="L24" s="13" t="str"/>
-      <c r="M24" s="13" t="str"/>
-      <c r="N24" s="13" t="str"/>
-      <c r="O24" s="13" t="str"/>
+      <c r="K24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t>NOW
+No Trade
+0.00
+score
+Price
+112.45
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+95.14
+Fib Zone
+93.19 - 97.09
+Swing Low
+85.44
+Swing High
+110.83
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="str"/>
-      <c r="B25" s="13" t="str"/>
-      <c r="C25" s="13" t="str"/>
-      <c r="D25" s="13" t="str"/>
-      <c r="E25" s="13" t="str"/>
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>466.38</v>
+      </c>
       <c r="F25" s="13" t="str"/>
       <c r="G25" s="13" t="str"/>
-      <c r="H25" s="13" t="str"/>
+      <c r="H25" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I25" s="13" t="str"/>
       <c r="J25" s="13" t="str"/>
-      <c r="K25" s="13" t="str"/>
-      <c r="L25" s="13" t="str"/>
-      <c r="M25" s="13" t="str"/>
-      <c r="N25" s="13" t="str"/>
-      <c r="O25" s="13" t="str"/>
+      <c r="K25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t>AMD
+No Trade
+0.00
+score
+Price
+466.38
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+100%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+298.44
+Fib Zone
+291.08 - 305.79
+Swing Low
+192.87
+Swing High
+469.22
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="str"/>
-      <c r="B26" s="13" t="str"/>
-      <c r="C26" s="13" t="str"/>
-      <c r="D26" s="13" t="str"/>
-      <c r="E26" s="13" t="str"/>
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>99.17</v>
+      </c>
       <c r="F26" s="13" t="str"/>
       <c r="G26" s="13" t="str"/>
-      <c r="H26" s="13" t="str"/>
+      <c r="H26" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I26" s="13" t="str"/>
       <c r="J26" s="13" t="str"/>
-      <c r="K26" s="13" t="str"/>
-      <c r="L26" s="13" t="str"/>
-      <c r="M26" s="13" t="str"/>
-      <c r="N26" s="13" t="str"/>
-      <c r="O26" s="13" t="str"/>
+      <c r="K26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M26" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N26" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O26" s="13" t="inlineStr">
+        <is>
+          <t>INTC
+No Trade
+0.00
+score
+Price
+99.17
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+45%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+111.66
+Fib Zone
+109.55 - 113.77
+Swing Low
+102.40
+Swing High
+126.64
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="str"/>
-      <c r="B27" s="13" t="str"/>
-      <c r="C27" s="13" t="str"/>
-      <c r="D27" s="13" t="str"/>
-      <c r="E27" s="13" t="str"/>
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>215.94</v>
+      </c>
       <c r="F27" s="13" t="str"/>
       <c r="G27" s="13" t="str"/>
-      <c r="H27" s="13" t="str"/>
+      <c r="H27" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I27" s="13" t="str"/>
       <c r="J27" s="13" t="str"/>
-      <c r="K27" s="13" t="str"/>
-      <c r="L27" s="13" t="str"/>
-      <c r="M27" s="13" t="str"/>
-      <c r="N27" s="13" t="str"/>
-      <c r="O27" s="13" t="str"/>
+      <c r="K27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M27" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N27" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O27" s="13" t="inlineStr">
+        <is>
+          <t>QCOM
+No Trade
+0.00
+score
+Price
+215.94
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+92%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+216.54
+Fib Zone
+212.06 - 221.02
+Swing Low
+190.32
+Swing High
+258.96
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="str"/>
-      <c r="B28" s="13" t="str"/>
-      <c r="C28" s="13" t="str"/>
-      <c r="D28" s="13" t="str"/>
-      <c r="E28" s="13" t="str"/>
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>285.06</v>
+      </c>
       <c r="F28" s="13" t="str"/>
       <c r="G28" s="13" t="str"/>
-      <c r="H28" s="13" t="str"/>
+      <c r="H28" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I28" s="13" t="str"/>
       <c r="J28" s="13" t="str"/>
-      <c r="K28" s="13" t="str"/>
-      <c r="L28" s="13" t="str"/>
-      <c r="M28" s="13" t="str"/>
-      <c r="N28" s="13" t="str"/>
-      <c r="O28" s="13" t="str"/>
+      <c r="K28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N28" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O28" s="13" t="inlineStr">
+        <is>
+          <t>TXN
+No Trade
+0.00
+score
+Price
+285.06
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+87%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+223.12
+Fib Zone
+220.05 - 226.19
+Swing Low
+184.01
+Swing High
+286.37
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="str"/>
-      <c r="B29" s="13" t="str"/>
-      <c r="C29" s="13" t="str"/>
-      <c r="D29" s="13" t="str"/>
-      <c r="E29" s="13" t="str"/>
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>154.27</v>
+      </c>
       <c r="F29" s="13" t="str"/>
       <c r="G29" s="13" t="str"/>
-      <c r="H29" s="13" t="str"/>
+      <c r="H29" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I29" s="13" t="str"/>
       <c r="J29" s="13" t="str"/>
-      <c r="K29" s="13" t="str"/>
-      <c r="L29" s="13" t="str"/>
-      <c r="M29" s="13" t="str"/>
-      <c r="N29" s="13" t="str"/>
-      <c r="O29" s="13" t="str"/>
+      <c r="K29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M29" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N29" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O29" s="13" t="inlineStr">
+        <is>
+          <t>ANET
+No Trade
+0.00
+score
+Price
+154.27
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+140.01
+Fib Zone
+137.88 - 142.14
+Swing Low
+115.42
+Swing High
+179.80
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="str"/>
-      <c r="B30" s="13" t="str"/>
-      <c r="C30" s="13" t="str"/>
-      <c r="D30" s="13" t="str"/>
-      <c r="E30" s="13" t="str"/>
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>272.05</v>
+      </c>
       <c r="F30" s="13" t="str"/>
       <c r="G30" s="13" t="str"/>
-      <c r="H30" s="13" t="str"/>
+      <c r="H30" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I30" s="13" t="str"/>
       <c r="J30" s="13" t="str"/>
-      <c r="K30" s="13" t="str"/>
-      <c r="L30" s="13" t="str"/>
-      <c r="M30" s="13" t="str"/>
-      <c r="N30" s="13" t="str"/>
-      <c r="O30" s="13" t="str"/>
+      <c r="K30" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M30" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N30" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O30" s="13" t="inlineStr">
+        <is>
+          <t>PANW
+No Trade
+0.00
+score
+Price
+272.05
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+157.16
+Fib Zone
+153.95 - 160.38
+Swing Low
+143.50
+Swing High
+179.27
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="str"/>
-      <c r="B31" s="13" t="str"/>
-      <c r="C31" s="13" t="str"/>
-      <c r="D31" s="13" t="str"/>
-      <c r="E31" s="13" t="str"/>
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>671.02</v>
+      </c>
       <c r="F31" s="13" t="str"/>
       <c r="G31" s="13" t="str"/>
-      <c r="H31" s="13" t="str"/>
+      <c r="H31" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="I31" s="13" t="str"/>
       <c r="J31" s="13" t="str"/>
-      <c r="K31" s="13" t="str"/>
-      <c r="L31" s="13" t="str"/>
-      <c r="M31" s="13" t="str"/>
-      <c r="N31" s="13" t="str"/>
-      <c r="O31" s="13" t="str"/>
+      <c r="K31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M31" s="13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O31" s="13" t="inlineStr">
+        <is>
+          <t>CRWD
+No Trade
+0.00
+score
+Price
+671.02
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+404.00
+Fib Zone
+395.22 - 412.77
+Swing Low
+364.47
+Swing High
+467.95
+No chart generated</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="str"/>
@@ -11937,17 +13150,51 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="str"/>
-      <c r="B3" s="13" t="str"/>
-      <c r="C3" s="13" t="str"/>
-      <c r="D3" s="13" t="str"/>
-      <c r="E3" s="13" t="str"/>
-      <c r="F3" s="13" t="str"/>
-      <c r="G3" s="13" t="str"/>
-      <c r="H3" s="13" t="str"/>
-      <c r="I3" s="13" t="str"/>
-      <c r="J3" s="13" t="str"/>
-      <c r="K3" s="13" t="str"/>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:44:52</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>20260606_104411</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>MSFT CRM ADBE AAPL NVDA AVGO ORCL NOW AMD INTC QCOM TXN ANET PANW CRWD</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>MSFT:HOLD, CRM:HOLD, ADBE:HOLD, AAPL:SKIP, NVDA:SKIP, AVGO:SKIP, ORCL:SKIP, NOW:SKIP, AMD:SKIP, INTC:SKIP, QCOM:SKIP, TXN:SKIP, ANET:SKIP, PANW:SKIP, CRWD:SKIP</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>71829.46000000001</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>28170.54</v>
+      </c>
+      <c r="H3" s="13" t="n">
+        <v>824.88</v>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>agent_results/summaries/market_lens_agent_20260606_104411.md</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>agent_results/screenshots/market_lens_agent_20260606_104411.png</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="str"/>

</xml_diff>

<commit_message>
Retry transient agent scans after reset
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -565,7 +565,7 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Starting Capital (USD)</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Starting Capital (USD)</t>
+          <t>Current Cash (USD)</t>
         </is>
       </c>
       <c r="B4" s="62">
@@ -612,7 +612,7 @@
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Current Cash (USD)</t>
+          <t>Open Exposure (USD)</t>
         </is>
       </c>
       <c r="B5" s="62">
@@ -636,7 +636,7 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Open Exposure (USD)</t>
+          <t>Total Portfolio Value (USD)</t>
         </is>
       </c>
       <c r="B6" s="62">
@@ -660,7 +660,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Total Portfolio Value (USD)</t>
+          <t>Open Risk (USD)</t>
         </is>
       </c>
       <c r="B7" s="62">
@@ -684,7 +684,7 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Open Risk (USD)</t>
+          <t>Closed P/L (USD)</t>
         </is>
       </c>
       <c r="B8" s="62">
@@ -758,7 +758,7 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Closed P/L (USD)</t>
+          <t>Agent Budget (USD)</t>
         </is>
       </c>
       <c r="B11" s="63">
@@ -1241,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="52" min="1" max="1"/>
@@ -1311,45 +1311,6 @@
       <c r="K1" s="48" t="inlineStr">
         <is>
           <t>Screenshot</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:25:39</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>20260606_162505</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
-        <v>100000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>agent_results/summaries/market_lens_agent_20260606_162505.md</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>agent_results/screenshots/market_lens_agent_20260606_162505.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reset and rerun paper agent
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -996,59 +996,168 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-06T16:38:39</t>
+          <t>2026-06-07T01:08:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E2" t="n">
+        <v>215.31</v>
+      </c>
+      <c r="F2" t="n">
+        <v>211.02</v>
+      </c>
+      <c r="G2" t="n">
+        <v>221.56</v>
+      </c>
+      <c r="H2" t="n">
+        <v>205.75</v>
+      </c>
+      <c r="I2" t="n">
+        <v>237.37</v>
+      </c>
+      <c r="J2" t="n">
+        <v>221.56</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Price (215.31) retesting broken resistance (221.56) as support. Breakout on 2026-05-29 with 1.5× avg volume. Volume confirmed breakout. Entry at 215.31, stop at 205.75.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>NTRA
+Breakout + Retest
+0.51
+score
+Price
+215.31
+R/R
+2.31x
+Grade
+A
+Quality
+83%
+Buy Zone
+211.02 - 221.56
+Stop
+205.75
+Targets
+237.37 / 221.56
+High-quality watchlist candidate
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+Trigger
+Close above 227.90 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 205.75 or setup support fails.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (215.31) retesting broken resistance (221.56) as support. Breakout on 2026-05-29 with 1.5× avg volume. Volume confirmed breakout. Entry at 215.31, stop at 205.75.
+Fib 61.8
+198.35
+Fib Zone
+195.71 - 200.98
+Swing Low
+184.00
+Swing High
+221.56
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>CAT</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Breakout + Retest</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D3" t="n">
         <v>0.46</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E3" t="n">
         <v>904.28</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F3" t="n">
         <v>901.0599999999999</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" t="n">
         <v>931.35</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H3" t="n">
         <v>885.92</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I3" t="n">
         <v>976.78</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J3" t="n">
         <v>931.35</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K3" t="n">
         <v>3.95</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Price (904.28) retesting broken resistance (931.35) as support. Breakout on 2026-06-04 with 1.2× avg volume. Entry at 904.28, stop at 885.92.</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>BUY_SIMULATED</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>CAT
 Breakout + Retest
@@ -1103,62 +1212,62 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Breakout + Retest</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>0.45</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>132.47</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F4" t="n">
         <v>131.09</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G4" t="n">
         <v>134.65</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H4" t="n">
         <v>129.31</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I4" t="n">
         <v>140</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J4" t="n">
         <v>134.65</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K4" t="n">
         <v>2.38</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Price (132.47) retesting broken resistance (134.65) as support. Breakout on 2026-06-04 with 1.1× avg volume. Entry at 132.47, stop at 129.31.</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>BUY_SIMULATED</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>C
 Breakout + Retest
@@ -1212,50 +1321,161 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E5" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="F5" t="n">
+        <v>62.05</v>
+      </c>
+      <c r="G5" t="n">
+        <v>64.13</v>
+      </c>
+      <c r="H5" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="I5" t="n">
+        <v>67.23999999999999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>69.36</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Price (62.59) retesting broken resistance (64.13) as support. Breakout on 2026-04-23 with 1.5× avg volume. Volume confirmed breakout. Entry at 62.59, stop at 61.01.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>BKR
+Breakout + Retest
+0.45
+score
+Price
+62.59
+R/R
+4.28x
+Grade
+B
+Quality
+65%
+Buy Zone
+62.05 - 64.13
+Stop
+61.01
+Targets
+67.24 / 69.36
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+45%
+Trigger
+Close above 66.24 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 61.01 or setup support fails.
+Trend quality is not clean.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (62.59) retesting broken resistance (64.13) as support. Breakout on 2026-04-23 with 1.5× avg volume. Volume confirmed breakout. Entry at 62.59, stop at 61.01.
+Fib 61.8
+64.55
+Fib Zone
+64.03 - 65.07
+Swing Low
+62.46
+Swing High
+67.92
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>AMAT</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>453.01</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>AMAT
 No Trade
@@ -1303,50 +1523,323 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>PANW
+No Trade
+0.00
+score
+Price
+272.05
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+157.16
+Fib Zone
+153.95 - 160.38
+Swing Low
+143.50
+Swing High
+179.27
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1929.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>KLAC
+No Trade
+0.00
+score
+Price
+1929.20
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+1745.04
+Fib Zone
+1720.95 - 1769.14
+Swing Low
+1643.90
+Swing High
+1908.67
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>213.68</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>ORCL
+No Trade
+0.00
+score
+Price
+213.68
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+175.76
+Fib Zone
+172.62 - 178.89
+Swing Low
+160.33
+Swing High
+200.71
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>UNH</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>399.47</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr">
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>UNH
 No Trade
@@ -1394,232 +1887,50 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>272.05</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>671.02</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>PANW
-No Trade
-0.00
-score
-Price
-272.05
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-157.16
-Fib Zone
-153.95 - 160.38
-Swing Low
-143.50
-Swing High
-179.27
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>213.68</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>ORCL
-No Trade
-0.00
-score
-Price
-213.68
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-175.76
-Fib Zone
-172.62 - 178.89
-Swing Low
-160.33
-Swing High
-200.71
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CRWD</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>671.02</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>CRWD
 No Trade
@@ -1667,57 +1978,57 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>KLAC</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1929.2</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>864.01</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>KLAC
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>MU
 No Trade
 0.00
 score
 Price
-1929.20
+864.01
 R/R
 0.00x
 Grade
@@ -1742,66 +2053,66 @@
 Institutional liquidity
 100%
 Volume
-Neutral
-50%
+Confirmed
+100%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-1745.04
+505.23
 Fib Zone
-1720.95 - 1769.14
+488.78 - 521.68
 Swing Low
-1643.90
+311.49
 Swing High
-1908.67
+818.67
 No chart generated</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
         <v>211.93</v>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>MS
 No Trade
@@ -1849,57 +2160,57 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>864.01</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="inlineStr">
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>167.04</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>MU
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>NTAP
 No Trade
 0.00
 score
 Price
-864.01
+167.04
 R/R
 0.00x
 Grade
@@ -1925,65 +2236,156 @@
 100%
 Volume
 Confirmed
-100%
+80%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-505.23
+102.11
 Fib Zone
-488.78 - 521.68
+99.95 - 104.26
 Swing Low
-311.49
+94.89
 Swing High
-818.67
+113.78
 No chart generated</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ARW</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>219.09</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>ARW
+No Trade
+0.00
+score
+Price
+219.09
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+166.00
+Fib Zone
+164.02 - 167.97
+Swing Low
+135.29
+Swing High
+215.68
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>GS</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>1038.68</v>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr">
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>GS
 No Trade
@@ -2031,50 +2433,50 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>URI</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>1067.77</v>
       </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="inlineStr">
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>URI
 No Trade
@@ -2122,50 +2524,50 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>SMCI</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>41.64</v>
       </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>SMCI
 No Trade
@@ -2213,50 +2615,141 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>HST
+No Trade
+0.00
+score
+Price
+24.62
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+21.35
+Fib Zone
+21.22 - 21.48
+Swing Low
+20.71
+Swing High
+22.39
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>ASML</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
         <v>1641.74</v>
       </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr">
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>ASML
 No Trade
@@ -2304,50 +2797,141 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1131.42</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>LLY
+No Trade
+0.00
+score
+Price
+1131.42
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+963.67
+Fib Zone
+954.73 - 972.61
+Swing Low
+849.05
+Swing High
+1149.10
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>MPC</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
         <v>262.01</v>
       </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>MPC
 No Trade
@@ -2395,141 +2979,50 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>307.34</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>255.82</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>AAPL
-No Trade
-0.00
-score
-Price
-307.34
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-257.26
-Fib Zone
-255.75 - 258.78
-Swing Low
-242.97
-Swing High
-280.39
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>VLO</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>255.82</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>VLO
 No Trade
@@ -2577,414 +3070,50 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TXN</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>285.06</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>TXN
-No Trade
-0.00
-score
-Price
-285.06
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-87%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-223.12
-Fib Zone
-220.05 - 226.19
-Swing Low
-184.01
-Swing High
-286.37
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>LLY</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1131.42</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>LLY
-No Trade
-0.00
-score
-Price
-1131.42
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-963.67
-Fib Zone
-954.73 - 972.61
-Swing Low
-849.05
-Swing High
-1149.10
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>EQIX</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1080.95</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>EQIX
-No Trade
-0.00
-score
-Price
-1080.95
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-76%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-1058.34
-Fib Zone
-1052.90 - 1063.78
-Swing Low
-1039.56
-Swing High
-1088.73
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PSX</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
-        <v>183.08</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>PSX
-No Trade
-0.00
-score
-Price
-183.08
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-172.07
-Fib Zone
-170.69 - 173.44
-Swing Low
-164.25
-Swing High
-184.72
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>BAC</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
-        <v>53.83</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>BAC
 No Trade
@@ -3032,50 +3161,232 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FRT</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>122.56</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>FRT
+No Trade
+0.00
+score
+Price
+122.56
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+105.71
+Fib Zone
+105.25 - 106.18
+Swing Low
+101.15
+Swing High
+113.09
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DOC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>DOC
+No Trade
+0.00
+score
+Price
+19.79
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+19.58
+Fib Zone
+19.45 - 19.70
+Swing Low
+19.15
+Swing High
+20.27
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>UPS</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>108.54</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr">
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>UPS
 No Trade
@@ -3123,232 +3434,50 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>368.53</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr">
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>272.32</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>GOOGL
-No Trade
-0.00
-score
-Price
-368.53
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-50%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-324.25
-Fib Zone
-321.74 - 326.76
-Swing Low
-272.11
-Swing High
-408.61
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
-        <v>66.90000000000001</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>D
-No Trade
-0.00
-score
-Price
-66.90
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-63.43
-Fib Zone
-63.06 - 63.81
-Swing Low
-60.43
-Swing High
-68.29
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>UNP</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>272.32</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>UNP
 No Trade
@@ -3396,106 +3525,15 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>SLB</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
-        <v>54.87</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>SLB
-No Trade
-0.00
-score
-Price
-54.87
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-54.77
-Fib Zone
-54.33 - 55.21
-Swing Low
-52.45
-Swing High
-58.51
-No chart generated</t>
-        </is>
-      </c>
-    </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-06T16:38:39</t>
+          <t>2026-06-07T01:08:59</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3507,7 +3545,7 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>507.9</v>
+        <v>120.79</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -3531,97 +3569,6 @@
         </is>
       </c>
       <c r="O29" t="inlineStr">
-        <is>
-          <t>LIN
-No Trade
-0.00
-score
-Price
-507.90
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-500.59
-Fib Zone
-498.17 - 503.02
-Swing Low
-488.85
-Swing High
-519.59
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
-        <v>120.79</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
         <is>
           <t>MRK
 No Trade
@@ -3669,57 +3616,57 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PLD</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="n">
-        <v>144.54</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="inlineStr">
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>312.37</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>PLD
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>JPM
 No Trade
 0.00
 score
 Price
-144.54
+312.37
 R/R
 0.00x
 Grade
@@ -3738,190 +3685,8 @@
 Leadership
 100%
 Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-143.13
-Fib Zone
-142.43 - 143.84
-Swing Low
-140.17
-Swing High
-147.93
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>MDLZ</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" t="n">
-        <v>62.04</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>MDLZ
-No Trade
-0.00
-score
-Price
-62.04
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-50%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-58.39
-Fib Zone
-58.07 - 58.71
-Swing Low
-55.79
-Swing High
-62.59
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>AMT</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
-        <v>194.12</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>AMT
-No Trade
-0.00
-score
-Price
-194.12
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
+Constructive
+58%
 Liquidity
 Institutional liquidity
 100%
@@ -3931,61 +3696,61 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-169.98
+299.88
 Fib Zone
-168.75 - 171.21
+298.30 - 301.47
 Swing Low
-163.45
+293.67
 Swing High
-180.56
+309.93
 No chart generated</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
         <v>328</v>
       </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="inlineStr">
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>GE
 No Trade
@@ -4033,57 +3798,57 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>CCI</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>IRM</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
-        <v>94.48999999999999</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="inlineStr">
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>124.66</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>CCI
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>IRM
 No Trade
 0.00
 score
 Price
-94.49
+124.66
 R/R
 0.00x
 Grade
@@ -4102,8 +3867,8 @@
 Leadership
 100%
 Trend Quality
-Clean uptrend
-86%
+Constructive
+68%
 Liquidity
 Institutional liquidity
 100%
@@ -4113,68 +3878,68 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-88.65
+119.20
 Fib Zone
-88.04 - 89.26
+118.31 - 120.10
 Swing Low
-85.47
+110.00
 Swing High
-93.79
+134.09
 No chart generated</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>312.37</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="inlineStr">
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>227.23</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>JPM
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>ABBV
 No Trade
 0.00
 score
 Price
-312.37
+227.23
 R/R
 0.00x
 Grade
@@ -4193,24 +3958,297 @@
 Leadership
 100%
 Trend Quality
-Constructive
-58%
+Clean uptrend
+86%
 Liquidity
 Institutional liquidity
 100%
 Volume
-Neutral
-65%
+Confirmed
+85%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-299.88
+207.66
 Fib Zone
-298.30 - 301.47
+206.26 - 209.05
 Swing Low
-293.67
+200.02
 Swing High
-309.93
+220.01
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>EXR</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>145.31</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>EXR
+No Trade
+0.00
+score
+Price
+145.31
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+140.71
+Fib Zone
+139.90 - 141.52
+Swing Low
+136.69
+Swing High
+147.22
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>39.18</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>HAL
+No Trade
+0.00
+score
+Price
+39.18
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+98%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+45%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+40.48
+Fib Zone
+40.16 - 40.79
+Swing Low
+38.67
+Swing High
+43.41
+No chart generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>56.93</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>OXY
+No Trade
+0.00
+score
+Price
+56.93
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+56.14
+Fib Zone
+55.67 - 56.61
+Swing Low
+52.99
+Swing High
+61.24
 No chart generated</t>
         </is>
       </c>
@@ -4229,7 +4267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4341,7 +4379,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-06T16:38:39</t>
+          <t>2026-06-07T01:08:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4351,41 +4389,41 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>NTRA</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>904.28</v>
+        <v>215.31</v>
       </c>
       <c r="F2" t="n">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>9947.08</v>
+        <v>9904.26</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>9947.08</v>
+        <v>9904.26</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>885.92</v>
+        <v>205.75</v>
       </c>
       <c r="M2" t="n">
-        <v>976.78</v>
+        <v>237.37</v>
       </c>
       <c r="N2" t="n">
-        <v>931.35</v>
+        <v>221.56</v>
       </c>
       <c r="O2" t="n">
-        <v>201.96</v>
+        <v>439.76</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -4394,14 +4432,14 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>agent_results/screenshots/market_lens_agent_20260606_163735.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-06T16:38:39</t>
+          <t>2026-06-07T01:08:59</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4411,50 +4449,170 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>132.47</v>
+        <v>904.28</v>
       </c>
       <c r="F3" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
+        <v>9947.08</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9947.08</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>885.92</v>
+      </c>
+      <c r="M3" t="n">
+        <v>976.78</v>
+      </c>
+      <c r="N3" t="n">
+        <v>931.35</v>
+      </c>
+      <c r="O3" t="n">
+        <v>201.96</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>132.47</v>
+      </c>
+      <c r="F4" t="n">
+        <v>75</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
         <v>9935.25</v>
       </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
         <v>9935.25</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
         <v>129.31</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M4" t="n">
         <v>140</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N4" t="n">
         <v>134.65</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O4" t="n">
         <v>237</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>agent_results/screenshots/market_lens_agent_20260606_163735.png</t>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="F5" t="n">
+        <v>159</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>9951.810000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>9951.809999999999</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="M5" t="n">
+        <v>67.23999999999999</v>
+      </c>
+      <c r="N5" t="n">
+        <v>69.36</v>
+      </c>
+      <c r="O5" t="n">
+        <v>251.22</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4572,31 +4730,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>NTRA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-06T16:38:39</t>
+          <t>2026-06-07T01:08:59</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>904.28</v>
+        <v>215.31</v>
       </c>
       <c r="D2" t="n">
-        <v>904.28</v>
+        <v>215.31</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="F2" t="n">
-        <v>885.92</v>
+        <v>205.75</v>
       </c>
       <c r="G2" t="n">
-        <v>976.78</v>
+        <v>237.37</v>
       </c>
       <c r="H2" t="n">
-        <v>931.35</v>
+        <v>221.56</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -4610,10 +4768,10 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>9947.08</v>
+        <v>9904.26</v>
       </c>
       <c r="M2" t="n">
-        <v>201.96</v>
+        <v>439.76</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -4622,64 +4780,178 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>agent_results/screenshots/market_lens_agent_20260606_163735.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>904.28</v>
+      </c>
+      <c r="D3" t="n">
+        <v>904.28</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F3" t="n">
+        <v>885.92</v>
+      </c>
+      <c r="G3" t="n">
+        <v>976.78</v>
+      </c>
+      <c r="H3" t="n">
+        <v>931.35</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>9947.08</v>
+      </c>
+      <c r="M3" t="n">
+        <v>201.96</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-06T16:38:39</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>132.47</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>132.47</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>75</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F4" t="n">
         <v>129.31</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G4" t="n">
         <v>140</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H4" t="n">
         <v>134.65</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
         <v>9935.25</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M4" t="n">
         <v>237</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>agent_results/screenshots/market_lens_agent_20260606_163735.png</t>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:08:59</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="D5" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="E5" t="n">
+        <v>159</v>
+      </c>
+      <c r="F5" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="G5" t="n">
+        <v>67.23999999999999</v>
+      </c>
+      <c r="H5" t="n">
+        <v>69.36</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>9951.809999999999</v>
+      </c>
+      <c r="M5" t="n">
+        <v>251.22</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
         </is>
       </c>
     </row>
@@ -4773,47 +5045,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-06T16:38:39</t>
+          <t>2026-06-07T01:08:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260606_163735</t>
+          <t>20260607_010640</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CAT C AMAT UNH PANW ORCL CRWD KLAC MS MU GS URI SMCI ASML MPC AAPL VLO TXN LLY EQIX PSX BAC UPS GOOGL D UNP SLB LIN MRK PLD MDLZ AMT GE CCI JPM</t>
+          <t>NTRA CAT C BKR AMAT PANW KLAC ORCL UNH CRWD MU MS NTAP ARW GS URI SMCI HST ASML LLY MPC VLO BAC FRT DOC UPS UNP MRK JPM GE IRM ABBV EXR HAL OXY</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CAT:BUY_SIMULATED, C:BUY_SIMULATED, AMAT:SKIP, UNH:SKIP, PANW:SKIP, ORCL:SKIP, CRWD:SKIP, KLAC:SKIP, MS:SKIP, MU:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, ASML:SKIP, MPC:SKIP, AAPL:SKIP, VLO:SKIP, TXN:SKIP, LLY:SKIP, EQIX:SKIP, PSX:SKIP, BAC:SKIP, UPS:SKIP, GOOGL:SKIP, D:SKIP, UNP:SKIP, SLB:SKIP, LIN:SKIP, MRK:SKIP, PLD:SKIP, MDLZ:SKIP, AMT:SKIP, GE:SKIP, CCI:SKIP, JPM:SKIP</t>
+          <t>NTRA:BUY_SIMULATED, CAT:BUY_SIMULATED, C:BUY_SIMULATED, BKR:BUY_SIMULATED, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, UNH:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, NTAP:SKIP, ARW:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, HST:SKIP, ASML:SKIP, LLY:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, FRT:SKIP, DOC:SKIP, UPS:SKIP, UNP:SKIP, MRK:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, EXR:SKIP, HAL:SKIP, OXY:SKIP</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>80117.67</v>
+        <v>60261.6</v>
       </c>
       <c r="G2" t="n">
-        <v>19882.33</v>
+        <v>39738.4</v>
       </c>
       <c r="H2" t="n">
-        <v>438.96</v>
+        <v>1129.94</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>agent_results/summaries/market_lens_agent_20260606_163735.md</t>
+          <t>agent_results\summaries\market_lens_agent_20260607_010640.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>agent_results/screenshots/market_lens_agent_20260606_163735.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh agent dashboard with charts and context
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Position Events" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -896,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -944,27 +945,27 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Buy Zone Low</t>
+          <t>Buy Zone Low USD</t>
         </is>
       </c>
       <c r="G1" s="30" t="inlineStr">
         <is>
-          <t>Buy Zone High</t>
+          <t>Buy Zone High USD</t>
         </is>
       </c>
       <c r="H1" s="30" t="inlineStr">
         <is>
-          <t>Stop Loss</t>
+          <t>Stop Loss USD</t>
         </is>
       </c>
       <c r="I1" s="30" t="inlineStr">
         <is>
-          <t>Target 1</t>
+          <t>Target 1 USD</t>
         </is>
       </c>
       <c r="J1" s="30" t="inlineStr">
         <is>
-          <t>Target 2</t>
+          <t>Target 2 USD</t>
         </is>
       </c>
       <c r="K1" s="30" t="inlineStr">
@@ -979,63 +980,73 @@
       </c>
       <c r="M1" s="30" t="inlineStr">
         <is>
-          <t>Agent Decision</t>
+          <t>Agent Action</t>
         </is>
       </c>
       <c r="N1" s="30" t="inlineStr">
         <is>
-          <t>Feedback</t>
+          <t>Agent Feedback</t>
         </is>
       </c>
       <c r="O1" s="30" t="inlineStr">
         <is>
           <t>Raw UI Text</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Chart URL</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Selection Context</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Breakout + Retest</t>
+          <t>Liquidity Trap Buy Zone</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.51</v>
+        <v>0.49</v>
       </c>
       <c r="E2" t="n">
-        <v>215.31</v>
+        <v>187.31</v>
       </c>
       <c r="F2" t="n">
-        <v>211.02</v>
+        <v>186.89</v>
       </c>
       <c r="G2" t="n">
-        <v>221.56</v>
+        <v>187.73</v>
       </c>
       <c r="H2" t="n">
-        <v>205.75</v>
+        <v>180.94</v>
       </c>
       <c r="I2" t="n">
-        <v>237.37</v>
+        <v>204.51</v>
       </c>
       <c r="J2" t="n">
-        <v>221.56</v>
+        <v>204.51</v>
       </c>
       <c r="K2" t="n">
-        <v>2.31</v>
+        <v>2.7</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Price (215.31) retesting broken resistance (221.56) as support. Breakout on 2026-05-29 with 1.5× avg volume. Volume confirmed breakout. Entry at 215.31, stop at 205.75.</t>
+          <t>Price (187.31) swept below VAL (182.14) and reclaimed it — liquidity trap confirmed. POC at 184.51 provides structural support. Entry at 187.31, stop at 180.94.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1050,62 +1061,73 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NTRA
-Breakout + Retest
-0.51
+          <t>CVX
+Liquidity Trap Buy Zone
+0.49
 score
 Price
-215.31
+187.31
 R/R
-2.31x
+2.70x
 Grade
-A
+B
 Quality
-83%
+67%
 Buy Zone
-211.02 - 221.56
+186.89 - 187.73
 Stop
-205.75
+180.94
 Targets
-237.37 / 221.56
-High-quality watchlist candidate
+204.51 / 204.51
+Tradable if trigger confirms
 Mixed
 Relative Strength
 Leadership
 100%
 Trend Quality
-Clean uptrend
-86%
+Messy
+18%
 Liquidity
 Institutional liquidity
 100%
 Volume
-Confirmed
-80%
+Neutral
+65%
 Trigger
-Close above 227.90 or reclaim of broken resistance.
+Break above prior-day high at 190.10 after holding buy zone.
 Invalidation
-Exit if price closes below 205.75 or setup support fails.
+Exit if price closes below 180.94 or setup support fails.
+Trend quality is not clean.
 Market regime: Mixed.
 Relative strength: Leadership.
-Price (215.31) retesting broken resistance (221.56) as support. Breakout on 2026-05-29 with 1.5× avg volume. Volume confirmed breakout. Entry at 215.31, stop at 205.75.
+Price (187.31) swept below VAL (182.14) and reclaimed it — liquidity trap confirmed. POC at 184.51 provides structural support. Entry at 187.31, stop at 180.94.
 Fib 61.8
-198.35
+185.91
 Fib Zone
-195.71 - 200.98
+184.85 - 186.97
 Swing Low
-184.00
+177.90
 Swing High
-221.56
+198.87
 Save setup
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>/charts/cvx-scan.png</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1211,11 +1233,21 @@
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>/charts/cat-scan.png</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1320,16 +1352,26 @@
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>/charts/c-scan.png</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1338,32 +1380,32 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="E5" t="n">
-        <v>62.59</v>
+        <v>472.8</v>
       </c>
       <c r="F5" t="n">
-        <v>62.05</v>
+        <v>466.86</v>
       </c>
       <c r="G5" t="n">
-        <v>64.13</v>
+        <v>481.83</v>
       </c>
       <c r="H5" t="n">
-        <v>61.01</v>
+        <v>459.37</v>
       </c>
       <c r="I5" t="n">
-        <v>67.23999999999999</v>
+        <v>504.29</v>
       </c>
       <c r="J5" t="n">
-        <v>69.36</v>
+        <v>528.33</v>
       </c>
       <c r="K5" t="n">
-        <v>4.28</v>
+        <v>4.14</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Price (62.59) retesting broken resistance (64.13) as support. Breakout on 2026-04-23 with 1.5× avg volume. Volume confirmed breakout. Entry at 62.59, stop at 61.01.</t>
+          <t>Price (472.80) retesting broken resistance (481.83) as support. Breakout on 2026-05-28 with 1.8× avg volume. Volume confirmed breakout. Entry at 472.80, stop at 459.37.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1378,24 +1420,24 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>BKR
+          <t>TMO
 Breakout + Retest
-0.45
+0.41
 score
 Price
-62.59
+472.80
 R/R
-4.28x
+4.14x
 Grade
 B
 Quality
-65%
+72%
 Buy Zone
-62.05 - 64.13
+466.86 - 481.83
 Stop
-61.01
+459.37
 Targets
-67.24 / 69.36
+504.29 / 528.33
 Tradable if trigger confirms
 Mixed
 Relative Strength
@@ -1403,79 +1445,207 @@
 100%
 Trend Quality
 Messy
-18%
+28%
 Liquidity
 Institutional liquidity
 100%
 Volume
-Distribution risk
-45%
+Confirmed
+80%
 Trigger
-Close above 66.24 or reclaim of broken resistance.
+Close above 488.65 or reclaim of broken resistance.
 Invalidation
-Exit if price closes below 61.01 or setup support fails.
+Exit if price closes below 459.37 or setup support fails.
 Trend quality is not clean.
-Recent volume shows distribution risk.
 Market regime: Mixed.
 Relative strength: Leadership.
-Price (62.59) retesting broken resistance (64.13) as support. Breakout on 2026-04-23 with 1.5× avg volume. Volume confirmed breakout. Entry at 62.59, stop at 61.01.
+Price (472.80) retesting broken resistance (481.83) as support. Breakout on 2026-05-28 with 1.8× avg volume. Volume confirmed breakout. Entry at 472.80, stop at 459.37.
 Fib 61.8
-64.55
+459.61
 Fib Zone
-64.03 - 65.07
+455.87 - 463.36
 Swing Low
-62.46
+435.27
 Swing High
-67.92
+499.00
 Save setup
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>/charts/tmo-scan.png</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 4.14x; price 472.80 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Swing Low + Volume Support Buy Zone</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="F6" t="n">
+        <v>229.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>233.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>224.36</v>
+      </c>
+      <c r="I6" t="n">
+        <v>233.08</v>
+      </c>
+      <c r="J6" t="n">
+        <v>244.4</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Price is pulling into a recent swing-low support (230.91) that overlaps with a high-volume area (POC at 230.12), creating structural + volume confluence. Liquidity sweep below swing low detected — wick and reclaim. Stop below 224.36.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>JNJ
+Swing Low + Volume Support Buy Zone
+0.41
+score
+Price
+232.77
+R/R
+2.06x
+Grade
+B
+Quality
+77%
+Buy Zone
+229.60 - 233.10
+Stop
+224.36
+Targets
+233.08 / 244.40
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Break above prior-day high at 232.77 after holding buy zone.
+Invalidation
+Exit if price closes below 224.36 or setup support fails.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price is pulling into a recent swing-low support (230.91) that overlaps with a high-volume area (POC at 230.12), creating structural + volume confluence. Liquidity sweep below swing low detected — wick and reclaim. Stop below 224.36.
+Fib 61.8
+224.86
+Fib Zone
+223.76 - 225.95
+Swing Low
+219.11
+Swing High
+234.15
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>/charts/jnj-scan.png</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Swing Low + Volume Support Buy Zone; score 0.41; R/R 2.06x; price 232.77 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>AMAT</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>453.01</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>AMAT
 No Trade
@@ -1519,54 +1689,64 @@
 376.60
 Swing High
 447.89
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>/charts/amat-scan.png</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>PANW</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>272.05</v>
       </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>PANW
 No Trade
@@ -1610,54 +1790,64 @@
 143.50
 Swing High
 179.27
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>/charts/panw-scan.png</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>KLAC</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>1929.2</v>
       </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>KLAC
 No Trade
@@ -1701,54 +1891,64 @@
 1643.90
 Swing High
 1908.67
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>/charts/klac-scan.png</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>213.68</v>
       </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>ORCL
 No Trade
@@ -1792,105 +1992,24 @@
 160.33
 Swing High
 200.71
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>UNH</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>399.47</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>UNH
-No Trade
-0.00
-score
-Price
-399.47
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-312.57
-Fib Zone
-310.10 - 315.05
-Swing Low
-255.97
-Swing High
-404.15
-No chart generated</t>
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>/charts/orcl-scan.png</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1974,14 +2093,24 @@
 364.47
 Swing High
 467.95
-No chart generated</t>
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>/charts/crwd-scan.png</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 671.02 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2065,14 +2194,24 @@
 311.49
 Swing High
 818.67
-No chart generated</t>
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>/charts/mu-scan.png</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 864.01 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2156,19 +2295,29 @@
 151.98
 Swing High
 193.55
-No chart generated</t>
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>/charts/ms-scan.png</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 211.93 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2180,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>167.04</v>
+        <v>41.64</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -2205,12 +2354,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>NTAP
+          <t>SMCI
 No Trade
 0.00
 score
 Price
-167.04
+41.64
 R/R
 0.00x
 Grade
@@ -2236,30 +2385,40 @@
 100%
 Volume
 Confirmed
-80%
+85%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-102.11
+29.63
 Fib Zone
-99.95 - 104.26
+28.83 - 30.42
 Swing Low
-94.89
+25.46
 Swing High
-113.78
-No chart generated</t>
+36.37
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>/charts/smci-scan.png</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ARW</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2271,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>219.09</v>
+        <v>1038.68</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -2295,97 +2454,6 @@
         </is>
       </c>
       <c r="O15" t="inlineStr">
-        <is>
-          <t>ARW
-No Trade
-0.00
-score
-Price
-219.09
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-166.00
-Fib Zone
-164.02 - 167.97
-Swing Low
-135.29
-Swing High
-215.68
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1038.68</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
         <is>
           <t>GS
 No Trade
@@ -2429,61 +2497,71 @@
 777.08
 Swing High
 947.83
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>URI</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>/charts/gs-scan.png</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1067.77</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1641.74</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>URI
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>ASML
 No Trade
 0.00
 score
 Price
-1067.77
+1641.74
 R/R
 0.00x
 Grade
@@ -2513,152 +2591,71 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-819.18
+1455.99
 Fib Zone
-811.20 - 827.15
+1438.81 - 1473.16
 Swing Low
-707.99
+1364.81
 Swing High
-999.06
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SMCI</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+1603.49
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>/charts/asml-scan.png</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>41.64</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="inlineStr">
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>SMCI
-No Trade
-0.00
-score
-Price
-41.64
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-29.63
-Fib Zone
-28.83 - 30.42
-Swing Low
-25.46
-Swing High
-36.37
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>HST</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>24.62</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>HST
 No Trade
@@ -2702,61 +2699,71 @@
 20.71
 Swing High
 22.39
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>ASML</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>/charts/hst-scan.png</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1641.74</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>285.06</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>ASML
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>TXN
 No Trade
 0.00
 score
 Price
-1641.74
+285.06
 R/R
 0.00x
 Grade
@@ -2773,10 +2780,10 @@
 Mixed
 Relative Strength
 Leadership
-100%
+87%
 Trend Quality
-Clean uptrend
-86%
+Constructive
+68%
 Liquidity
 Institutional liquidity
 100%
@@ -2786,152 +2793,71 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-1455.99
+223.12
 Fib Zone
-1438.81 - 1473.16
+220.05 - 226.19
 Swing Low
-1364.81
+184.01
 Swing High
-1603.49
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>LLY</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+286.37
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>/charts/txn-scan.png</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1131.42</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="inlineStr">
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>262.01</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>LLY
-No Trade
-0.00
-score
-Price
-1131.42
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-963.67
-Fib Zone
-954.73 - 972.61
-Swing Low
-849.05
-Swing High
-1149.10
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>MPC</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
-        <v>262.01</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>MPC
 No Trade
@@ -2975,54 +2901,64 @@
 233.25
 Swing High
 264.14
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>/charts/mpc-scan.png</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>VLO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
         <v>255.82</v>
       </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr">
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>VLO
 No Trade
@@ -3066,54 +3002,64 @@
 226.18
 Swing High
 262.50
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>/charts/vlo-scan.png</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>BAC</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
         <v>53.83</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr">
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>BAC
 No Trade
@@ -3157,236 +3103,64 @@
 45.88
 Swing High
 55.11
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>FRT</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>/charts/bac-scan.png</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>122.56</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr">
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>108.54</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>FRT
-No Trade
-0.00
-score
-Price
-122.56
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-105.71
-Fib Zone
-105.25 - 106.18
-Swing Low
-101.15
-Swing High
-113.09
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>DOC</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
-        <v>19.79</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>DOC
-No Trade
-0.00
-score
-Price
-19.79
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-19.58
-Fib Zone
-19.45 - 19.70
-Swing Low
-19.15
-Swing High
-20.27
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>UPS</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>108.54</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>UPS
 No Trade
@@ -3430,54 +3204,367 @@
 92.50
 Swing High
 108.02
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>/charts/ups-scan.png</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>AMH</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>33.27</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>AMH
+No Trade
+0.00
+score
+Price
+33.27
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+28.73
+Fib Zone
+28.57 - 28.89
+Swing Low
+27.22
+Swing High
+31.18
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>/charts/amh-scan.png</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>183.08</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>PSX
+No Trade
+0.00
+score
+Price
+183.08
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+172.07
+Fib Zone
+170.69 - 173.44
+Swing Low
+164.25
+Swing High
+184.72
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>/charts/psx-scan.png</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 183.08 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LAMR</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>151.42</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>LAMR
+No Trade
+0.00
+score
+Price
+151.42
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+148.26
+Fib Zone
+147.52 - 149.00
+Swing Low
+144.11
+Swing High
+154.97
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>/charts/lamr-scan.png</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>UNP</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
         <v>272.32</v>
       </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="inlineStr">
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>UNP
 No Trade
@@ -3521,54 +3608,64 @@
 259.69
 Swing High
 274.97
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>/charts/unp-scan.png</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>MRK</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>120.79</v>
       </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="inlineStr">
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>MRK
 No Trade
@@ -3612,54 +3709,165 @@
 110.94
 Swing High
 123.13
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>/charts/mrk-scan.png</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 120.79 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>UDR</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>UDR
+No Trade
+0.00
+score
+Price
+39.20
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+35.12
+Fib Zone
+34.93 - 35.31
+Swing Low
+33.07
+Swing High
+38.44
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>/charts/udr-scan.png</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 39.20 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>JPM</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
         <v>312.37</v>
       </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="inlineStr">
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>JPM
 No Trade
@@ -3703,54 +3911,64 @@
 293.67
 Swing High
 309.93
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>/charts/jpm-scan.png</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 312.37 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
         <v>328</v>
       </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="inlineStr">
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>GE
 No Trade
@@ -3794,54 +4012,64 @@
 268.91
 Swing High
 310.00
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>/charts/ge-scan.png</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 328.00 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>IRM</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" t="n">
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
         <v>124.66</v>
       </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="inlineStr">
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>IRM
 No Trade
@@ -3885,54 +4113,64 @@
 110.00
 Swing High
 134.09
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>/charts/irm-scan.png</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 124.66 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>ABBV</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
         <v>227.23</v>
       </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="inlineStr">
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>ABBV
 No Trade
@@ -3976,61 +4214,71 @@
 200.02
 Swing High
 220.01
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>EXR</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>/charts/abbv-scan.png</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
-        <v>145.31</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="inlineStr">
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>54.87</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>EXR
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>SLB
 No Trade
 0.00
 score
 Price
-145.31
+54.87
 R/R
 0.00x
 Grade
@@ -4049,79 +4297,89 @@
 Leadership
 100%
 Trend Quality
-Clean uptrend
-86%
+Constructive
+68%
 Liquidity
 Institutional liquidity
 100%
 Volume
-Confirmed
-85%
+Distribution risk
+30%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-140.71
+54.77
 Fib Zone
-139.90 - 141.52
+54.33 - 55.21
 Swing Low
-136.69
+52.45
 Swing High
-147.22
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>HAL</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+58.51
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>/charts/slb-scan.png</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ETN</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
-        <v>39.18</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="inlineStr">
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>395.94</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>HAL
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>ETN
 No Trade
 0.00
 score
 Price
-39.18
+395.94
 R/R
 0.00x
 Grade
@@ -4138,7 +4396,7 @@
 Mixed
 Relative Strength
 Leadership
-98%
+100%
 Trend Quality
 Messy
 18%
@@ -4146,73 +4404,83 @@
 Institutional liquidity
 100%
 Volume
-Distribution risk
-45%
+Confirmed
+80%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-40.48
+376.65
 Fib Zone
-40.16 - 40.79
+372.93 - 380.37
 Swing Low
-38.67
+341.06
 Swing High
-43.41
-No chart generated</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-06-07T01:08:59</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>OXY</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+434.23
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>/charts/etn-scan.png</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 395.94 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>56.93</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="inlineStr">
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>81.67</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>OXY
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>MDT
 No Trade
 0.00
 score
 Price
-56.93
+81.67
 R/R
 0.00x
 Grade
@@ -4231,25 +4499,35 @@
 Leadership
 100%
 Trend Quality
-Messy
-0%
+Constructive
+58%
 Liquidity
 Institutional liquidity
 100%
 Volume
 Confirmed
-80%
+85%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-56.14
+76.25
 Fib Zone
-55.67 - 56.61
+75.75 - 76.75
 Swing Low
-52.99
+74.40
 Swing High
-61.24
-No chart generated</t>
+79.25
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>/charts/mdt-scan.png</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 81.67 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4322,47 +4600,47 @@
       </c>
       <c r="G1" s="36" t="inlineStr">
         <is>
-          <t>Currency Rate</t>
+          <t>USD/ILS</t>
         </is>
       </c>
       <c r="H1" s="36" t="inlineStr">
         <is>
-          <t>Buy Value USD</t>
+          <t>Buy Value</t>
         </is>
       </c>
       <c r="I1" s="36" t="inlineStr">
         <is>
-          <t>Sell Value USD</t>
+          <t>Sell Value</t>
         </is>
       </c>
       <c r="J1" s="36" t="inlineStr">
         <is>
-          <t>Cash Out USD</t>
+          <t>Cash Out</t>
         </is>
       </c>
       <c r="K1" s="36" t="inlineStr">
         <is>
-          <t>Cash In USD</t>
+          <t>Cash In</t>
         </is>
       </c>
       <c r="L1" s="36" t="inlineStr">
         <is>
-          <t>Stop Loss</t>
+          <t>Stop Loss USD</t>
         </is>
       </c>
       <c r="M1" s="36" t="inlineStr">
         <is>
-          <t>Target 1</t>
+          <t>Target 1 USD</t>
         </is>
       </c>
       <c r="N1" s="36" t="inlineStr">
         <is>
-          <t>Target 2</t>
+          <t>Target 2 USD</t>
         </is>
       </c>
       <c r="O1" s="36" t="inlineStr">
         <is>
-          <t>Risk USD</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="P1" s="36" t="inlineStr">
@@ -4373,13 +4651,23 @@
       <c r="Q1" s="36" t="inlineStr">
         <is>
           <t>Screenshot</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Chart URL</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Selection Context</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4389,41 +4677,41 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>215.31</v>
+        <v>187.31</v>
       </c>
       <c r="F2" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>9904.26</v>
+        <v>9927.43</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>9904.26</v>
+        <v>9927.43</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>205.75</v>
+        <v>180.94</v>
       </c>
       <c r="M2" t="n">
-        <v>237.37</v>
+        <v>204.51</v>
       </c>
       <c r="N2" t="n">
-        <v>221.56</v>
+        <v>204.51</v>
       </c>
       <c r="O2" t="n">
-        <v>439.76</v>
+        <v>337.61</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -4432,14 +4720,24 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>/charts/cvx-scan.png</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4492,14 +4790,24 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>/charts/cat-scan.png</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4552,14 +4860,24 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>/charts/c-scan.png</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4569,41 +4887,41 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>62.59</v>
+        <v>472.8</v>
       </c>
       <c r="F5" t="n">
-        <v>159</v>
+        <v>21</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>9951.810000000001</v>
+        <v>9928.800000000001</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>9951.809999999999</v>
+        <v>9928.799999999999</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>61.01</v>
+        <v>459.37</v>
       </c>
       <c r="M5" t="n">
-        <v>67.23999999999999</v>
+        <v>504.29</v>
       </c>
       <c r="N5" t="n">
-        <v>69.36</v>
+        <v>528.33</v>
       </c>
       <c r="O5" t="n">
-        <v>251.22</v>
+        <v>282.03</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -4612,7 +4930,87 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>/charts/tmo-scan.png</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 4.14x; price 472.80 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>224.36</v>
+      </c>
+      <c r="M6" t="n">
+        <v>233.08</v>
+      </c>
+      <c r="N6" t="n">
+        <v>244.4</v>
+      </c>
+      <c r="O6" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>/charts/jnj-scan.png</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Swing Low + Volume Support Buy Zone; score 0.41; R/R 2.06x; price 232.77 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
@@ -4630,7 +5028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4678,17 +5076,17 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Stop Loss</t>
+          <t>Stop Loss USD</t>
         </is>
       </c>
       <c r="G1" s="42" t="inlineStr">
         <is>
-          <t>Target 1</t>
+          <t>Target 1 USD</t>
         </is>
       </c>
       <c r="H1" s="42" t="inlineStr">
         <is>
-          <t>Target 2</t>
+          <t>Target 2 USD</t>
         </is>
       </c>
       <c r="I1" s="42" t="inlineStr">
@@ -4703,17 +5101,17 @@
       </c>
       <c r="K1" s="42" t="inlineStr">
         <is>
-          <t>Unrealized P/L USD</t>
+          <t>Unrealized P/L</t>
         </is>
       </c>
       <c r="L1" s="42" t="inlineStr">
         <is>
-          <t>Exposure USD</t>
+          <t>Exposure</t>
         </is>
       </c>
       <c r="M1" s="42" t="inlineStr">
         <is>
-          <t>Open Risk USD</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="N1" s="42" t="inlineStr">
@@ -4723,38 +5121,48 @@
       </c>
       <c r="O1" s="42" t="inlineStr">
         <is>
-          <t>Last Screenshot</t>
+          <t>Screenshot</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Chart URL</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Selection Context</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>215.31</v>
+        <v>187.31</v>
       </c>
       <c r="D2" t="n">
-        <v>215.31</v>
+        <v>187.31</v>
       </c>
       <c r="E2" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F2" t="n">
-        <v>205.75</v>
+        <v>180.94</v>
       </c>
       <c r="G2" t="n">
-        <v>237.37</v>
+        <v>204.51</v>
       </c>
       <c r="H2" t="n">
-        <v>221.56</v>
+        <v>204.51</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -4768,10 +5176,10 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>9904.26</v>
+        <v>9927.43</v>
       </c>
       <c r="M2" t="n">
-        <v>439.76</v>
+        <v>337.61</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -4780,7 +5188,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>/charts/cvx-scan.png</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
@@ -4792,7 +5210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -4837,7 +5255,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>/charts/cat-scan.png</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
@@ -4849,7 +5277,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -4894,38 +5322,48 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>/charts/c-scan.png</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>62.59</v>
+        <v>472.8</v>
       </c>
       <c r="D5" t="n">
-        <v>62.59</v>
+        <v>472.8</v>
       </c>
       <c r="E5" t="n">
-        <v>159</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>61.01</v>
+        <v>459.37</v>
       </c>
       <c r="G5" t="n">
-        <v>67.23999999999999</v>
+        <v>504.29</v>
       </c>
       <c r="H5" t="n">
-        <v>69.36</v>
+        <v>528.33</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -4939,10 +5377,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>9951.809999999999</v>
+        <v>9928.799999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>251.22</v>
+        <v>282.03</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -4951,7 +5389,84 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>/charts/tmo-scan.png</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 4.14x; price 472.80 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:58:25</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="D6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>224.36</v>
+      </c>
+      <c r="G6" t="n">
+        <v>233.08</v>
+      </c>
+      <c r="H6" t="n">
+        <v>244.4</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="M6" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>/charts/jnj-scan.png</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Swing Low + Volume Support Buy Zone; score 0.41; R/R 2.06x; price 232.77 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
@@ -5013,17 +5528,17 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Cash USD</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="G1" s="48" t="inlineStr">
         <is>
-          <t>Exposure USD</t>
+          <t>Exposure</t>
         </is>
       </c>
       <c r="H1" s="48" t="inlineStr">
         <is>
-          <t>Open Risk USD</t>
+          <t>Open Risk</t>
         </is>
       </c>
       <c r="I1" s="48" t="inlineStr">
@@ -5033,7 +5548,7 @@
       </c>
       <c r="J1" s="48" t="inlineStr">
         <is>
-          <t>Summary File</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="K1" s="48" t="inlineStr">
@@ -5045,47 +5560,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T01:08:59</t>
+          <t>2026-06-07T09:58:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260607_010640</t>
+          <t>20260607_095300</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NTRA CAT C BKR AMAT PANW KLAC ORCL UNH CRWD MU MS NTAP ARW GS URI SMCI HST ASML LLY MPC VLO BAC FRT DOC UPS UNP MRK JPM GE IRM ABBV EXR HAL OXY</t>
+          <t>CVX CAT C TMO JNJ AMAT PANW KLAC ORCL CRWD MU MS SMCI GS ASML HST TXN MPC VLO BAC UPS AMH PSX LAMR UNP MRK UDR JPM GE IRM ABBV SLB ETN MDT</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NTRA:BUY_SIMULATED, CAT:BUY_SIMULATED, C:BUY_SIMULATED, BKR:BUY_SIMULATED, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, UNH:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, NTAP:SKIP, ARW:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, HST:SKIP, ASML:SKIP, LLY:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, FRT:SKIP, DOC:SKIP, UPS:SKIP, UNP:SKIP, MRK:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, EXR:SKIP, HAL:SKIP, OXY:SKIP</t>
+          <t>CVX:BUY_SIMULATED, CAT:BUY_SIMULATED, C:BUY_SIMULATED, TMO:BUY_SIMULATED, JNJ:BUY_SIMULATED, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, SMCI:SKIP, GS:SKIP, ASML:SKIP, HST:SKIP, TXN:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, SLB:SKIP, ETN:SKIP, MDT:SKIP</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>60261.6</v>
+        <v>60028.67</v>
       </c>
       <c r="G2" t="n">
-        <v>39738.4</v>
+        <v>39971.32999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>1129.94</v>
+        <v>1067.01</v>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>agent_results\summaries\market_lens_agent_20260607_010640.md</t>
+          <t>agent_results\summaries\market_lens_agent_20260607_095300.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_010640.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
         </is>
       </c>
     </row>
@@ -5787,4 +6302,95 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Run ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Triggered At</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Trigger Price USD</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Bar High USD</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Bar Low USD</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Bar Close USD</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Cash In</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Stop Loss USD</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Target 1 USD</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Target 2 USD</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Store agent chart images in results
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -1007,7 +1007,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>/charts/cvx-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_cvx.png</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -1127,59 +1127,178 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>ELAN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="E3" t="n">
+        <v>23.63</v>
+      </c>
+      <c r="F3" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="G3" t="n">
+        <v>23.69</v>
+      </c>
+      <c r="H3" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>23.94</v>
+      </c>
+      <c r="J3" t="n">
+        <v>26.29</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (23.40) with confluence at POC, VWAP. Entry at zone low 23.11, stop below fib 78.6% at 22.50.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>BUY_SIMULATED</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ELAN
+Fib 61.8 Confluence Buy Zone
+0.47
+score
+Price
+23.63
+R/R
+5.20x
+Grade
+B
+Quality
+70%
+Buy Zone
+23.11 - 23.69
+Stop
+22.50
+Targets
+23.94 / 26.29
+Tradable if trigger confirms
+Mixed
+Relative Strength
+In line
+50%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+Trigger
+Break above prior-day high at 26.23 after holding buy zone.
+Invalidation
+Exit if price closes below 22.50 or setup support fails.
+Market regime: Mixed.
+Relative strength: In line.
+Price at 61.8% fib retracement (23.40) with confluence at POC, VWAP. Entry at zone low 23.11, stop below fib 78.6% at 22.50.
+Fib 61.8
+23.40
+Fib Zone
+23.11 - 23.69
+Swing Low
+21.62
+Swing High
+26.29
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_elan.png</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>CAT</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Breakout + Retest</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>0.46</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>904.28</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F4" t="n">
         <v>901.0599999999999</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G4" t="n">
         <v>931.35</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H4" t="n">
         <v>885.92</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I4" t="n">
         <v>976.78</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J4" t="n">
         <v>931.35</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K4" t="n">
         <v>3.95</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Price (904.28) retesting broken resistance (931.35) as support. Breakout on 2026-06-04 with 1.2× avg volume. Entry at 904.28, stop at 885.92.</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>BUY_SIMULATED</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>CAT
 Breakout + Retest
@@ -1233,73 +1352,73 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>/charts/cat-scan.png</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_cat.png</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Breakout + Retest</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D5" t="n">
         <v>0.45</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E5" t="n">
         <v>132.47</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F5" t="n">
         <v>131.09</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G5" t="n">
         <v>134.65</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H5" t="n">
         <v>129.31</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I5" t="n">
         <v>140</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J5" t="n">
         <v>134.65</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K5" t="n">
         <v>2.38</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Price (132.47) retesting broken resistance (134.65) as support. Breakout on 2026-06-04 with 1.1× avg volume. Entry at 132.47, stop at 129.31.</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>BUY_SIMULATED</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>C
 Breakout + Retest
@@ -1352,300 +1471,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>/charts/c-scan.png</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_c.png</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>TMO</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Breakout + Retest</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="E5" t="n">
-        <v>472.8</v>
-      </c>
-      <c r="F5" t="n">
-        <v>466.86</v>
-      </c>
-      <c r="G5" t="n">
-        <v>481.83</v>
-      </c>
-      <c r="H5" t="n">
-        <v>459.37</v>
-      </c>
-      <c r="I5" t="n">
-        <v>504.29</v>
-      </c>
-      <c r="J5" t="n">
-        <v>528.33</v>
-      </c>
-      <c r="K5" t="n">
-        <v>4.14</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Price (472.80) retesting broken resistance (481.83) as support. Breakout on 2026-05-28 with 1.8× avg volume. Volume confirmed breakout. Entry at 472.80, stop at 459.37.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>TMO
-Breakout + Retest
-0.41
-score
-Price
-472.80
-R/R
-4.14x
-Grade
-B
-Quality
-72%
-Buy Zone
-466.86 - 481.83
-Stop
-459.37
-Targets
-504.29 / 528.33
-Tradable if trigger confirms
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Messy
-28%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-80%
-Trigger
-Close above 488.65 or reclaim of broken resistance.
-Invalidation
-Exit if price closes below 459.37 or setup support fails.
-Trend quality is not clean.
-Market regime: Mixed.
-Relative strength: Leadership.
-Price (472.80) retesting broken resistance (481.83) as support. Breakout on 2026-05-28 with 1.8× avg volume. Volume confirmed breakout. Entry at 472.80, stop at 459.37.
-Fib 61.8
-459.61
-Fib Zone
-455.87 - 463.36
-Swing Low
-435.27
-Swing High
-499.00
-Save setup
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>/charts/tmo-scan.png</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 4.14x; price 472.80 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Swing Low + Volume Support Buy Zone</t>
+          <t>No Trade</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.41</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="F6" t="n">
-        <v>229.6</v>
-      </c>
-      <c r="G6" t="n">
-        <v>233.1</v>
+        <v>453.01</v>
       </c>
       <c r="H6" t="n">
-        <v>224.36</v>
-      </c>
-      <c r="I6" t="n">
-        <v>233.08</v>
-      </c>
-      <c r="J6" t="n">
-        <v>244.4</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>2.06</v>
+        <v>0</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Price is pulling into a recent swing-low support (230.91) that overlaps with a high-volume area (POC at 230.12), creating structural + volume confluence. Liquidity sweep below swing low detected — wick and reclaim. Stop below 224.36.</t>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>BUY_SIMULATED</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>No Trade result.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
-        <is>
-          <t>JNJ
-Swing Low + Volume Support Buy Zone
-0.41
-score
-Price
-232.77
-R/R
-2.06x
-Grade
-B
-Quality
-77%
-Buy Zone
-229.60 - 233.10
-Stop
-224.36
-Targets
-233.08 / 244.40
-Tradable if trigger confirms
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-Trigger
-Break above prior-day high at 232.77 after holding buy zone.
-Invalidation
-Exit if price closes below 224.36 or setup support fails.
-Market regime: Mixed.
-Relative strength: Leadership.
-Price is pulling into a recent swing-low support (230.91) that overlaps with a high-volume area (POC at 230.12), creating structural + volume confluence. Liquidity sweep below swing low detected — wick and reclaim. Stop below 224.36.
-Fib 61.8
-224.86
-Fib Zone
-223.76 - 225.95
-Swing Low
-219.11
-Swing High
-234.15
-Save setup
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>/charts/jnj-scan.png</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Swing Low + Volume Support Buy Zone; score 0.41; R/R 2.06x; price 232.77 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>AMAT</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>453.01</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
         <is>
           <t>AMAT
 No Trade
@@ -1692,61 +1572,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>/charts/amat-scan.png</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_amat.png</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>PANW</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>272.05</v>
       </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>PANW
 No Trade
@@ -1793,61 +1673,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>/charts/panw-scan.png</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_panw.png</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>KLAC</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>1929.2</v>
       </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>KLAC
 No Trade
@@ -1894,61 +1774,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>/charts/klac-scan.png</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_klac.png</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>213.68</v>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>ORCL
 No Trade
@@ -1995,21 +1875,122 @@
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_orcl.png</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>399.47</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>UNH
+No Trade
+0.00
+score
+Price
+399.47
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+312.57
+Fib Zone
+310.10 - 315.05
+Swing Low
+255.97
+Swing High
+404.15
+Click chart to open full size</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>/charts/orcl-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_unh.png</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 399.47 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2098,7 +2079,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>/charts/crwd-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_crwd.png</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -2110,7 +2091,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2199,7 +2180,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>/charts/mu-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_mu.png</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -2211,7 +2192,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2300,7 +2281,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>/charts/ms-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_ms.png</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -2312,47 +2293,249 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1038.68</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>GS
+No Trade
+0.00
+score
+Price
+1038.68
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+842.30
+Fib Zone
+834.41 - 850.20
+Swing Low
+777.08
+Swing High
+947.83
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_gs.png</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1067.77</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>URI
+No Trade
+0.00
+score
+Price
+1067.77
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+819.18
+Fib Zone
+811.20 - 827.15
+Swing Low
+707.99
+Swing High
+999.06
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_uri.png</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1067.77 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>SMCI</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>41.64</v>
       </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>SMCI
 No Trade
@@ -2399,68 +2582,68 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>/charts/smci-scan.png</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_smci.png</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1038.68</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr">
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>GS
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>HST
 No Trade
 0.00
 score
 Price
-1038.68
+24.62
 R/R
 0.00x
 Grade
@@ -2490,71 +2673,71 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-842.30
+21.35
 Fib Zone
-834.41 - 850.20
+21.22 - 21.48
 Swing Low
-777.08
+20.71
 Swing High
-947.83
+22.39
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>/charts/gs-scan.png</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Agent action: SKIP - No Trade result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_hst.png</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>ASML</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>1641.74</v>
       </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>ASML
 No Trade
@@ -2601,162 +2784,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>/charts/asml-scan.png</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_asml.png</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>HST</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>24.62</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>285.06</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>HST
-No Trade
-0.00
-score
-Price
-24.62
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-21.35
-Fib Zone
-21.22 - 21.48
-Swing Low
-20.71
-Swing High
-22.39
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>/charts/hst-scan.png</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Agent action: SKIP - No Trade result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>TXN</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>285.06</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>TXN
 No Trade
@@ -2803,61 +2885,162 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>/charts/txn-scan.png</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_txn.png</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1131.42</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>No Trade result.</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>LLY
+No Trade
+0.00
+score
+Price
+1131.42
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+963.67
+Fib Zone
+954.73 - 972.61
+Swing Low
+849.05
+Swing High
+1149.10
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_lly.png</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1131.42 | Agent action: SKIP - No Trade result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>MPC</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
         <v>262.01</v>
       </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>MPC
 No Trade
@@ -2904,61 +3087,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>/charts/mpc-scan.png</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_mpc.png</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>VLO</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
         <v>255.82</v>
       </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>VLO
 No Trade
@@ -3005,61 +3188,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>/charts/vlo-scan.png</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_vlo.png</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>BAC</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
         <v>53.83</v>
       </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="inlineStr">
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>BAC
 No Trade
@@ -3106,61 +3289,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>/charts/bac-scan.png</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_bac.png</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>UPS</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
         <v>108.54</v>
       </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="inlineStr">
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>UPS
 No Trade
@@ -3207,61 +3390,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>/charts/ups-scan.png</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_ups.png</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>AMH</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
         <v>33.27</v>
       </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr">
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>AMH
 No Trade
@@ -3308,61 +3491,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>/charts/amh-scan.png</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_amh.png</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>PSX</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
         <v>183.08</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr">
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>PSX
 No Trade
@@ -3409,61 +3592,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>/charts/psx-scan.png</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_psx.png</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 183.08 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>LAMR</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>151.42</v>
       </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr">
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>LAMR
 No Trade
@@ -3510,61 +3693,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>/charts/lamr-scan.png</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_lamr.png</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>UNP</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
         <v>272.32</v>
       </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="inlineStr">
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>UNP
 No Trade
@@ -3611,61 +3794,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>/charts/unp-scan.png</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_unp.png</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>MRK</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
         <v>120.79</v>
       </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="inlineStr">
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>MRK
 No Trade
@@ -3712,61 +3895,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>/charts/mrk-scan.png</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_mrk.png</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 120.79 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>UDR</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
         <v>39.2</v>
       </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="inlineStr">
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>UDR
 No Trade
@@ -3813,61 +3996,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>/charts/udr-scan.png</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_udr.png</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 39.20 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>JPM</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
         <v>312.37</v>
       </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="inlineStr">
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>JPM
 No Trade
@@ -3914,61 +4097,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>/charts/jpm-scan.png</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_jpm.png</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 312.37 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
         <v>328</v>
       </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="inlineStr">
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>GE
 No Trade
@@ -4015,61 +4198,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>/charts/ge-scan.png</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_ge.png</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 328.00 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>IRM</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
         <v>124.66</v>
       </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="inlineStr">
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>IRM
 No Trade
@@ -4116,61 +4299,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>/charts/irm-scan.png</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_irm.png</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 124.66 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>ABBV</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" t="n">
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
         <v>227.23</v>
       </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="inlineStr">
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>ABBV
 No Trade
@@ -4217,61 +4400,61 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>/charts/abbv-scan.png</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_abbv.png</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:10:42</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>SLB</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
         <v>54.87</v>
       </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="inlineStr">
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>No Trade result.</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>SLB
 No Trade
@@ -4318,216 +4501,14 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>/charts/slb-scan.png</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_slb.png</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Agent action: SKIP - No Trade result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>ETN</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
-        <v>395.94</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>ETN
-No Trade
-0.00
-score
-Price
-395.94
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Messy
-18%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-80%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-376.65
-Fib Zone
-372.93 - 380.37
-Swing Low
-341.06
-Swing High
-434.23
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>/charts/etn-scan.png</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 395.94 | Agent action: SKIP - No Trade result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>MDT</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
-        <v>81.67</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>No Trade result.</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>MDT
-No Trade
-0.00
-score
-Price
-81.67
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-58%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-76.25
-Fib Zone
-75.75 - 76.75
-Swing Low
-74.40
-Swing High
-79.25
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>/charts/mdt-scan.png</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 81.67 | Agent action: SKIP - No Trade result.</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4667,7 +4648,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4720,12 +4701,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>/charts/cvx-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_cvx.png</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -4737,7 +4718,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4747,41 +4728,41 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>ELAN</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>904.28</v>
+        <v>23.63</v>
       </c>
       <c r="F3" t="n">
-        <v>11</v>
+        <v>423</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>9947.08</v>
+        <v>9995.49</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>9947.08</v>
+        <v>9995.49</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>885.92</v>
+        <v>22.5</v>
       </c>
       <c r="M3" t="n">
-        <v>976.78</v>
+        <v>23.94</v>
       </c>
       <c r="N3" t="n">
-        <v>931.35</v>
+        <v>26.29</v>
       </c>
       <c r="O3" t="n">
-        <v>201.96</v>
+        <v>477.99</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -4790,24 +4771,24 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>/charts/cat-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_elan.png</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4817,41 +4798,41 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>132.47</v>
+        <v>904.28</v>
       </c>
       <c r="F4" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>9935.25</v>
+        <v>9947.08</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>9935.25</v>
+        <v>9947.08</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>129.31</v>
+        <v>885.92</v>
       </c>
       <c r="M4" t="n">
-        <v>140</v>
+        <v>976.78</v>
       </c>
       <c r="N4" t="n">
-        <v>134.65</v>
+        <v>931.35</v>
       </c>
       <c r="O4" t="n">
-        <v>237</v>
+        <v>201.96</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -4860,24 +4841,24 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>/charts/c-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_cat.png</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4887,41 +4868,41 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>472.8</v>
+        <v>132.47</v>
       </c>
       <c r="F5" t="n">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>9928.800000000001</v>
+        <v>9935.25</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>9928.799999999999</v>
+        <v>9935.25</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>459.37</v>
+        <v>129.31</v>
       </c>
       <c r="M5" t="n">
-        <v>504.29</v>
+        <v>140</v>
       </c>
       <c r="N5" t="n">
-        <v>528.33</v>
+        <v>134.65</v>
       </c>
       <c r="O5" t="n">
-        <v>282.03</v>
+        <v>237</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -4930,87 +4911,17 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>/charts/tmo-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_c.png</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 4.14x; price 472.80 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>224.36</v>
-      </c>
-      <c r="M6" t="n">
-        <v>233.08</v>
-      </c>
-      <c r="N6" t="n">
-        <v>244.4</v>
-      </c>
-      <c r="O6" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>/charts/jnj-scan.png</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Swing Low + Volume Support Buy Zone; score 0.41; R/R 2.06x; price 232.77 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
@@ -5028,7 +4939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -5143,7 +5054,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -5188,12 +5099,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>/charts/cvx-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_cvx.png</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -5205,31 +5116,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>ELAN</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>904.28</v>
+        <v>23.63</v>
       </c>
       <c r="D3" t="n">
-        <v>904.28</v>
+        <v>23.63</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>423</v>
       </c>
       <c r="F3" t="n">
-        <v>885.92</v>
+        <v>22.5</v>
       </c>
       <c r="G3" t="n">
-        <v>976.78</v>
+        <v>23.94</v>
       </c>
       <c r="H3" t="n">
-        <v>931.35</v>
+        <v>26.29</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -5243,10 +5154,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>9947.08</v>
+        <v>9995.49</v>
       </c>
       <c r="M3" t="n">
-        <v>201.96</v>
+        <v>477.99</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -5255,48 +5166,48 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>/charts/cat-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_elan.png</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>132.47</v>
+        <v>904.28</v>
       </c>
       <c r="D4" t="n">
-        <v>132.47</v>
+        <v>904.28</v>
       </c>
       <c r="E4" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>129.31</v>
+        <v>885.92</v>
       </c>
       <c r="G4" t="n">
-        <v>140</v>
+        <v>976.78</v>
       </c>
       <c r="H4" t="n">
-        <v>134.65</v>
+        <v>931.35</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -5310,10 +5221,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>9935.25</v>
+        <v>9947.08</v>
       </c>
       <c r="M4" t="n">
-        <v>237</v>
+        <v>201.96</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -5322,48 +5233,48 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>/charts/c-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_cat.png</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>472.8</v>
+        <v>132.47</v>
       </c>
       <c r="D5" t="n">
-        <v>472.8</v>
+        <v>132.47</v>
       </c>
       <c r="E5" t="n">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>459.37</v>
+        <v>129.31</v>
       </c>
       <c r="G5" t="n">
-        <v>504.29</v>
+        <v>140</v>
       </c>
       <c r="H5" t="n">
-        <v>528.33</v>
+        <v>134.65</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -5377,10 +5288,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>9928.799999999999</v>
+        <v>9935.25</v>
       </c>
       <c r="M5" t="n">
-        <v>282.03</v>
+        <v>237</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -5389,84 +5300,17 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>/charts/tmo-scan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_100446_c.png</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 4.14x; price 472.80 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-06-07T09:58:25</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="D6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>224.36</v>
-      </c>
-      <c r="G6" t="n">
-        <v>233.08</v>
-      </c>
-      <c r="H6" t="n">
-        <v>244.4</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>232.77</v>
-      </c>
-      <c r="M6" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>/charts/jnj-scan.png</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Swing Low + Volume Support Buy Zone; score 0.41; R/R 2.06x; price 232.77 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
         </is>
       </c>
     </row>
@@ -5560,47 +5404,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T09:58:25</t>
+          <t>2026-06-07T10:10:42</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260607_095300</t>
+          <t>20260607_100446</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CVX CAT C TMO JNJ AMAT PANW KLAC ORCL CRWD MU MS SMCI GS ASML HST TXN MPC VLO BAC UPS AMH PSX LAMR UNP MRK UDR JPM GE IRM ABBV SLB ETN MDT</t>
+          <t>CVX ELAN CAT C AMAT PANW KLAC ORCL UNH CRWD MU MS GS URI SMCI HST ASML TXN LLY MPC VLO BAC UPS AMH PSX LAMR UNP MRK UDR JPM GE IRM ABBV SLB</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CVX:BUY_SIMULATED, CAT:BUY_SIMULATED, C:BUY_SIMULATED, TMO:BUY_SIMULATED, JNJ:BUY_SIMULATED, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, SMCI:SKIP, GS:SKIP, ASML:SKIP, HST:SKIP, TXN:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, SLB:SKIP, ETN:SKIP, MDT:SKIP</t>
+          <t>CVX:BUY_SIMULATED, ELAN:BUY_SIMULATED, CAT:BUY_SIMULATED, C:BUY_SIMULATED, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, UNH:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, HST:SKIP, ASML:SKIP, TXN:SKIP, LLY:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, SLB:SKIP</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>60028.67</v>
+        <v>60194.75</v>
       </c>
       <c r="G2" t="n">
-        <v>39971.32999999999</v>
+        <v>39805.25</v>
       </c>
       <c r="H2" t="n">
-        <v>1067.01</v>
+        <v>1254.56</v>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>agent_results\summaries\market_lens_agent_20260607_095300.md</t>
+          <t>agent_results\summaries\market_lens_agent_20260607_100446.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_095300.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reset and rerun Market Lens agent
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -897,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -1003,11 +1003,16 @@
           <t>Selection Context</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Decision JSON</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1051,12 +1056,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>BUY_SIMULATED</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>WATCH: Sector exposure limit would be exceeded by this trade.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1115,19 +1120,24 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_cvx.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_cvx.png</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.57; Factors: Energy | Agent action: WATCH - WATCH: Sector exposure limit would be exceeded by this trade.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 187.73, "buy_zone_low": 186.89, "cash_available": 100000.0, "company_name": "Chevron Corporation", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-07-31T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1311, "estimated_spread": 0.0937, "factor_exposure_after": {"Energy": 9927.43}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_rr": 2.7, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 373046166318.62, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_63D_RESISTANCE", "net_rr": 2.574, "normalized_atr_score": 100.0, "normalized_liquidity_score": 49.74, "normalized_momentum_score": 54.93, "normalized_quality_score": 64.64, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 53 shares, cash 9927.43, risk 337.61.", "previous_resistance": 198.87, "price": 187.31, "prior_high_20": 198.87, "prior_high_63": 212.7613, "reason": "WATCH: Sector exposure limit would be exceeded by this trade.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 9927.43, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.49, "setup_type": "Liquidity Trap Buy Zone", "spread_source": "liquidity_fallback", "stock_score": 0.49, "stop_loss": 180.94, "target_1": 204.51, "target_1_atr_distance": 4.0483, "target_2": 204.51, "target_2_atr_distance": 4.0483, "target_feasibility_status": "OK", "ticker": "CVX", "timestamp": "2026-06-07T14:36:41", "warnings": ["Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1171,12 +1181,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>BUY_SIMULATED</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>WATCH: Gross R/R is valid, but Net R/R 1.20 failed after slippage/spread adjustment.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -1234,19 +1244,24 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_elan.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_elan.png</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.20; Factors: Defensive, Healthcare | Agent action: WATCH - WATCH: Gross R/R is valid, but Net R/R 1.20 failed after slippage/spread adjustment.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 23.69, "buy_zone_low": 23.11, "cash_available": 100000.0, "company_name": "Elanco Animal Health Incorporated", "correlation_warning": false, "days_to_earnings": 43, "earnings_blackout": false, "earnings_date": "2026-08-06T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0354, "estimated_spread": 0.0236, "factor_exposure_after": {"Defensive": 9995.49, "Healthcare": 9995.49}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "WATCH", "gross_rr": 5.2, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 11801993227.14, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_rr": 1.1992, "normalized_atr_score": 100.0, "normalized_liquidity_score": 23.93, "normalized_momentum_score": 43.32, "normalized_quality_score": 51.67, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 423 shares, cash 9995.49, risk 477.99.", "previous_resistance": 26.23, "price": 23.63, "prior_high_20": 26.23, "prior_high_63": 26.29, "reason": "WATCH: Gross R/R is valid, but Net R/R 1.20 failed after slippage/spread adjustment.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 9995.49, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.47, "setup_type": "Fib 61.8 Confluence Buy Zone", "spread_source": "liquidity_fallback", "stock_score": 0.47, "stop_loss": 22.5, "target_1": 23.94, "target_1_atr_distance": 0.268, "target_2": 26.29, "target_2_atr_distance": 2.2992, "target_feasibility_status": "LOW_REWARD_DISTANCE", "ticker": "ELAN", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target 1 is close versus daily ATR.", "Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Sector exposure limit would be exceeded by this trade.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1290,12 +1305,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>BUY_SIMULATED</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>WATCH: Gross R/R is valid, but Net R/R 2.45 failed after slippage/spread adjustment.</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1354,19 +1369,24 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_cat.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_cat.png</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.45; Factors: Industrials | Agent action: WATCH - WATCH: Gross R/R is valid, but Net R/R 2.45 failed after slippage/spread adjustment.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 931.35, "buy_zone_low": 901.06, "cash_available": 100000.0, "company_name": "Caterpillar Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.9495, "estimated_spread": 0.4521, "factor_exposure_after": {"Industrials": 9947.08}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "WATCH", "gross_rr": 3.95, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 416504131881.15, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "BREAKOUT_MEASURED_MOVE", "net_rr": 2.4483, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.89, "normalized_momentum_score": 100, "normalized_quality_score": 87.07, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 11 shares, cash 9947.08, risk 201.96.", "previous_resistance": 946.83, "price": 904.28, "prior_high_20": 946.83, "prior_high_63": 946.83, "reason": "WATCH: Gross R/R is valid, but Net R/R 2.45 failed after slippage/spread adjustment.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 9947.08, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.46, "setup_type": "Breakout + Retest", "spread_source": "liquidity_fallback", "stock_score": 0.46, "stop_loss": 885.92, "target_1": 976.78, "target_1_atr_distance": 2.3939, "target_2": 931.35, "target_2_atr_distance": 0.8938, "target_feasibility_status": "OK", "ticker": "CAT", "timestamp": "2026-06-07T14:36:41", "warnings": ["Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Sector exposure limit would be exceeded by this trade.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1410,12 +1430,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>BUY_SIMULATED</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>WATCH: Gross R/R is valid, but Net R/R 1.38 failed after slippage/spread adjustment.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1473,19 +1493,24 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_c.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_c.png</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.38; Factors: Financials | Agent action: WATCH - WATCH: Gross R/R is valid, but Net R/R 1.38 failed after slippage/spread adjustment.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 134.65, "buy_zone_low": 131.09, "cash_available": 100000.0, "company_name": "Citigroup Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1391, "estimated_spread": 0.0662, "factor_exposure_after": {"Financials": 9935.25}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_rr": 2.38, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 225937781310.85, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "BREAKOUT_MEASURED_MOVE", "net_rr": 1.3816, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.28, "normalized_momentum_score": 100, "normalized_quality_score": 82.68, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 75 shares, cash 9935.25, risk 237.00.", "previous_resistance": 135.67, "price": 132.47, "prior_high_20": 135.67, "prior_high_63": 135.67, "reason": "WATCH: Gross R/R is valid, but Net R/R 1.38 failed after slippage/spread adjustment.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 9935.25, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.45, "setup_type": "Breakout + Retest", "spread_source": "liquidity_fallback", "stock_score": 0.45, "stop_loss": 129.31, "target_1": 140.0, "target_1_atr_distance": 2.1141, "target_2": 134.65, "target_2_atr_distance": 0.6121, "target_feasibility_status": "OK", "ticker": "C", "timestamp": "2026-06-07T14:36:41", "warnings": ["Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Sector exposure limit would be exceeded by this trade.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1522,7 +1547,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1574,19 +1599,24 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_amat.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_amat.png</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Applied Materials, Inc.", "correlation_warning": false, "days_to_earnings": 48, "earnings_blackout": false, "earnings_date": "2026-08-13T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3171, "estimated_spread": 0.2265, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 359671569137.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 98.01, "normalized_liquidity_score": 69.65, "normalized_momentum_score": 100, "normalized_quality_score": 90.4, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 453.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "AMAT", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1623,7 +1653,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1675,19 +1705,24 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_panw.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_panw.png</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Palo Alto Networks, Inc.", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1904, "estimated_spread": 0.136, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 221720740051.27, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.83, "normalized_momentum_score": 100, "normalized_quality_score": 87.95, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.05, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "PANW", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1724,7 +1759,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1776,19 +1811,24 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_klac.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_klac.png</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "KLA Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3504, "estimated_spread": 0.9646, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 252006607134.9, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 97.97, "normalized_liquidity_score": 51.67, "normalized_momentum_score": 100, "normalized_quality_score": 84.99, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1929.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "KLAC", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1825,7 +1865,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1877,19 +1917,24 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_orcl.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_orcl.png</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Oracle Corporation", "correlation_warning": false, "days_to_earnings": 2, "earnings_blackout": true, "earnings_date": "2026-06-10T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1496, "estimated_spread": 0.1068, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 614553488215.21, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 88.94, "normalized_liquidity_score": 75.35, "normalized_momentum_score": 100, "normalized_quality_score": 89.84, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 213.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "ORCL", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable.", "Earnings blackout active."]}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1926,7 +1971,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1978,19 +2023,24 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_unh.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_unh.png</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 399.47 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 399.47 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UnitedHealth Group Incorporated", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2796, "estimated_spread": 0.1997, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 362776446174.45, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.49, "normalized_momentum_score": 100, "normalized_quality_score": 88.45, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 399.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UNH", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2027,7 +2077,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -2079,19 +2129,24 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_crwd.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_crwd.png</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 671.02 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 671.02 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "CrowdStrike Holdings, Inc.", "correlation_warning": false, "days_to_earnings": 61, "earnings_blackout": false, "earnings_date": "2026-09-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4697, "estimated_spread": 0.3355, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 170818090488.37, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 94.37, "normalized_momentum_score": 100, "normalized_quality_score": 98.31, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 671.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "CRWD", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2128,7 +2183,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -2180,19 +2235,24 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_mu.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_mu.png</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 864.01 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 864.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Micron Technology, Inc.", "correlation_warning": false, "days_to_earnings": 12, "earnings_blackout": false, "earnings_date": "2026-06-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.756, "estimated_spread": 0.432, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 974373508417.54, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 70.68, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 92.67, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 864.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MU", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2229,7 +2289,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -2281,19 +2341,24 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_ms.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_ms.png</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 211.93 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 211.93 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Morgan Stanley", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1484, "estimated_spread": 0.106, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 334273959714.43, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.49, "normalized_momentum_score": 100, "normalized_quality_score": 81.85, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 211.93, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MS", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2330,7 +2395,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -2382,19 +2447,24 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_gs.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_gs.png</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Goldman Sachs Group, Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.7271, "estimated_spread": 0.5193, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 306418323889.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 55.06, "normalized_momentum_score": 100, "normalized_quality_score": 86.52, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1038.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "GS", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2431,7 +2501,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2483,19 +2553,24 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_uri.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_uri.png</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1067.77 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1067.77 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Rentals, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.6017, "estimated_spread": 1.0678, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 66892115391.46, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 47.57, "normalized_momentum_score": 100, "normalized_quality_score": 84.27, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1067.77, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "URI", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2532,7 +2607,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2584,19 +2659,24 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_smci.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_smci.png</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Super Micro Computer, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0364, "estimated_spread": 0.0208, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 25043065223.4, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 80.49, "normalized_liquidity_score": 81.49, "normalized_momentum_score": 100, "normalized_quality_score": 89.57, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 41.64, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "SMCI", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2633,7 +2713,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2685,19 +2765,24 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_hst.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_hst.png</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Host Hotels &amp; Resorts", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0369, "estimated_spread": 0.0246, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 16861728472.99, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 26.55, "normalized_momentum_score": 100, "normalized_quality_score": 77.97, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 24.62, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "HST", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2734,7 +2819,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2786,19 +2871,24 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_asml.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_asml.png</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ASML Holding N.V.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.1492, "estimated_spread": 0.8209, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 632755593573.26, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.26, "normalized_momentum_score": 100, "normalized_quality_score": 88.08, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1641.74, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "ASML", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2835,7 +2925,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2887,19 +2977,24 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_txn.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_txn.png</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Texas Instruments Incorporated", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1995, "estimated_spread": 0.1425, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 259431048780.55, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.24, "normalized_momentum_score": 100, "normalized_quality_score": 87.47, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 285.06, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "TXN", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2936,7 +3031,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2988,19 +3083,24 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_lly.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_lly.png</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1131.42 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1131.42 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Eli Lilly and Company", "correlation_warning": false, "days_to_earnings": 42, "earnings_blackout": false, "earnings_date": "2026-08-05T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.792, "estimated_spread": 0.5657, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1008934100764.37, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 66.54, "normalized_momentum_score": 100, "normalized_quality_score": 89.96, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1131.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "LLY", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3037,7 +3137,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -3089,19 +3189,24 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_mpc.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_mpc.png</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Marathon Petroleum Corporation", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1834, "estimated_spread": 0.131, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 76490320587.29, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.86, "normalized_momentum_score": 100, "normalized_quality_score": 85.86, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 262.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MPC", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3138,7 +3243,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -3190,19 +3295,24 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_vlo.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_vlo.png</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Valero Energy Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1791, "estimated_spread": 0.1279, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 75961346466.04, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.08, "normalized_momentum_score": 100, "normalized_quality_score": 87.12, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 255.82, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "VLO", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3239,7 +3349,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3291,19 +3401,24 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_bac.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_bac.png</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Bank of America Corporation", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0377, "estimated_spread": 0.0269, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 382009487737.58, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.83, "normalized_momentum_score": 100, "normalized_quality_score": 85.85, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 53.83, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "BAC", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3340,7 +3455,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3392,19 +3507,24 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_ups.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_ups.png</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Parcel Service, Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.076, "estimated_spread": 0.0543, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 92259682300.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 51.52, "normalized_momentum_score": 99.81, "normalized_quality_score": 85.37, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 108.54, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UPS", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3441,7 +3561,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3493,19 +3613,24 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_amh.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_amh.png</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "American Homes 4 Rent Common Shares of Beneficial Interest", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0499, "estimated_spread": 0.0333, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 11997015510.91, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 17.57, "normalized_momentum_score": 99.67, "normalized_quality_score": 75.12, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 33.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "AMH", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3542,7 +3667,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -3594,19 +3719,24 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_psx.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_psx.png</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 183.08 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 183.08 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Phillips 66", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2746, "estimated_spread": 0.1831, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 73403184195.73, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.74, "normalized_momentum_score": 100, "normalized_quality_score": 82.82, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 183.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "PSX", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3643,7 +3773,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -3695,19 +3825,24 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_lamr.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_lamr.png</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lamar Advertising Company", "correlation_warning": false, "days_to_earnings": 44, "earnings_blackout": false, "earnings_date": "2026-08-07T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2271, "estimated_spread": 0.1514, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 15365359607.61, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 16.68, "normalized_momentum_score": 90.76, "normalized_quality_score": 70.85, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 151.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "LAMR", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3744,7 +3879,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -3796,19 +3931,24 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_unp.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_unp.png</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Union Pacific Corporation", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1906, "estimated_spread": 0.1362, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 161679986512.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.12, "normalized_momentum_score": 80.74, "normalized_quality_score": 79.67, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.32, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UNP", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3845,7 +3985,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3897,19 +4037,24 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_mrk.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_mrk.png</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 120.79 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 120.79 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Merck &amp; Co., Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0846, "estimated_spread": 0.0604, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 298330093349.04, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.49, "normalized_momentum_score": 76.16, "normalized_quality_score": 70.82, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 120.79, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MRK", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3946,7 +4091,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -3998,19 +4143,24 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_udr.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_udr.png</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 39.20 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 39.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UDR, Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0588, "estimated_spread": 0.0392, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 12736693845.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 28.69, "normalized_momentum_score": 81.18, "normalized_quality_score": 70.14, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 39.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UDR", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4047,7 +4197,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4099,19 +4249,24 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_jpm.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_jpm.png</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 312.37 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 312.37 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "JPMorgan Chase &amp; Co.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2187, "estimated_spread": 0.1562, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 836998968557.11, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.16, "normalized_momentum_score": 83.05, "normalized_quality_score": 80.42, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 312.37, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "JPM", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4148,7 +4303,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -4200,19 +4355,24 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_ge.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_ge.png</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 328.00 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 328.00 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "GE Aerospace", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2296, "estimated_spread": 0.164, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 342704109784.0, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 45.05, "normalized_momentum_score": 70.2, "normalized_quality_score": 70.11, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 328.0, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "GE", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4249,7 +4409,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -4301,19 +4461,24 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_irm.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_irm.png</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 124.66 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 124.66 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Iron Mountain", "correlation_warning": false, "days_to_earnings": -26, "earnings_blackout": false, "earnings_date": "2026-04-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.187, "estimated_spread": 0.1247, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 37089427823.03, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 24.67, "normalized_momentum_score": 100, "normalized_quality_score": 77.4, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 124.66, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "IRM", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4350,7 +4515,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -4402,19 +4567,24 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_abbv.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_abbv.png</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "AbbVie Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1591, "estimated_spread": 0.1136, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 401468325167.28, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.65, "normalized_momentum_score": 71.99, "normalized_quality_score": 69.29, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 227.23, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "ABBV", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4451,7 +4621,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>No Trade result.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -4503,12 +4673,17 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_slb.png</t>
+          <t>agent_results\charts\market_lens_agent_20260607_143045_slb.png</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Agent action: SKIP - No Trade result.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Schlumberger Limited", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0384, "estimated_spread": 0.0274, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 82033812262.18, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.73, "normalized_momentum_score": 100, "normalized_quality_score": 87.02, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 54.87, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "SLB", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4644,284 +4819,9 @@
           <t>Selection Context</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CVX</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>187.31</v>
-      </c>
-      <c r="F2" t="n">
-        <v>53</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>9927.43</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>9927.43</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>180.94</v>
-      </c>
-      <c r="M2" t="n">
-        <v>204.51</v>
-      </c>
-      <c r="N2" t="n">
-        <v>204.51</v>
-      </c>
-      <c r="O2" t="n">
-        <v>337.61</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_cvx.png</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ELAN</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="F3" t="n">
-        <v>423</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>9995.49</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>9995.49</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="M3" t="n">
-        <v>23.94</v>
-      </c>
-      <c r="N3" t="n">
-        <v>26.29</v>
-      </c>
-      <c r="O3" t="n">
-        <v>477.99</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_elan.png</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CAT</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>904.28</v>
-      </c>
-      <c r="F4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>9947.08</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>9947.08</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>885.92</v>
-      </c>
-      <c r="M4" t="n">
-        <v>976.78</v>
-      </c>
-      <c r="N4" t="n">
-        <v>931.35</v>
-      </c>
-      <c r="O4" t="n">
-        <v>201.96</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_cat.png</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>132.47</v>
-      </c>
-      <c r="F5" t="n">
-        <v>75</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>9935.25</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>9935.25</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>129.31</v>
-      </c>
-      <c r="M5" t="n">
-        <v>140</v>
-      </c>
-      <c r="N5" t="n">
-        <v>134.65</v>
-      </c>
-      <c r="O5" t="n">
-        <v>237</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_c.png</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Decision JSON</t>
         </is>
       </c>
     </row>
@@ -4939,7 +4839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -5045,272 +4945,9 @@
           <t>Selection Context</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CVX</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>187.31</v>
-      </c>
-      <c r="D2" t="n">
-        <v>187.31</v>
-      </c>
-      <c r="E2" t="n">
-        <v>53</v>
-      </c>
-      <c r="F2" t="n">
-        <v>180.94</v>
-      </c>
-      <c r="G2" t="n">
-        <v>204.51</v>
-      </c>
-      <c r="H2" t="n">
-        <v>204.51</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>9927.43</v>
-      </c>
-      <c r="M2" t="n">
-        <v>337.61</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_cvx.png</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ELAN</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="D3" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="E3" t="n">
-        <v>423</v>
-      </c>
-      <c r="F3" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="G3" t="n">
-        <v>23.94</v>
-      </c>
-      <c r="H3" t="n">
-        <v>26.29</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>9995.49</v>
-      </c>
-      <c r="M3" t="n">
-        <v>477.99</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_elan.png</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CAT</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>904.28</v>
-      </c>
-      <c r="D4" t="n">
-        <v>904.28</v>
-      </c>
-      <c r="E4" t="n">
-        <v>11</v>
-      </c>
-      <c r="F4" t="n">
-        <v>885.92</v>
-      </c>
-      <c r="G4" t="n">
-        <v>976.78</v>
-      </c>
-      <c r="H4" t="n">
-        <v>931.35</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>9947.08</v>
-      </c>
-      <c r="M4" t="n">
-        <v>201.96</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_cat.png</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-07T10:10:42</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>132.47</v>
-      </c>
-      <c r="D5" t="n">
-        <v>132.47</v>
-      </c>
-      <c r="E5" t="n">
-        <v>75</v>
-      </c>
-      <c r="F5" t="n">
-        <v>129.31</v>
-      </c>
-      <c r="G5" t="n">
-        <v>140</v>
-      </c>
-      <c r="H5" t="n">
-        <v>134.65</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>9935.25</v>
-      </c>
-      <c r="M5" t="n">
-        <v>237</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_100446_c.png</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Agent action: BUY_SIMULATED - Price is inside buy zone, R/R is valid, and simulated risk limits allow entry.</t>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Decision JSON</t>
         </is>
       </c>
     </row>
@@ -5328,7 +4965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="52" min="1" max="1"/>
@@ -5400,16 +5037,21 @@
           <t>Screenshot</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Decision JSONL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T10:10:42</t>
+          <t>2026-06-07T14:36:41</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260607_100446</t>
+          <t>20260607_143045</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5422,29 +5064,34 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CVX:BUY_SIMULATED, ELAN:BUY_SIMULATED, CAT:BUY_SIMULATED, C:BUY_SIMULATED, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, UNH:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, HST:SKIP, ASML:SKIP, TXN:SKIP, LLY:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, SLB:SKIP</t>
+          <t>CVX:WATCH, ELAN:WATCH, CAT:WATCH, C:WATCH, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, UNH:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, HST:SKIP, ASML:SKIP, TXN:SKIP, LLY:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, SLB:SKIP</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>60194.75</v>
+        <v>100000</v>
       </c>
       <c r="G2" t="n">
-        <v>39805.25</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1254.56</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>agent_results\summaries\market_lens_agent_20260607_100446.md</t>
+          <t>agent_results\summaries\market_lens_agent_20260607_143045.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_100446.png</t>
+          <t>agent_results\screenshots\market_lens_agent_20260607_143045.png</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>agent_results\decisions\market_lens_agent_20260607_143045.jsonl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine agent risk scoring and reset dashboard run
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -1012,545 +1012,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Liquidity Trap Buy Zone</t>
+          <t>No Trade</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>187.31</v>
-      </c>
-      <c r="F2" t="n">
-        <v>186.89</v>
-      </c>
-      <c r="G2" t="n">
-        <v>187.73</v>
+        <v>453.01</v>
       </c>
       <c r="H2" t="n">
-        <v>180.94</v>
-      </c>
-      <c r="I2" t="n">
-        <v>204.51</v>
-      </c>
-      <c r="J2" t="n">
-        <v>204.51</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Price (187.31) swept below VAL (182.14) and reclaimed it — liquidity trap confirmed. POC at 184.51 provides structural support. Entry at 187.31, stop at 180.94.</t>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>WATCH: Sector exposure limit would be exceeded by this trade.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
-        <is>
-          <t>CVX
-Liquidity Trap Buy Zone
-0.49
-score
-Price
-187.31
-R/R
-2.70x
-Grade
-B
-Quality
-67%
-Buy Zone
-186.89 - 187.73
-Stop
-180.94
-Targets
-204.51 / 204.51
-Tradable if trigger confirms
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Messy
-18%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-Trigger
-Break above prior-day high at 190.10 after holding buy zone.
-Invalidation
-Exit if price closes below 180.94 or setup support fails.
-Trend quality is not clean.
-Market regime: Mixed.
-Relative strength: Leadership.
-Price (187.31) swept below VAL (182.14) and reclaimed it — liquidity trap confirmed. POC at 184.51 provides structural support. Entry at 187.31, stop at 180.94.
-Fib 61.8
-185.91
-Fib Zone
-184.85 - 186.97
-Swing Low
-177.90
-Swing High
-198.87
-Save setup
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_cvx.png</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Liquidity Trap Buy Zone; score 0.49; R/R 2.70x; price 187.31 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.57; Factors: Energy | Agent action: WATCH - WATCH: Sector exposure limit would be exceeded by this trade.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 187.73, "buy_zone_low": 186.89, "cash_available": 100000.0, "company_name": "Chevron Corporation", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-07-31T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1311, "estimated_spread": 0.0937, "factor_exposure_after": {"Energy": 9927.43}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_rr": 2.7, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 373046166318.62, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_63D_RESISTANCE", "net_rr": 2.574, "normalized_atr_score": 100.0, "normalized_liquidity_score": 49.74, "normalized_momentum_score": 54.93, "normalized_quality_score": 64.64, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 53 shares, cash 9927.43, risk 337.61.", "previous_resistance": 198.87, "price": 187.31, "prior_high_20": 198.87, "prior_high_63": 212.7613, "reason": "WATCH: Sector exposure limit would be exceeded by this trade.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 9927.43, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.49, "setup_type": "Liquidity Trap Buy Zone", "spread_source": "liquidity_fallback", "stock_score": 0.49, "stop_loss": 180.94, "target_1": 204.51, "target_1_atr_distance": 4.0483, "target_2": 204.51, "target_2_atr_distance": 4.0483, "target_feasibility_status": "OK", "ticker": "CVX", "timestamp": "2026-06-07T14:36:41", "warnings": ["Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ELAN</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Fib 61.8 Confluence Buy Zone</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="E3" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="F3" t="n">
-        <v>23.11</v>
-      </c>
-      <c r="G3" t="n">
-        <v>23.69</v>
-      </c>
-      <c r="H3" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="I3" t="n">
-        <v>23.94</v>
-      </c>
-      <c r="J3" t="n">
-        <v>26.29</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Price at 61.8% fib retracement (23.40) with confluence at POC, VWAP. Entry at zone low 23.11, stop below fib 78.6% at 22.50.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>WATCH: Gross R/R is valid, but Net R/R 1.20 failed after slippage/spread adjustment.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>ELAN
-Fib 61.8 Confluence Buy Zone
-0.47
-score
-Price
-23.63
-R/R
-5.20x
-Grade
-B
-Quality
-70%
-Buy Zone
-23.11 - 23.69
-Stop
-22.50
-Targets
-23.94 / 26.29
-Tradable if trigger confirms
-Mixed
-Relative Strength
-In line
-50%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-80%
-Trigger
-Break above prior-day high at 26.23 after holding buy zone.
-Invalidation
-Exit if price closes below 22.50 or setup support fails.
-Market regime: Mixed.
-Relative strength: In line.
-Price at 61.8% fib retracement (23.40) with confluence at POC, VWAP. Entry at zone low 23.11, stop below fib 78.6% at 22.50.
-Fib 61.8
-23.40
-Fib Zone
-23.11 - 23.69
-Swing Low
-21.62
-Swing High
-26.29
-Save setup
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_elan.png</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.47; R/R 5.20x; price 23.63 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.20; Factors: Defensive, Healthcare | Agent action: WATCH - WATCH: Gross R/R is valid, but Net R/R 1.20 failed after slippage/spread adjustment.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 23.69, "buy_zone_low": 23.11, "cash_available": 100000.0, "company_name": "Elanco Animal Health Incorporated", "correlation_warning": false, "days_to_earnings": 43, "earnings_blackout": false, "earnings_date": "2026-08-06T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0354, "estimated_spread": 0.0236, "factor_exposure_after": {"Defensive": 9995.49, "Healthcare": 9995.49}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "WATCH", "gross_rr": 5.2, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 11801993227.14, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_rr": 1.1992, "normalized_atr_score": 100.0, "normalized_liquidity_score": 23.93, "normalized_momentum_score": 43.32, "normalized_quality_score": 51.67, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 423 shares, cash 9995.49, risk 477.99.", "previous_resistance": 26.23, "price": 23.63, "prior_high_20": 26.23, "prior_high_63": 26.29, "reason": "WATCH: Gross R/R is valid, but Net R/R 1.20 failed after slippage/spread adjustment.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 9995.49, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.47, "setup_type": "Fib 61.8 Confluence Buy Zone", "spread_source": "liquidity_fallback", "stock_score": 0.47, "stop_loss": 22.5, "target_1": 23.94, "target_1_atr_distance": 0.268, "target_2": 26.29, "target_2_atr_distance": 2.2992, "target_feasibility_status": "LOW_REWARD_DISTANCE", "ticker": "ELAN", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target 1 is close versus daily ATR.", "Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Sector exposure limit would be exceeded by this trade.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>CAT</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Breakout + Retest</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="E4" t="n">
-        <v>904.28</v>
-      </c>
-      <c r="F4" t="n">
-        <v>901.0599999999999</v>
-      </c>
-      <c r="G4" t="n">
-        <v>931.35</v>
-      </c>
-      <c r="H4" t="n">
-        <v>885.92</v>
-      </c>
-      <c r="I4" t="n">
-        <v>976.78</v>
-      </c>
-      <c r="J4" t="n">
-        <v>931.35</v>
-      </c>
-      <c r="K4" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Price (904.28) retesting broken resistance (931.35) as support. Breakout on 2026-06-04 with 1.2× avg volume. Entry at 904.28, stop at 885.92.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>WATCH: Gross R/R is valid, but Net R/R 2.45 failed after slippage/spread adjustment.</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>CAT
-Breakout + Retest
-0.46
-score
-Price
-904.28
-R/R
-3.95x
-Grade
-A
-Quality
-78%
-Buy Zone
-901.06 - 931.35
-Stop
-885.92
-Targets
-976.78 / 931.35
-High-quality watchlist candidate
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-Trigger
-Close above 946.83 or reclaim of broken resistance.
-Invalidation
-Exit if price closes below 885.92 or setup support fails.
-Recent volume shows distribution risk.
-Market regime: Mixed.
-Relative strength: Leadership.
-Price (904.28) retesting broken resistance (931.35) as support. Breakout on 2026-06-04 with 1.2× avg volume. Entry at 904.28, stop at 885.92.
-Fib 61.8
-764.64
-Fib Zone
-757.07 - 772.21
-Swing Low
-661.59
-Swing High
-931.35
-Save setup
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_cat.png</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: Breakout + Retest; score 0.46; R/R 3.95x; price 904.28 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.45; Factors: Industrials | Agent action: WATCH - WATCH: Gross R/R is valid, but Net R/R 2.45 failed after slippage/spread adjustment.</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 931.35, "buy_zone_low": 901.06, "cash_available": 100000.0, "company_name": "Caterpillar Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.9495, "estimated_spread": 0.4521, "factor_exposure_after": {"Industrials": 9947.08}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "WATCH", "gross_rr": 3.95, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 416504131881.15, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "BREAKOUT_MEASURED_MOVE", "net_rr": 2.4483, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.89, "normalized_momentum_score": 100, "normalized_quality_score": 87.07, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 11 shares, cash 9947.08, risk 201.96.", "previous_resistance": 946.83, "price": 904.28, "prior_high_20": 946.83, "prior_high_63": 946.83, "reason": "WATCH: Gross R/R is valid, but Net R/R 2.45 failed after slippage/spread adjustment.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 9947.08, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.46, "setup_type": "Breakout + Retest", "spread_source": "liquidity_fallback", "stock_score": 0.46, "stop_loss": 885.92, "target_1": 976.78, "target_1_atr_distance": 2.3939, "target_2": 931.35, "target_2_atr_distance": 0.8938, "target_feasibility_status": "OK", "ticker": "CAT", "timestamp": "2026-06-07T14:36:41", "warnings": ["Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Sector exposure limit would be exceeded by this trade.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Breakout + Retest</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E5" t="n">
-        <v>132.47</v>
-      </c>
-      <c r="F5" t="n">
-        <v>131.09</v>
-      </c>
-      <c r="G5" t="n">
-        <v>134.65</v>
-      </c>
-      <c r="H5" t="n">
-        <v>129.31</v>
-      </c>
-      <c r="I5" t="n">
-        <v>140</v>
-      </c>
-      <c r="J5" t="n">
-        <v>134.65</v>
-      </c>
-      <c r="K5" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Price (132.47) retesting broken resistance (134.65) as support. Breakout on 2026-06-04 with 1.1× avg volume. Entry at 132.47, stop at 129.31.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>WATCH: Gross R/R is valid, but Net R/R 1.38 failed after slippage/spread adjustment.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>C
-Breakout + Retest
-0.45
-score
-Price
-132.47
-R/R
-2.38x
-Grade
-A
-Quality
-84%
-Buy Zone
-131.09 - 134.65
-Stop
-129.31
-Targets
-140.00 / 134.65
-High-quality watchlist candidate
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-Trigger
-Close above 135.67 or reclaim of broken resistance.
-Invalidation
-Exit if price closes below 129.31 or setup support fails.
-Market regime: Mixed.
-Relative strength: Leadership.
-Price (132.47) retesting broken resistance (134.65) as support. Breakout on 2026-06-04 with 1.1× avg volume. Entry at 132.47, stop at 129.31.
-Fib 61.8
-114.18
-Fib Zone
-113.29 - 115.07
-Swing Low
-101.53
-Swing High
-134.65
-Save setup
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_c.png</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Breakout + Retest; score 0.45; R/R 2.38x; price 132.47 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.38; Factors: Financials | Agent action: WATCH - WATCH: Gross R/R is valid, but Net R/R 1.38 failed after slippage/spread adjustment.</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": 134.65, "buy_zone_low": 131.09, "cash_available": 100000.0, "company_name": "Citigroup Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1391, "estimated_spread": 0.0662, "factor_exposure_after": {"Financials": 9935.25}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_rr": 2.38, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 225937781310.85, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "BREAKOUT_MEASURED_MOVE", "net_rr": 1.3816, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.28, "normalized_momentum_score": 100, "normalized_quality_score": 82.68, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 75 shares, cash 9935.25, risk 237.00.", "previous_resistance": 135.67, "price": 132.47, "prior_high_20": 135.67, "prior_high_63": 135.67, "reason": "WATCH: Gross R/R is valid, but Net R/R 1.38 failed after slippage/spread adjustment.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 9935.25, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.45, "setup_type": "Breakout + Retest", "spread_source": "liquidity_fallback", "stock_score": 0.45, "stop_loss": 129.31, "target_1": 140.0, "target_1_atr_distance": 2.1141, "target_2": 134.65, "target_2_atr_distance": 0.6121, "target_feasibility_status": "OK", "ticker": "C", "timestamp": "2026-06-07T14:36:41", "warnings": ["Sector exposure limit would be exceeded.", "Factor/theme exposure limit would be exceeded.", "WATCH: Sector exposure limit would be exceeded by this trade.", "WATCH: Factor/theme exposure limit would be exceeded by this trade."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>AMAT</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>453.01</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
         <is>
           <t>AMAT
 No Trade
@@ -1597,66 +1099,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_amat.png</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_amat.png</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Applied Materials, Inc.", "correlation_warning": false, "days_to_earnings": 48, "earnings_blackout": false, "earnings_date": "2026-08-13T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3171, "estimated_spread": 0.2265, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 359671569137.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 98.01, "normalized_liquidity_score": 69.65, "normalized_momentum_score": 100, "normalized_quality_score": 90.4, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 453.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "AMAT", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Applied Materials, Inc.", "correlation_warning": false, "days_to_earnings": 48, "earnings_blackout": false, "earnings_date": "2026-08-13T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6342, "estimated_spread": 0.1359, "executable_entry": 453.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 453.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 359671569137.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 453.3951, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 453.7801, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3851, "net_target_1_assumption": -0.2265, "net_target_2_assumption": -0.2265, "normalized_atr_score": 98.01, "normalized_liquidity_score": 69.65, "normalized_momentum_score": 100, "normalized_quality_score": 90.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 453.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 453.01, "ticker": "AMAT", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>PANW</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>272.05</v>
       </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>PANW
 No Trade
@@ -1703,66 +1205,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_panw.png</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_panw.png</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Palo Alto Networks, Inc.", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1904, "estimated_spread": 0.136, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 221720740051.27, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.83, "normalized_momentum_score": 100, "normalized_quality_score": 87.95, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.05, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "PANW", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Palo Alto Networks, Inc.", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3809, "estimated_spread": 0.0816, "executable_entry": 272.05, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.05, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 221720740051.27, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.2812, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.5125, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2312, "net_target_1_assumption": -0.136, "net_target_2_assumption": -0.136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.83, "normalized_momentum_score": 100, "normalized_quality_score": 87.95, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.05, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.05, "ticker": "PANW", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>KLAC</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>1929.2</v>
       </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>KLAC
 No Trade
@@ -1809,66 +1311,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_klac.png</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_klac.png</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "KLA Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3504, "estimated_spread": 0.9646, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 252006607134.9, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 97.97, "normalized_liquidity_score": 51.67, "normalized_momentum_score": 100, "normalized_quality_score": 84.99, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1929.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "KLAC", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "KLA Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.7009, "estimated_spread": 0.5788, "executable_entry": 1929.2, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1929.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 252006607134.9, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1930.8398, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1932.4796, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.6398, "net_target_1_assumption": -0.9646, "net_target_2_assumption": -0.9646, "normalized_atr_score": 97.97, "normalized_liquidity_score": 51.67, "normalized_momentum_score": 100, "normalized_quality_score": 84.99, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1929.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1929.2, "ticker": "KLAC", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>213.68</v>
       </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>ORCL
 No Trade
@@ -1915,172 +1417,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_orcl.png</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_orcl.png</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Oracle Corporation", "correlation_warning": false, "days_to_earnings": 2, "earnings_blackout": true, "earnings_date": "2026-06-10T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1496, "estimated_spread": 0.1068, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 614553488215.21, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 88.94, "normalized_liquidity_score": 75.35, "normalized_momentum_score": 100, "normalized_quality_score": 89.84, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 213.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "ORCL", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable.", "Earnings blackout active."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>UNH</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Oracle Corporation", "correlation_warning": false, "days_to_earnings": 2, "earnings_blackout": true, "earnings_date": "2026-06-10T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2992, "estimated_spread": 0.0641, "executable_entry": 213.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 213.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 614553488215.21, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 213.8616, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 214.0433, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1816, "net_target_1_assumption": -0.1068, "net_target_2_assumption": -0.1068, "normalized_atr_score": 88.94, "normalized_liquidity_score": 75.35, "normalized_momentum_score": 100, "normalized_quality_score": 89.84, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 213.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 213.68, "ticker": "ORCL", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable.", "Earnings blackout active."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>399.47</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>671.02</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>UNH
-No Trade
-0.00
-score
-Price
-399.47
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-312.57
-Fib Zone
-310.10 - 315.05
-Swing Low
-255.97
-Swing High
-404.15
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_unh.png</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 399.47 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UnitedHealth Group Incorporated", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2796, "estimated_spread": 0.1997, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 362776446174.45, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.49, "normalized_momentum_score": 100, "normalized_quality_score": 88.45, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 399.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UNH", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CRWD</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>671.02</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>CRWD
 No Trade
@@ -2127,66 +1523,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_crwd.png</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_crwd.png</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 671.02 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "CrowdStrike Holdings, Inc.", "correlation_warning": false, "days_to_earnings": 61, "earnings_blackout": false, "earnings_date": "2026-09-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4697, "estimated_spread": 0.3355, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 170818090488.37, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 94.37, "normalized_momentum_score": 100, "normalized_quality_score": 98.31, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 671.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "CRWD", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "CrowdStrike Holdings, Inc.", "correlation_warning": false, "days_to_earnings": 61, "earnings_blackout": false, "earnings_date": "2026-09-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.9394, "estimated_spread": 0.2013, "executable_entry": 671.02, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 671.02, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 170818090488.37, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 671.5904, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 672.1607, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.5704, "net_target_1_assumption": -0.3355, "net_target_2_assumption": -0.3355, "normalized_atr_score": 100.0, "normalized_liquidity_score": 94.37, "normalized_momentum_score": 100, "normalized_quality_score": 98.31, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 671.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 671.02, "ticker": "CRWD", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>864.01</v>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr">
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>MU
 No Trade
@@ -2233,66 +1629,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_mu.png</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_mu.png</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 864.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Micron Technology, Inc.", "correlation_warning": false, "days_to_earnings": 12, "earnings_blackout": false, "earnings_date": "2026-06-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.756, "estimated_spread": 0.432, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 974373508417.54, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 70.68, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 92.67, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 864.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MU", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Micron Technology, Inc.", "correlation_warning": false, "days_to_earnings": 12, "earnings_blackout": false, "earnings_date": "2026-06-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3911, "estimated_spread": 0.2592, "executable_entry": 864.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 864.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 974373508417.54, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 864.8351, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 865.6603, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8251, "net_target_1_assumption": -0.4774, "net_target_2_assumption": -0.4774, "normalized_atr_score": 70.68, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 92.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 864.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 864.01, "ticker": "MU", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>211.93</v>
       </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="inlineStr">
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>MS
 No Trade
@@ -2339,66 +1735,278 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_ms.png</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_ms.png</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 211.93 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Morgan Stanley", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1484, "estimated_spread": 0.106, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 334273959714.43, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.49, "normalized_momentum_score": 100, "normalized_quality_score": 81.85, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 211.93, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MS", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Morgan Stanley", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2967, "estimated_spread": 0.0636, "executable_entry": 211.93, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 211.93, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 334273959714.43, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 212.1101, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 212.2903, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1801, "net_target_1_assumption": -0.106, "net_target_2_assumption": -0.106, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.49, "normalized_momentum_score": 100, "normalized_quality_score": 81.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 211.93, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 211.93, "ticker": "MS", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>41.64</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>SMCI
+No Trade
+0.00
+score
+Price
+41.64
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+29.63
+Fib Zone
+28.83 - 30.42
+Swing Low
+25.46
+Swing High
+36.37
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_smci.png</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Super Micro Computer, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.067, "estimated_spread": 0.0125, "executable_entry": 41.64, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 41.64, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 25043065223.4, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 41.6798, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 41.7195, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0398, "net_target_1_assumption": -0.023, "net_target_2_assumption": -0.023, "normalized_atr_score": 80.49, "normalized_liquidity_score": 81.49, "normalized_momentum_score": 100, "normalized_quality_score": 89.57, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 41.64, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 41.64, "ticker": "SMCI", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>904.28</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>CAT
+No Trade
+0.00
+score
+Price
+904.28
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+764.64
+Fib Zone
+757.07 - 772.21
+Swing Low
+661.59
+Swing High
+931.35
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_cat.png</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 904.28 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Caterpillar Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.266, "estimated_spread": 0.2713, "executable_entry": 904.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 904.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 416504131881.15, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 905.0486, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 905.8173, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.7686, "net_target_1_assumption": -0.4521, "net_target_2_assumption": -0.4521, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.89, "normalized_momentum_score": 100, "normalized_quality_score": 87.07, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 904.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 904.28, "ticker": "CAT", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>GS</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>1038.68</v>
       </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>GS
 No Trade
@@ -2445,73 +2053,73 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_gs.png</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_gs.png</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Goldman Sachs Group, Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.7271, "estimated_spread": 0.5193, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 306418323889.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 55.06, "normalized_momentum_score": 100, "normalized_quality_score": 86.52, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1038.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "GS", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>URI</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Goldman Sachs Group, Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.4542, "estimated_spread": 0.3116, "executable_entry": 1038.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1038.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 306418323889.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1039.5629, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1040.4458, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8829, "net_target_1_assumption": -0.5193, "net_target_2_assumption": -0.5193, "normalized_atr_score": 100.0, "normalized_liquidity_score": 55.06, "normalized_momentum_score": 100, "normalized_quality_score": 86.52, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1038.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1038.68, "ticker": "GS", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1067.77</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr">
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1641.74</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>URI
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ASML
 No Trade
 0.00
 score
 Price
-1067.77
+1641.74
 R/R
 0.00x
 Grade
@@ -2541,182 +2149,76 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-819.18
+1455.99
 Fib Zone
-811.20 - 827.15
+1438.81 - 1473.16
 Swing Low
-707.99
+1364.81
 Swing High
-999.06
+1603.49
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_uri.png</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1067.77 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Rentals, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.6017, "estimated_spread": 1.0678, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 66892115391.46, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 47.57, "normalized_momentum_score": 100, "normalized_quality_score": 84.27, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1067.77, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "URI", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SMCI</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_asml.png</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ASML Holding N.V.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.2984, "estimated_spread": 0.4925, "executable_entry": 1641.74, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1641.74, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 632755593573.26, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1643.1355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1644.531, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.3955, "net_target_1_assumption": -0.8209, "net_target_2_assumption": -0.8209, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.26, "normalized_momentum_score": 100, "normalized_quality_score": 88.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1641.74, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1641.74, "ticker": "ASML", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>41.64</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>SMCI
-No Trade
-0.00
-score
-Price
-41.64
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-29.63
-Fib Zone
-28.83 - 30.42
-Swing Low
-25.46
-Swing High
-36.37
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_smci.png</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Super Micro Computer, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0364, "estimated_spread": 0.0208, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 25043065223.4, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 80.49, "normalized_liquidity_score": 81.49, "normalized_momentum_score": 100, "normalized_quality_score": 89.57, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 41.64, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "SMCI", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>HST</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>24.62</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>HST
 No Trade
@@ -2763,73 +2265,73 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_hst.png</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_hst.png</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Host Hotels &amp; Resorts", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0369, "estimated_spread": 0.0246, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 16861728472.99, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 26.55, "normalized_momentum_score": 100, "normalized_quality_score": 77.97, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 24.62, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "HST", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ASML</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Host Hotels &amp; Resorts", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0739, "estimated_spread": 0.0197, "executable_entry": 24.62, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 24.62, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 16861728472.99, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 24.6668, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 24.7136, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0468, "net_target_1_assumption": -0.0283, "net_target_2_assumption": -0.0283, "normalized_atr_score": 100.0, "normalized_liquidity_score": 26.55, "normalized_momentum_score": 100, "normalized_quality_score": 77.97, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 24.62, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 24.62, "ticker": "HST", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1641.74</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="inlineStr">
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>303.28</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>ASML
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>LRCX
 No Trade
 0.00
 score
 Price
-1641.74
+303.28
 R/R
 0.00x
 Grade
@@ -2848,8 +2350,8 @@
 Leadership
 100%
 Trend Quality
-Clean uptrend
-86%
+Constructive
+68%
 Liquidity
 Institutional liquidity
 100%
@@ -2859,76 +2361,76 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-1455.99
+227.21
 Fib Zone
-1438.81 - 1473.16
+223.23 - 231.20
 Swing Low
-1364.81
+198.60
 Swing High
-1603.49
+273.50
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_asml.png</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ASML Holding N.V.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.1492, "estimated_spread": 0.8209, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 632755593573.26, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.26, "normalized_momentum_score": 100, "normalized_quality_score": 88.08, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1641.74, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "ASML", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_lrcx.png</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 303.28 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lam Research Corporation", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4246, "estimated_spread": 0.091, "executable_entry": 303.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 303.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 379263466393.46, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 303.5378, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 303.7956, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2578, "net_target_1_assumption": -0.1516, "net_target_2_assumption": -0.1516, "normalized_atr_score": 95.25, "normalized_liquidity_score": 60.92, "normalized_momentum_score": 100, "normalized_quality_score": 87.09, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 303.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 303.28, "ticker": "LRCX", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>TXN</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>285.06</v>
       </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>TXN
 No Trade
@@ -2975,73 +2477,179 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_txn.png</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_txn.png</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Texas Instruments Incorporated", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1995, "estimated_spread": 0.1425, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["AI / Semiconductors", "Technology"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 259431048780.55, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.24, "normalized_momentum_score": 100, "normalized_quality_score": 87.47, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 285.06, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "TXN", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>LLY</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Texas Instruments Incorporated", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3991, "estimated_spread": 0.0855, "executable_entry": 285.06, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 285.06, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 259431048780.55, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 285.3023, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 285.5446, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2423, "net_target_1_assumption": -0.1425, "net_target_2_assumption": -0.1425, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.24, "normalized_momentum_score": 100, "normalized_quality_score": 87.47, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 285.06, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 285.06, "ticker": "TXN", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1131.42</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>466.38</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>LLY
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>AMD
 No Trade
 0.00
 score
 Price
-1131.42
+466.38
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+100%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+298.44
+Fib Zone
+291.08 - 305.79
+Swing Low
+192.87
+Swing High
+469.22
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_amd.png</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 466.38 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Advanced Micro Devices, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.7509, "estimated_spread": 0.1399, "executable_entry": 466.38, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 466.38, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 760479533978.74, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 466.8254, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 467.2708, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4454, "net_target_1_assumption": -0.2577, "net_target_2_assumption": -0.2577, "normalized_atr_score": 84.31, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 96.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 466.38, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 466.38, "ticker": "AMD", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>132.47</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>C
+No Trade
+0.00
+score
+Price
+132.47
 R/R
 0.00x
 Grade
@@ -3071,76 +2679,182 @@
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-963.67
+114.18
 Fib Zone
-954.73 - 972.61
+113.29 - 115.07
 Swing Low
-849.05
+101.53
 Swing High
-1149.10
+134.65
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_lly.png</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1131.42 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Eli Lilly and Company", "correlation_warning": false, "days_to_earnings": 42, "earnings_blackout": false, "earnings_date": "2026-08-05T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.792, "estimated_spread": 0.5657, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1008934100764.37, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 66.54, "normalized_momentum_score": 100, "normalized_quality_score": 89.96, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1131.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "LLY", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_c.png</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 132.47 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Citigroup Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1855, "estimated_spread": 0.0397, "executable_entry": 132.47, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 132.47, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 225937781310.85, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 132.5826, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 132.6952, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1126, "net_target_1_assumption": -0.0662, "net_target_2_assumption": -0.0662, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.28, "normalized_momentum_score": 100, "normalized_quality_score": 82.68, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 132.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 132.47, "ticker": "C", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>307.34</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>AAPL
+No Trade
+0.00
+score
+Price
+307.34
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+257.26
+Fib Zone
+255.75 - 258.78
+Swing Low
+242.97
+Swing High
+280.39
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_aapl.png</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 307.34 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Apple Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4303, "estimated_spread": 0.0922, "executable_entry": 307.34, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 307.34, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 4514011939253.3, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 307.6012, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 307.8625, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2612, "net_target_1_assumption": -0.1537, "net_target_2_assumption": -0.1537, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 100.0, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 307.34, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 307.34, "ticker": "AAPL", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>MPC</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>262.01</v>
       </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="inlineStr">
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>MPC
 No Trade
@@ -3187,66 +2901,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_mpc.png</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_mpc.png</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Marathon Petroleum Corporation", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1834, "estimated_spread": 0.131, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 76490320587.29, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.86, "normalized_momentum_score": 100, "normalized_quality_score": 85.86, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 262.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MPC", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Marathon Petroleum Corporation", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3668, "estimated_spread": 0.0786, "executable_entry": 262.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 262.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 76490320587.29, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 262.2327, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 262.4554, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2227, "net_target_1_assumption": -0.131, "net_target_2_assumption": -0.131, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.86, "normalized_momentum_score": 100, "normalized_quality_score": 85.86, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 262.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 262.01, "ticker": "MPC", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>VLO</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
         <v>255.82</v>
       </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="inlineStr">
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>VLO
 No Trade
@@ -3293,66 +3007,172 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_vlo.png</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_vlo.png</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Valero Energy Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1791, "estimated_spread": 0.1279, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 75961346466.04, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.08, "normalized_momentum_score": 100, "normalized_quality_score": 87.12, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 255.82, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "VLO", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Valero Energy Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3581, "estimated_spread": 0.0767, "executable_entry": 255.82, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 255.82, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 75961346466.04, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 256.0374, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 256.2549, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2174, "net_target_1_assumption": -0.1279, "net_target_2_assumption": -0.1279, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.08, "normalized_momentum_score": 100, "normalized_quality_score": 87.12, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 255.82, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 255.82, "ticker": "VLO", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>415.17</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>TSM
+No Trade
+0.00
+score
+Price
+415.17
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+381.16
+Fib Zone
+376.97 - 385.35
+Swing Low
+360.55
+Swing High
+414.50
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_tsm.png</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 415.17 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Taiwan Semiconductor Manufacturing Company Limited", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5812, "estimated_spread": 0.1246, "executable_entry": 415.17, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 415.17, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 2153268485619.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 415.5229, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 415.8758, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3529, "net_target_1_assumption": -0.2076, "net_target_2_assumption": -0.2076, "normalized_atr_score": 100.0, "normalized_liquidity_score": 80.47, "normalized_momentum_score": 100, "normalized_quality_score": 94.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 415.17, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 415.17, "ticker": "TSM", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>BAC</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
         <v>53.83</v>
       </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr">
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>BAC
 No Trade
@@ -3399,66 +3219,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_bac.png</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_bac.png</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Bank of America Corporation", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0377, "estimated_spread": 0.0269, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 382009487737.58, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.83, "normalized_momentum_score": 100, "normalized_quality_score": 85.85, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 53.83, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "BAC", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Bank of America Corporation", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0754, "estimated_spread": 0.0161, "executable_entry": 53.83, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 53.83, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 382009487737.58, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 53.8758, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 53.9215, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0458, "net_target_1_assumption": -0.0269, "net_target_2_assumption": -0.0269, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.83, "normalized_momentum_score": 100, "normalized_quality_score": 85.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 53.83, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 53.83, "ticker": "BAC", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>UPS</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
         <v>108.54</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr">
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>UPS
 No Trade
@@ -3505,66 +3325,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_ups.png</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_ups.png</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Parcel Service, Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.076, "estimated_spread": 0.0543, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 92259682300.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 51.52, "normalized_momentum_score": 99.81, "normalized_quality_score": 85.37, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 108.54, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UPS", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Parcel Service, Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.152, "estimated_spread": 0.0326, "executable_entry": 108.54, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 108.54, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 92259682300.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 108.6323, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 108.7245, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0923, "net_target_1_assumption": -0.0543, "net_target_2_assumption": -0.0543, "normalized_atr_score": 100.0, "normalized_liquidity_score": 51.52, "normalized_momentum_score": 99.81, "normalized_quality_score": 85.37, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 108.54, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 108.54, "ticker": "UPS", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>AMH</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
         <v>33.27</v>
       </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr">
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>AMH
 No Trade
@@ -3611,66 +3431,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_amh.png</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_amh.png</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "American Homes 4 Rent Common Shares of Beneficial Interest", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0499, "estimated_spread": 0.0333, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 11997015510.91, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 17.57, "normalized_momentum_score": 99.67, "normalized_quality_score": 75.12, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 33.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "AMH", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "American Homes 4 Rent Common Shares of Beneficial Interest", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0998, "estimated_spread": 0.0266, "executable_entry": 33.27, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 33.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 11997015510.91, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 33.3332, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 33.3964, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0632, "net_target_1_assumption": -0.0383, "net_target_2_assumption": -0.0383, "normalized_atr_score": 100.0, "normalized_liquidity_score": 17.57, "normalized_momentum_score": 99.67, "normalized_quality_score": 75.12, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 33.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 33.27, "ticker": "AMH", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>PSX</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" t="n">
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
         <v>183.08</v>
       </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="inlineStr">
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>PSX
 No Trade
@@ -3717,66 +3537,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_psx.png</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_psx.png</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 183.08 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Phillips 66", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2746, "estimated_spread": 0.1831, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 73403184195.73, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.74, "normalized_momentum_score": 100, "normalized_quality_score": 82.82, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 183.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "PSX", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Phillips 66", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5492, "estimated_spread": 0.1465, "executable_entry": 183.08, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 183.08, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 73403184195.73, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 183.4279, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 183.7757, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3479, "net_target_1_assumption": -0.2105, "net_target_2_assumption": -0.2105, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.74, "normalized_momentum_score": 100, "normalized_quality_score": 82.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 183.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 183.08, "ticker": "PSX", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>LAMR</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
         <v>151.42</v>
       </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="inlineStr">
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>LAMR
 No Trade
@@ -3823,66 +3643,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_lamr.png</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_lamr.png</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lamar Advertising Company", "correlation_warning": false, "days_to_earnings": 44, "earnings_blackout": false, "earnings_date": "2026-08-07T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2271, "estimated_spread": 0.1514, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 15365359607.61, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 16.68, "normalized_momentum_score": 90.76, "normalized_quality_score": 70.85, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 151.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "LAMR", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lamar Advertising Company", "correlation_warning": false, "days_to_earnings": 44, "earnings_blackout": false, "earnings_date": "2026-08-07T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4543, "estimated_spread": 0.1211, "executable_entry": 151.42, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 151.42, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 15365359607.61, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 151.7077, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 151.9954, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2877, "net_target_1_assumption": -0.1741, "net_target_2_assumption": -0.1741, "normalized_atr_score": 100.0, "normalized_liquidity_score": 16.68, "normalized_momentum_score": 90.76, "normalized_quality_score": 70.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 151.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 151.42, "ticker": "LAMR", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>UNP</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>272.32</v>
       </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="inlineStr">
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>UNP
 No Trade
@@ -3929,26 +3749,132 @@
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_unp.png</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Union Pacific Corporation", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3812, "estimated_spread": 0.0817, "executable_entry": 272.32, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.32, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 161679986512.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.5515, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.7829, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2315, "net_target_1_assumption": -0.1362, "net_target_2_assumption": -0.1362, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.12, "normalized_momentum_score": 80.74, "normalized_quality_score": 79.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.32, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.32, "ticker": "UNP", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>154.27</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>ANET
+No Trade
+0.00
+score
+Price
+154.27
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+140.01
+Fib Zone
+137.88 - 142.14
+Swing Low
+115.42
+Swing High
+179.80
+Click chart to open full size</t>
+        </is>
+      </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_unp.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_anet.png</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 154.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Union Pacific Corporation", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1906, "estimated_spread": 0.1362, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 161679986512.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.12, "normalized_momentum_score": 80.74, "normalized_quality_score": 79.67, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.32, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UNP", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Arista Networks, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.216, "estimated_spread": 0.0463, "executable_entry": 154.27, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 154.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 194252074580.01, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 154.4011, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 154.5323, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1311, "net_target_1_assumption": -0.0771, "net_target_2_assumption": -0.0771, "normalized_atr_score": 99.78, "normalized_liquidity_score": 82.35, "normalized_momentum_score": 100, "normalized_quality_score": 94.65, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 154.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 154.27, "ticker": "ANET", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4037,7 +3963,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_mrk.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_mrk.png</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -4047,14 +3973,14 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Merck &amp; Co., Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0846, "estimated_spread": 0.0604, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 298330093349.04, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.49, "normalized_momentum_score": 76.16, "normalized_quality_score": 70.82, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 120.79, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "MRK", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Merck &amp; Co., Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1691, "estimated_spread": 0.0362, "executable_entry": 120.79, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 120.79, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 298330093349.04, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 120.8927, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 120.9953, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1027, "net_target_1_assumption": -0.0604, "net_target_2_assumption": -0.0604, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.49, "normalized_momentum_score": 76.16, "normalized_quality_score": 70.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 120.79, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 120.79, "ticker": "MRK", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4143,7 +4069,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_udr.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_udr.png</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -4153,14 +4079,14 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UDR, Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0588, "estimated_spread": 0.0392, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 12736693845.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 28.69, "normalized_momentum_score": 81.18, "normalized_quality_score": 70.14, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 39.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "UDR", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UDR, Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1176, "estimated_spread": 0.0314, "executable_entry": 39.2, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 39.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 12736693845.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 39.2745, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 39.349, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0745, "net_target_1_assumption": -0.0451, "net_target_2_assumption": -0.0451, "normalized_atr_score": 100.0, "normalized_liquidity_score": 28.69, "normalized_momentum_score": 81.18, "normalized_quality_score": 70.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 39.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 39.2, "ticker": "UDR", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4249,7 +4175,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_jpm.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_jpm.png</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -4259,14 +4185,14 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "JPMorgan Chase &amp; Co.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2187, "estimated_spread": 0.1562, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 836998968557.11, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.16, "normalized_momentum_score": 83.05, "normalized_quality_score": 80.42, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 312.37, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "JPM", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "JPMorgan Chase &amp; Co.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4373, "estimated_spread": 0.0937, "executable_entry": 312.37, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 312.37, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 836998968557.11, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 312.6355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 312.901, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2655, "net_target_1_assumption": -0.1562, "net_target_2_assumption": -0.1562, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.16, "normalized_momentum_score": 83.05, "normalized_quality_score": 80.42, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 312.37, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 312.37, "ticker": "JPM", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4355,7 +4281,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_ge.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_ge.png</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -4365,14 +4291,14 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "GE Aerospace", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2296, "estimated_spread": 0.164, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 342704109784.0, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 45.05, "normalized_momentum_score": 70.2, "normalized_quality_score": 70.11, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 328.0, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "GE", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "GE Aerospace", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4592, "estimated_spread": 0.0984, "executable_entry": 328.0, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 328.0, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 342704109784.0, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 328.2788, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 328.5576, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2788, "net_target_1_assumption": -0.164, "net_target_2_assumption": -0.164, "normalized_atr_score": 100.0, "normalized_liquidity_score": 45.05, "normalized_momentum_score": 70.2, "normalized_quality_score": 70.11, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 328.0, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 328.0, "ticker": "GE", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4461,7 +4387,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_irm.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_irm.png</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -4471,54 +4397,160 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Iron Mountain", "correlation_warning": false, "days_to_earnings": -26, "earnings_blackout": false, "earnings_date": "2026-04-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.187, "estimated_spread": 0.1247, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 37089427823.03, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 24.67, "normalized_momentum_score": 100, "normalized_quality_score": 77.4, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 124.66, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "IRM", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Iron Mountain", "correlation_warning": false, "days_to_earnings": -26, "earnings_blackout": false, "earnings_date": "2026-04-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.374, "estimated_spread": 0.0997, "executable_entry": 124.66, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 124.66, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 37089427823.03, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 124.8969, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 125.1337, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2369, "net_target_1_assumption": -0.1434, "net_target_2_assumption": -0.1434, "normalized_atr_score": 100.0, "normalized_liquidity_score": 24.67, "normalized_momentum_score": 100, "normalized_quality_score": 77.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 124.66, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 124.66, "ticker": "IRM", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>323.57</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>V
+No Trade
+0.00
+score
+Price
+323.57
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+323.02
+Fib Zone
+321.22 - 324.81
+Swing Low
+315.51
+Swing High
+335.17
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_v.png</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 323.57 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Visa Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.453, "estimated_spread": 0.0971, "executable_entry": 323.57, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 323.57, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 615347255294.79, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 323.845, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 324.1201, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.275, "net_target_1_assumption": -0.1618, "net_target_2_assumption": -0.1618, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.95, "normalized_momentum_score": 60.9, "normalized_quality_score": 70.39, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 323.57, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 323.57, "ticker": "V", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:27:03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>ABBV</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
         <v>227.23</v>
       </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="inlineStr">
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>ABBV
 No Trade
@@ -4565,125 +4597,19 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_abbv.png</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_abbv.png</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "AbbVie Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1591, "estimated_spread": 0.1136, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 401468325167.28, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.65, "normalized_momentum_score": 71.99, "normalized_quality_score": 69.29, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 227.23, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "ABBV", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-06-07T14:36:41</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>SLB</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
-        <v>54.87</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>SLB
-No Trade
-0.00
-score
-Price
-54.87
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-54.77
-Fib Zone
-54.33 - 55.21
-Swing Low
-52.45
-Swing High
-58.51
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260607_143045_slb.png</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>{"ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Schlumberger Limited", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0384, "estimated_spread": 0.0274, "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_rr": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 82033812262.18, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_rr": 0.0, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.73, "normalized_momentum_score": 100, "normalized_quality_score": 87.02, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 54.87, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "ticker": "SLB", "timestamp": "2026-06-07T14:36:41", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "AbbVie Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3181, "estimated_spread": 0.0682, "executable_entry": 227.23, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 227.23, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 401468325167.28, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 227.4231, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 227.6163, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1931, "net_target_1_assumption": -0.1136, "net_target_2_assumption": -0.1136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.65, "normalized_momentum_score": 71.99, "normalized_quality_score": 69.29, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 227.23, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 227.23, "ticker": "ABBV", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
@@ -5046,25 +4972,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T14:36:41</t>
+          <t>2026-06-07T19:27:03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260607_143045</t>
+          <t>20260607_192436</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CVX ELAN CAT C AMAT PANW KLAC ORCL UNH CRWD MU MS GS URI SMCI HST ASML TXN LLY MPC VLO BAC UPS AMH PSX LAMR UNP MRK UDR JPM GE IRM ABBV SLB</t>
+          <t>AMAT PANW KLAC ORCL CRWD MU MS SMCI CAT GS ASML HST LRCX TXN AMD C AAPL MPC VLO TSM BAC UPS AMH PSX LAMR UNP ANET MRK UDR JPM GE IRM V ABBV</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CVX:WATCH, ELAN:WATCH, CAT:WATCH, C:WATCH, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, UNH:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, GS:SKIP, URI:SKIP, SMCI:SKIP, HST:SKIP, ASML:SKIP, TXN:SKIP, LLY:SKIP, MPC:SKIP, VLO:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, ABBV:SKIP, SLB:SKIP</t>
+          <t>AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, SMCI:SKIP, CAT:SKIP, GS:SKIP, ASML:SKIP, HST:SKIP, LRCX:SKIP, TXN:SKIP, AMD:SKIP, C:SKIP, AAPL:SKIP, MPC:SKIP, VLO:SKIP, TSM:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, ANET:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, V:SKIP, ABBV:SKIP</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -5081,17 +5007,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>agent_results\summaries\market_lens_agent_20260607_143045.md</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\summaries\market_lens_agent_20260607_192436.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>agent_results\screenshots\market_lens_agent_20260607_143045.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\screenshots\market_lens_agent_20260607_192436.png</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>agent_results\decisions\market_lens_agent_20260607_143045.jsonl</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\decisions\market_lens_agent_20260607_192436.jsonl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep setup candidates visible in agent scans
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -897,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -1012,47 +1012,172 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T19:27:03</t>
+          <t>2026-06-08T00:27:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E2" t="n">
+        <v>323.57</v>
+      </c>
+      <c r="F2" t="n">
+        <v>321.22</v>
+      </c>
+      <c r="G2" t="n">
+        <v>324.81</v>
+      </c>
+      <c r="H2" t="n">
+        <v>319</v>
+      </c>
+      <c r="I2" t="n">
+        <v>325.34</v>
+      </c>
+      <c r="J2" t="n">
+        <v>338.49</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (323.02) with confluence at VWAP. Planned entry at zone low 321.22; executable entry 323.57, stop below fib 78.6% at 319.00.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>V
+Fib 61.8 Confluence Buy Zone
+0.45
+score
+Price
+323.57
+R/R
+1.39x
+Grade
+B
+Quality
+70%
+Buy Zone
+321.22 - 324.81
+Stop
+319.00
+Targets
+325.34 / 338.49
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+Trigger
+Break above prior-day high at 324.76 after holding buy zone.
+Invalidation
+Exit if price closes below 319.00 or setup support fails.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (323.02) with confluence at VWAP. Planned entry at zone low 321.22; executable entry 323.57, stop below fib 78.6% at 319.00.
+Fib 61.8
+323.02
+Fib Zone
+321.22 - 324.81
+Swing Low
+315.51
+Swing High
+335.17
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_v.png</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.45; R/R 1.39x; price 323.57 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.16; Factors: Financials | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 324.81, "buy_zone_low": 321.22, "cash_available": 100000.0, "company_name": "Visa Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.453, "estimated_spread": 0.0971, "executable_entry": 323.57, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_reward_1_per_share": 1.77, "gross_reward_2_per_share": 14.92, "gross_risk_per_share": 4.57, "gross_rr": 1.3944, "gross_rr_1": 0.3873, "gross_rr_2": 3.2648, "gross_rr_decision": 1.3944, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 615347255294.79, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 323.845, "net_reward_1_per_share": 1.3332, "net_reward_2_per_share": 14.4832, "net_risk_per_share": 5.1201, "net_rr": 1.1593, "net_rr_1": 0.2604, "net_rr_2": 2.8287, "net_stop_assumption": 318.725, "net_target_1_assumption": 325.1782, "net_target_2_assumption": 338.3282, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.95, "normalized_momentum_score": 60.9, "normalized_quality_score": 70.39, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 335.17, "price": 323.57, "prior_high_20": 335.17, "prior_high_63": 341.2725, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.45, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.45, "stop_loss": 319.0, "target_1": 325.34, "target_1_atr_distance": 0.2466, "target_2": 338.49, "target_2_atr_distance": 2.0787, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 321.22, "ticker": "V", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>AMAT</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>453.01</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>AMAT
 No Trade
@@ -1099,66 +1224,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_amat.png</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_amat.png</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Applied Materials, Inc.", "correlation_warning": false, "days_to_earnings": 48, "earnings_blackout": false, "earnings_date": "2026-08-13T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6342, "estimated_spread": 0.1359, "executable_entry": 453.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 453.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 359671569137.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 453.3951, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 453.7801, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3851, "net_target_1_assumption": -0.2265, "net_target_2_assumption": -0.2265, "normalized_atr_score": 98.01, "normalized_liquidity_score": 69.65, "normalized_momentum_score": 100, "normalized_quality_score": 90.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 453.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 453.01, "ticker": "AMAT", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Applied Materials, Inc.", "correlation_warning": false, "days_to_earnings": 48, "earnings_blackout": false, "earnings_date": "2026-08-13T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6342, "estimated_spread": 0.1359, "executable_entry": 453.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 453.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 359671569137.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 453.3951, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 453.7801, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3851, "net_target_1_assumption": -0.2265, "net_target_2_assumption": -0.2265, "normalized_atr_score": 98.01, "normalized_liquidity_score": 69.65, "normalized_momentum_score": 100, "normalized_quality_score": 90.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 453.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 453.01, "ticker": "AMAT", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>PANW</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>272.05</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>PANW
 No Trade
@@ -1205,66 +1330,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_panw.png</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_panw.png</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Palo Alto Networks, Inc.", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3809, "estimated_spread": 0.0816, "executable_entry": 272.05, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.05, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 221720740051.27, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.2812, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.5125, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2312, "net_target_1_assumption": -0.136, "net_target_2_assumption": -0.136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.83, "normalized_momentum_score": 100, "normalized_quality_score": 87.95, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.05, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.05, "ticker": "PANW", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Palo Alto Networks, Inc.", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3809, "estimated_spread": 0.0816, "executable_entry": 272.05, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.05, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 221720740051.27, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.2812, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.5125, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2312, "net_target_1_assumption": -0.136, "net_target_2_assumption": -0.136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.83, "normalized_momentum_score": 100, "normalized_quality_score": 87.95, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.05, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.05, "ticker": "PANW", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>KLAC</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>1929.2</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>KLAC
 No Trade
@@ -1311,66 +1436,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_klac.png</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_klac.png</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "KLA Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.7009, "estimated_spread": 0.5788, "executable_entry": 1929.2, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1929.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 252006607134.9, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1930.8398, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1932.4796, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.6398, "net_target_1_assumption": -0.9646, "net_target_2_assumption": -0.9646, "normalized_atr_score": 97.97, "normalized_liquidity_score": 51.67, "normalized_momentum_score": 100, "normalized_quality_score": 84.99, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1929.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1929.2, "ticker": "KLAC", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "KLA Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.7009, "estimated_spread": 0.5788, "executable_entry": 1929.2, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1929.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 252006607134.9, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1930.8398, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1932.4796, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.6398, "net_target_1_assumption": -0.9646, "net_target_2_assumption": -0.9646, "normalized_atr_score": 97.97, "normalized_liquidity_score": 51.67, "normalized_momentum_score": 100, "normalized_quality_score": 84.99, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1929.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1929.2, "ticker": "KLAC", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>213.68</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr">
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>ORCL
 No Trade
@@ -1417,66 +1542,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_orcl.png</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_orcl.png</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Oracle Corporation", "correlation_warning": false, "days_to_earnings": 2, "earnings_blackout": true, "earnings_date": "2026-06-10T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2992, "estimated_spread": 0.0641, "executable_entry": 213.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 213.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 614553488215.21, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 213.8616, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 214.0433, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1816, "net_target_1_assumption": -0.1068, "net_target_2_assumption": -0.1068, "normalized_atr_score": 88.94, "normalized_liquidity_score": 75.35, "normalized_momentum_score": 100, "normalized_quality_score": 89.84, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 213.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 213.68, "ticker": "ORCL", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable.", "Earnings blackout active."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Oracle Corporation", "correlation_warning": false, "days_to_earnings": 2, "earnings_blackout": true, "earnings_date": "2026-06-10T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2992, "estimated_spread": 0.0641, "executable_entry": 213.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 213.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 614553488215.21, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 213.8616, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 214.0433, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1816, "net_target_1_assumption": -0.1068, "net_target_2_assumption": -0.1068, "normalized_atr_score": 88.94, "normalized_liquidity_score": 75.35, "normalized_momentum_score": 100, "normalized_quality_score": 89.84, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 213.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 213.68, "ticker": "ORCL", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable.", "Earnings blackout active."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>CRWD</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>671.02</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>CRWD
 No Trade
@@ -1523,66 +1648,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_crwd.png</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_crwd.png</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 671.02 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "CrowdStrike Holdings, Inc.", "correlation_warning": false, "days_to_earnings": 61, "earnings_blackout": false, "earnings_date": "2026-09-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.9394, "estimated_spread": 0.2013, "executable_entry": 671.02, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 671.02, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 170818090488.37, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 671.5904, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 672.1607, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.5704, "net_target_1_assumption": -0.3355, "net_target_2_assumption": -0.3355, "normalized_atr_score": 100.0, "normalized_liquidity_score": 94.37, "normalized_momentum_score": 100, "normalized_quality_score": 98.31, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 671.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 671.02, "ticker": "CRWD", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "CrowdStrike Holdings, Inc.", "correlation_warning": false, "days_to_earnings": 61, "earnings_blackout": false, "earnings_date": "2026-09-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.9394, "estimated_spread": 0.2013, "executable_entry": 671.02, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 671.02, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 170818090488.37, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 671.5904, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 672.1607, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.5704, "net_target_1_assumption": -0.3355, "net_target_2_assumption": -0.3355, "normalized_atr_score": 100.0, "normalized_liquidity_score": 94.37, "normalized_momentum_score": 100, "normalized_quality_score": 98.31, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 671.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 671.02, "ticker": "CRWD", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>864.01</v>
       </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>MU
 No Trade
@@ -1629,66 +1754,172 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_mu.png</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_mu.png</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 864.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Micron Technology, Inc.", "correlation_warning": false, "days_to_earnings": 12, "earnings_blackout": false, "earnings_date": "2026-06-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3911, "estimated_spread": 0.2592, "executable_entry": 864.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 864.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 974373508417.54, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 864.8351, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 865.6603, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8251, "net_target_1_assumption": -0.4774, "net_target_2_assumption": -0.4774, "normalized_atr_score": 70.68, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 92.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 864.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 864.01, "ticker": "MU", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Micron Technology, Inc.", "correlation_warning": false, "days_to_earnings": 12, "earnings_blackout": false, "earnings_date": "2026-06-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3911, "estimated_spread": 0.2592, "executable_entry": 864.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 864.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 974373508417.54, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 864.8351, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 865.6603, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8251, "net_target_1_assumption": -0.4774, "net_target_2_assumption": -0.4774, "normalized_atr_score": 70.68, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 92.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 864.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 864.01, "ticker": "MU", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>399.47</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>UNH
+No Trade
+0.00
+score
+Price
+399.47
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+312.57
+Fib Zone
+310.10 - 315.05
+Swing Low
+255.97
+Swing High
+404.15
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_unh.png</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 399.47 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UnitedHealth Group Incorporated", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5593, "estimated_spread": 0.1198, "executable_entry": 399.47, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 399.47, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 362776446174.45, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 399.8095, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 400.1491, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3395, "net_target_1_assumption": -0.1997, "net_target_2_assumption": -0.1997, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.49, "normalized_momentum_score": 100, "normalized_quality_score": 88.45, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 399.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 399.47, "ticker": "UNH", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>211.93</v>
       </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>MS
 No Trade
@@ -1735,66 +1966,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_ms.png</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_ms.png</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 211.93 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Morgan Stanley", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2967, "estimated_spread": 0.0636, "executable_entry": 211.93, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 211.93, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 334273959714.43, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 212.1101, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 212.2903, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1801, "net_target_1_assumption": -0.106, "net_target_2_assumption": -0.106, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.49, "normalized_momentum_score": 100, "normalized_quality_score": 81.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 211.93, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 211.93, "ticker": "MS", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Morgan Stanley", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2967, "estimated_spread": 0.0636, "executable_entry": 211.93, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 211.93, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 334273959714.43, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 212.1101, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 212.2903, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1801, "net_target_1_assumption": -0.106, "net_target_2_assumption": -0.106, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.49, "normalized_momentum_score": 100, "normalized_quality_score": 81.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 211.93, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 211.93, "ticker": "MS", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>SMCI</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>41.64</v>
       </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>SMCI
 No Trade
@@ -1841,66 +2072,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_smci.png</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_smci.png</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Super Micro Computer, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.067, "estimated_spread": 0.0125, "executable_entry": 41.64, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 41.64, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 25043065223.4, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 41.6798, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 41.7195, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0398, "net_target_1_assumption": -0.023, "net_target_2_assumption": -0.023, "normalized_atr_score": 80.49, "normalized_liquidity_score": 81.49, "normalized_momentum_score": 100, "normalized_quality_score": 89.57, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 41.64, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 41.64, "ticker": "SMCI", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Super Micro Computer, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.067, "estimated_spread": 0.0125, "executable_entry": 41.64, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 41.64, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 25043065223.4, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 41.6798, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 41.7195, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0398, "net_target_1_assumption": -0.023, "net_target_2_assumption": -0.023, "normalized_atr_score": 80.49, "normalized_liquidity_score": 81.49, "normalized_momentum_score": 100, "normalized_quality_score": 89.57, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 41.64, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 41.64, "ticker": "SMCI", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>CAT</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
         <v>904.28</v>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>CAT
 No Trade
@@ -1947,66 +2178,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_cat.png</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_cat.png</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 904.28 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Caterpillar Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.266, "estimated_spread": 0.2713, "executable_entry": 904.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 904.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 416504131881.15, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 905.0486, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 905.8173, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.7686, "net_target_1_assumption": -0.4521, "net_target_2_assumption": -0.4521, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.89, "normalized_momentum_score": 100, "normalized_quality_score": 87.07, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 904.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 904.28, "ticker": "CAT", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Caterpillar Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.266, "estimated_spread": 0.2713, "executable_entry": 904.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 904.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 416504131881.15, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 905.0486, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 905.8173, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.7686, "net_target_1_assumption": -0.4521, "net_target_2_assumption": -0.4521, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.89, "normalized_momentum_score": 100, "normalized_quality_score": 87.07, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 904.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 904.28, "ticker": "CAT", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>GS</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
         <v>1038.68</v>
       </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="inlineStr">
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>GS
 No Trade
@@ -2053,66 +2284,172 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_gs.png</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_gs.png</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Goldman Sachs Group, Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.4542, "estimated_spread": 0.3116, "executable_entry": 1038.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1038.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 306418323889.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1039.5629, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1040.4458, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8829, "net_target_1_assumption": -0.5193, "net_target_2_assumption": -0.5193, "normalized_atr_score": 100.0, "normalized_liquidity_score": 55.06, "normalized_momentum_score": 100, "normalized_quality_score": 86.52, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1038.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1038.68, "ticker": "GS", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Goldman Sachs Group, Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.4542, "estimated_spread": 0.3116, "executable_entry": 1038.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1038.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 306418323889.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1039.5629, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1040.4458, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8829, "net_target_1_assumption": -0.5193, "net_target_2_assumption": -0.5193, "normalized_atr_score": 100.0, "normalized_liquidity_score": 55.06, "normalized_momentum_score": 100, "normalized_quality_score": 86.52, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1038.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1038.68, "ticker": "GS", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1067.77</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>URI
+No Trade
+0.00
+score
+Price
+1067.77
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+819.18
+Fib Zone
+811.20 - 827.15
+Swing Low
+707.99
+Swing High
+999.06
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_uri.png</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1067.77 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Rentals, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 3.2033, "estimated_spread": 0.8542, "executable_entry": 1067.77, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1067.77, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 66892115391.46, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1069.7988, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1071.8275, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -2.0288, "net_target_1_assumption": -1.2279, "net_target_2_assumption": -1.2279, "normalized_atr_score": 100.0, "normalized_liquidity_score": 47.57, "normalized_momentum_score": 100, "normalized_quality_score": 84.27, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1067.77, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1067.77, "ticker": "URI", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>ASML</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>1641.74</v>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr">
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>ASML
 No Trade
@@ -2159,172 +2496,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_asml.png</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_asml.png</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ASML Holding N.V.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.2984, "estimated_spread": 0.4925, "executable_entry": 1641.74, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1641.74, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 632755593573.26, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1643.1355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1644.531, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.3955, "net_target_1_assumption": -0.8209, "net_target_2_assumption": -0.8209, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.26, "normalized_momentum_score": 100, "normalized_quality_score": 88.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1641.74, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1641.74, "ticker": "ASML", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>HST</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ASML Holding N.V.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.2984, "estimated_spread": 0.4925, "executable_entry": 1641.74, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1641.74, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 632755593573.26, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1643.1355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1644.531, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.3955, "net_target_1_assumption": -0.8209, "net_target_2_assumption": -0.8209, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.26, "normalized_momentum_score": 100, "normalized_quality_score": 88.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1641.74, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1641.74, "ticker": "ASML", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>24.62</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="inlineStr">
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>303.28</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>HST
-No Trade
-0.00
-score
-Price
-24.62
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-21.35
-Fib Zone
-21.22 - 21.48
-Swing Low
-20.71
-Swing High
-22.39
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_hst.png</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Host Hotels &amp; Resorts", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0739, "estimated_spread": 0.0197, "executable_entry": 24.62, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 24.62, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 16861728472.99, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 24.6668, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 24.7136, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0468, "net_target_1_assumption": -0.0283, "net_target_2_assumption": -0.0283, "normalized_atr_score": 100.0, "normalized_liquidity_score": 26.55, "normalized_momentum_score": 100, "normalized_quality_score": 77.97, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 24.62, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 24.62, "ticker": "HST", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>LRCX</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>303.28</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>LRCX
 No Trade
@@ -2371,66 +2602,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_lrcx.png</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_lrcx.png</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 303.28 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lam Research Corporation", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4246, "estimated_spread": 0.091, "executable_entry": 303.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 303.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 379263466393.46, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 303.5378, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 303.7956, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2578, "net_target_1_assumption": -0.1516, "net_target_2_assumption": -0.1516, "normalized_atr_score": 95.25, "normalized_liquidity_score": 60.92, "normalized_momentum_score": 100, "normalized_quality_score": 87.09, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 303.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 303.28, "ticker": "LRCX", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lam Research Corporation", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4246, "estimated_spread": 0.091, "executable_entry": 303.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 303.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 379263466393.46, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 303.5378, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 303.7956, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2578, "net_target_1_assumption": -0.1516, "net_target_2_assumption": -0.1516, "normalized_atr_score": 95.25, "normalized_liquidity_score": 60.92, "normalized_momentum_score": 100, "normalized_quality_score": 87.09, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 303.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 303.28, "ticker": "LRCX", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>TXN</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>285.06</v>
       </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr">
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>TXN
 No Trade
@@ -2477,66 +2708,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_txn.png</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_txn.png</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Texas Instruments Incorporated", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3991, "estimated_spread": 0.0855, "executable_entry": 285.06, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 285.06, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 259431048780.55, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 285.3023, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 285.5446, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2423, "net_target_1_assumption": -0.1425, "net_target_2_assumption": -0.1425, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.24, "normalized_momentum_score": 100, "normalized_quality_score": 87.47, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 285.06, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 285.06, "ticker": "TXN", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Texas Instruments Incorporated", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3991, "estimated_spread": 0.0855, "executable_entry": 285.06, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 285.06, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 259431048780.55, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 285.3023, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 285.5446, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2423, "net_target_1_assumption": -0.1425, "net_target_2_assumption": -0.1425, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.24, "normalized_momentum_score": 100, "normalized_quality_score": 87.47, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 285.06, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 285.06, "ticker": "TXN", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>AMD</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>466.38</v>
       </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>AMD
 No Trade
@@ -2583,66 +2814,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_amd.png</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_amd.png</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 466.38 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Advanced Micro Devices, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.7509, "estimated_spread": 0.1399, "executable_entry": 466.38, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 466.38, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 760479533978.74, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 466.8254, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 467.2708, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4454, "net_target_1_assumption": -0.2577, "net_target_2_assumption": -0.2577, "normalized_atr_score": 84.31, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 96.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 466.38, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 466.38, "ticker": "AMD", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Advanced Micro Devices, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.7509, "estimated_spread": 0.1399, "executable_entry": 466.38, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 466.38, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 760479533978.74, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 466.8254, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 467.2708, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4454, "net_target_1_assumption": -0.2577, "net_target_2_assumption": -0.2577, "normalized_atr_score": 84.31, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 96.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 466.38, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 466.38, "ticker": "AMD", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>132.47</v>
       </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>C
 No Trade
@@ -2689,66 +2920,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_c.png</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_c.png</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 132.47 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Citigroup Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1855, "estimated_spread": 0.0397, "executable_entry": 132.47, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 132.47, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 225937781310.85, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 132.5826, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 132.6952, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1126, "net_target_1_assumption": -0.0662, "net_target_2_assumption": -0.0662, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.28, "normalized_momentum_score": 100, "normalized_quality_score": 82.68, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 132.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 132.47, "ticker": "C", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Citigroup Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1855, "estimated_spread": 0.0397, "executable_entry": 132.47, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 132.47, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 225937781310.85, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 132.5826, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 132.6952, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1126, "net_target_1_assumption": -0.0662, "net_target_2_assumption": -0.0662, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.28, "normalized_momentum_score": 100, "normalized_quality_score": 82.68, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 132.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 132.47, "ticker": "C", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
         <v>307.34</v>
       </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="inlineStr">
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>AAPL
 No Trade
@@ -2795,73 +3026,73 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_aapl.png</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_aapl.png</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 307.34 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Apple Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4303, "estimated_spread": 0.0922, "executable_entry": 307.34, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 307.34, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 4514011939253.3, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 307.6012, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 307.8625, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2612, "net_target_1_assumption": -0.1537, "net_target_2_assumption": -0.1537, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 100.0, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 307.34, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 307.34, "ticker": "AAPL", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>MPC</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Apple Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4303, "estimated_spread": 0.0922, "executable_entry": 307.34, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 307.34, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 4514011939253.3, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 307.6012, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 307.8625, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2612, "net_target_1_assumption": -0.1537, "net_target_2_assumption": -0.1537, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 100.0, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 307.34, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 307.34, "ticker": "AAPL", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>262.01</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1131.42</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>MPC
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>LLY
 No Trade
 0.00
 score
 Price
-262.01
+1131.42
 R/R
 0.00x
 Grade
@@ -2886,187 +3117,81 @@
 Institutional liquidity
 100%
 Volume
-Distribution risk
-30%
+Confirmed
+85%
 No actionable setup detected.
 No clean technical setup detected. Price in middle of value area or poor risk/reward.
 Fib 61.8
-245.05
+963.67
 Fib Zone
-242.88 - 247.22
+954.73 - 972.61
 Swing Low
-233.25
+849.05
 Swing High
-264.14
+1149.10
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_mpc.png</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Marathon Petroleum Corporation", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3668, "estimated_spread": 0.0786, "executable_entry": 262.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 262.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 76490320587.29, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 262.2327, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 262.4554, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2227, "net_target_1_assumption": -0.131, "net_target_2_assumption": -0.131, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.86, "normalized_momentum_score": 100, "normalized_quality_score": 85.86, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 262.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 262.01, "ticker": "MPC", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>VLO</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_lly.png</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1131.42 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Eli Lilly and Company", "correlation_warning": false, "days_to_earnings": 42, "earnings_blackout": false, "earnings_date": "2026-08-05T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.584, "estimated_spread": 0.3394, "executable_entry": 1131.42, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1131.42, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1008934100764.37, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1132.3817, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1133.3434, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.9617, "net_target_1_assumption": -0.5657, "net_target_2_assumption": -0.5657, "normalized_atr_score": 100.0, "normalized_liquidity_score": 66.54, "normalized_momentum_score": 100, "normalized_quality_score": 89.96, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1131.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1131.42, "ticker": "LLY", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>255.82</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>415.17</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>VLO
-No Trade
-0.00
-score
-Price
-255.82
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Neutral
-65%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-240.05
-Fib Zone
-237.85 - 242.25
-Swing Low
-226.18
-Swing High
-262.50
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_vlo.png</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Valero Energy Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3581, "estimated_spread": 0.0767, "executable_entry": 255.82, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 255.82, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 75961346466.04, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 256.0374, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 256.2549, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2174, "net_target_1_assumption": -0.1279, "net_target_2_assumption": -0.1279, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.08, "normalized_momentum_score": 100, "normalized_quality_score": 87.12, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 255.82, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 255.82, "ticker": "VLO", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>415.17</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>TSM
 No Trade
@@ -3113,66 +3238,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_tsm.png</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_tsm.png</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 415.17 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Taiwan Semiconductor Manufacturing Company Limited", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5812, "estimated_spread": 0.1246, "executable_entry": 415.17, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 415.17, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 2153268485619.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 415.5229, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 415.8758, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3529, "net_target_1_assumption": -0.2076, "net_target_2_assumption": -0.2076, "normalized_atr_score": 100.0, "normalized_liquidity_score": 80.47, "normalized_momentum_score": 100, "normalized_quality_score": 94.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 415.17, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 415.17, "ticker": "TSM", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Taiwan Semiconductor Manufacturing Company Limited", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5812, "estimated_spread": 0.1246, "executable_entry": 415.17, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 415.17, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 2153268485619.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 415.5229, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 415.8758, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3529, "net_target_1_assumption": -0.2076, "net_target_2_assumption": -0.2076, "normalized_atr_score": 100.0, "normalized_liquidity_score": 80.47, "normalized_momentum_score": 100, "normalized_quality_score": 94.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 415.17, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 415.17, "ticker": "TSM", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>BAC</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
         <v>53.83</v>
       </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="inlineStr">
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>BAC
 No Trade
@@ -3219,66 +3344,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_bac.png</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_bac.png</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Bank of America Corporation", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0754, "estimated_spread": 0.0161, "executable_entry": 53.83, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 53.83, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 382009487737.58, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 53.8758, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 53.9215, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0458, "net_target_1_assumption": -0.0269, "net_target_2_assumption": -0.0269, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.83, "normalized_momentum_score": 100, "normalized_quality_score": 85.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 53.83, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 53.83, "ticker": "BAC", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Bank of America Corporation", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0754, "estimated_spread": 0.0161, "executable_entry": 53.83, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 53.83, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 382009487737.58, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 53.8758, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 53.9215, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0458, "net_target_1_assumption": -0.0269, "net_target_2_assumption": -0.0269, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.83, "normalized_momentum_score": 100, "normalized_quality_score": 85.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 53.83, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 53.83, "ticker": "BAC", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>UPS</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
         <v>108.54</v>
       </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr">
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>UPS
 No Trade
@@ -3325,132 +3450,26 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_ups.png</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_ups.png</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Parcel Service, Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.152, "estimated_spread": 0.0326, "executable_entry": 108.54, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 108.54, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 92259682300.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 108.6323, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 108.7245, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0923, "net_target_1_assumption": -0.0543, "net_target_2_assumption": -0.0543, "normalized_atr_score": 100.0, "normalized_liquidity_score": 51.52, "normalized_momentum_score": 99.81, "normalized_quality_score": 85.37, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 108.54, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 108.54, "ticker": "UPS", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>AMH</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>33.27</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>AMH
-No Trade
-0.00
-score
-Price
-33.27
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-28.73
-Fib Zone
-28.57 - 28.89
-Swing Low
-27.22
-Swing High
-31.18
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_amh.png</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "American Homes 4 Rent Common Shares of Beneficial Interest", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0998, "estimated_spread": 0.0266, "executable_entry": 33.27, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 33.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 11997015510.91, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 33.3332, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 33.3964, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0632, "net_target_1_assumption": -0.0383, "net_target_2_assumption": -0.0383, "normalized_atr_score": 100.0, "normalized_liquidity_score": 17.57, "normalized_momentum_score": 99.67, "normalized_quality_score": 75.12, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 33.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 33.27, "ticker": "AMH", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Parcel Service, Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.152, "estimated_spread": 0.0326, "executable_entry": 108.54, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 108.54, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 92259682300.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 108.6323, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 108.7245, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0923, "net_target_1_assumption": -0.0543, "net_target_2_assumption": -0.0543, "normalized_atr_score": 100.0, "normalized_liquidity_score": 51.52, "normalized_momentum_score": 99.81, "normalized_quality_score": 85.37, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 108.54, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 108.54, "ticker": "UPS", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-07T19:27:03</t>
+          <t>2026-06-08T00:27:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3539,7 +3558,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_psx.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_psx.png</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3549,19 +3568,19 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Phillips 66", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5492, "estimated_spread": 0.1465, "executable_entry": 183.08, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 183.08, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 73403184195.73, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 183.4279, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 183.7757, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3479, "net_target_1_assumption": -0.2105, "net_target_2_assumption": -0.2105, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.74, "normalized_momentum_score": 100, "normalized_quality_score": 82.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 183.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 183.08, "ticker": "PSX", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Phillips 66", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5492, "estimated_spread": 0.1465, "executable_entry": 183.08, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 183.08, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 73403184195.73, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 183.4279, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 183.7757, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3479, "net_target_1_assumption": -0.2105, "net_target_2_assumption": -0.2105, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.74, "normalized_momentum_score": 100, "normalized_quality_score": 82.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 183.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 183.08, "ticker": "PSX", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-07T19:27:03</t>
+          <t>2026-06-08T00:27:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LAMR</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3573,7 +3592,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>151.42</v>
+        <v>272.32</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -3593,116 +3612,10 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
-        <is>
-          <t>LAMR
-No Trade
-0.00
-score
-Price
-151.42
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Clean uptrend
-86%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-148.26
-Fib Zone
-147.52 - 149.00
-Swing Low
-144.11
-Swing High
-154.97
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_lamr.png</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lamar Advertising Company", "correlation_warning": false, "days_to_earnings": 44, "earnings_blackout": false, "earnings_date": "2026-08-07T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4543, "estimated_spread": 0.1211, "executable_entry": 151.42, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 151.42, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 15365359607.61, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 151.7077, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 151.9954, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2877, "net_target_1_assumption": -0.1741, "net_target_2_assumption": -0.1741, "normalized_atr_score": 100.0, "normalized_liquidity_score": 16.68, "normalized_momentum_score": 90.76, "normalized_quality_score": 70.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 151.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 151.42, "ticker": "LAMR", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>UNP</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>272.32</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
         <is>
           <t>UNP
 No Trade
@@ -3749,66 +3662,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_unp.png</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_unp.png</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Union Pacific Corporation", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3812, "estimated_spread": 0.0817, "executable_entry": 272.32, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.32, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 161679986512.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.5515, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.7829, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2315, "net_target_1_assumption": -0.1362, "net_target_2_assumption": -0.1362, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.12, "normalized_momentum_score": 80.74, "normalized_quality_score": 79.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.32, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.32, "ticker": "UNP", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Union Pacific Corporation", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3812, "estimated_spread": 0.0817, "executable_entry": 272.32, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.32, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 161679986512.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.5515, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.7829, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2315, "net_target_1_assumption": -0.1362, "net_target_2_assumption": -0.1362, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.12, "normalized_momentum_score": 80.74, "normalized_quality_score": 79.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.32, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.32, "ticker": "UNP", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>ANET</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>154.27</v>
       </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="inlineStr">
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>ANET
 No Trade
@@ -3855,66 +3768,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_anet.png</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_anet.png</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 154.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Arista Networks, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.216, "estimated_spread": 0.0463, "executable_entry": 154.27, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 154.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 194252074580.01, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 154.4011, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 154.5323, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1311, "net_target_1_assumption": -0.0771, "net_target_2_assumption": -0.0771, "normalized_atr_score": 99.78, "normalized_liquidity_score": 82.35, "normalized_momentum_score": 100, "normalized_quality_score": 94.65, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 154.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 154.27, "ticker": "ANET", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Arista Networks, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.216, "estimated_spread": 0.0463, "executable_entry": 154.27, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 154.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 194252074580.01, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 154.4011, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 154.5323, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1311, "net_target_1_assumption": -0.0771, "net_target_2_assumption": -0.0771, "normalized_atr_score": 99.78, "normalized_liquidity_score": 82.35, "normalized_momentum_score": 100, "normalized_quality_score": 94.65, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 154.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 154.27, "ticker": "ANET", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>MRK</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
         <v>120.79</v>
       </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="inlineStr">
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>MRK
 No Trade
@@ -3961,66 +3874,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_mrk.png</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_mrk.png</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 120.79 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Merck &amp; Co., Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1691, "estimated_spread": 0.0362, "executable_entry": 120.79, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 120.79, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 298330093349.04, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 120.8927, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 120.9953, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1027, "net_target_1_assumption": -0.0604, "net_target_2_assumption": -0.0604, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.49, "normalized_momentum_score": 76.16, "normalized_quality_score": 70.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 120.79, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 120.79, "ticker": "MRK", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Merck &amp; Co., Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1691, "estimated_spread": 0.0362, "executable_entry": 120.79, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 120.79, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 298330093349.04, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 120.8927, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 120.9953, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1027, "net_target_1_assumption": -0.0604, "net_target_2_assumption": -0.0604, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.49, "normalized_momentum_score": 76.16, "normalized_quality_score": 70.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 120.79, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 120.79, "ticker": "MRK", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>UDR</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
         <v>39.2</v>
       </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="inlineStr">
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>UDR
 No Trade
@@ -4067,66 +3980,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_udr.png</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_udr.png</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 39.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UDR, Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1176, "estimated_spread": 0.0314, "executable_entry": 39.2, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 39.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 12736693845.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 39.2745, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 39.349, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0745, "net_target_1_assumption": -0.0451, "net_target_2_assumption": -0.0451, "normalized_atr_score": 100.0, "normalized_liquidity_score": 28.69, "normalized_momentum_score": 81.18, "normalized_quality_score": 70.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 39.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 39.2, "ticker": "UDR", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UDR, Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1176, "estimated_spread": 0.0314, "executable_entry": 39.2, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 39.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 12736693845.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 39.2745, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 39.349, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0745, "net_target_1_assumption": -0.0451, "net_target_2_assumption": -0.0451, "normalized_atr_score": 100.0, "normalized_liquidity_score": 28.69, "normalized_momentum_score": 81.18, "normalized_quality_score": 70.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 39.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 39.2, "ticker": "UDR", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>JPM</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
         <v>312.37</v>
       </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="inlineStr">
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>JPM
 No Trade
@@ -4173,66 +4086,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_jpm.png</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_jpm.png</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 312.37 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "JPMorgan Chase &amp; Co.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4373, "estimated_spread": 0.0937, "executable_entry": 312.37, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 312.37, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 836998968557.11, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 312.6355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 312.901, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2655, "net_target_1_assumption": -0.1562, "net_target_2_assumption": -0.1562, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.16, "normalized_momentum_score": 83.05, "normalized_quality_score": 80.42, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 312.37, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 312.37, "ticker": "JPM", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "JPMorgan Chase &amp; Co.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4373, "estimated_spread": 0.0937, "executable_entry": 312.37, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 312.37, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 836998968557.11, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 312.6355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 312.901, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2655, "net_target_1_assumption": -0.1562, "net_target_2_assumption": -0.1562, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.16, "normalized_momentum_score": 83.05, "normalized_quality_score": 80.42, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 312.37, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 312.37, "ticker": "JPM", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" t="n">
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
         <v>328</v>
       </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="inlineStr">
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>GE
 No Trade
@@ -4279,278 +4192,66 @@
 Click chart to open full size</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_ge.png</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_ge.png</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 328.00 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "GE Aerospace", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4592, "estimated_spread": 0.0984, "executable_entry": 328.0, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 328.0, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 342704109784.0, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 328.2788, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 328.5576, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2788, "net_target_1_assumption": -0.164, "net_target_2_assumption": -0.164, "normalized_atr_score": 100.0, "normalized_liquidity_score": 45.05, "normalized_momentum_score": 70.2, "normalized_quality_score": 70.11, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 328.0, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 328.0, "ticker": "GE", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>IRM</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "GE Aerospace", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4592, "estimated_spread": 0.0984, "executable_entry": 328.0, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 328.0, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 342704109784.0, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 328.2788, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 328.5576, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2788, "net_target_1_assumption": -0.164, "net_target_2_assumption": -0.164, "normalized_atr_score": 100.0, "normalized_liquidity_score": 45.05, "normalized_momentum_score": 70.2, "normalized_quality_score": 70.11, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 328.0, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 328.0, "ticker": "GE", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>No Trade</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
-        <v>124.66</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="inlineStr">
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>227.23</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>IRM
-No Trade
-0.00
-score
-Price
-124.66
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Confirmed
-85%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-119.20
-Fib Zone
-118.31 - 120.10
-Swing Low
-110.00
-Swing High
-134.09
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_irm.png</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 124.66 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Iron Mountain", "correlation_warning": false, "days_to_earnings": -26, "earnings_blackout": false, "earnings_date": "2026-04-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.374, "estimated_spread": 0.0997, "executable_entry": 124.66, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 124.66, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 37089427823.03, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 124.8969, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 125.1337, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2369, "net_target_1_assumption": -0.1434, "net_target_2_assumption": -0.1434, "normalized_atr_score": 100.0, "normalized_liquidity_score": 24.67, "normalized_momentum_score": 100, "normalized_quality_score": 77.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 124.66, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 124.66, "ticker": "IRM", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
-        <v>323.57</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>V
-No Trade
-0.00
-score
-Price
-323.57
-R/R
-0.00x
-Grade
-No Trade
-Quality
-0%
-Buy Zone
--
-Stop
-0.00
-Targets
--
-Skip
-Mixed
-Relative Strength
-Leadership
-100%
-Trend Quality
-Constructive
-68%
-Liquidity
-Institutional liquidity
-100%
-Volume
-Distribution risk
-30%
-No actionable setup detected.
-No clean technical setup detected. Price in middle of value area or poor risk/reward.
-Fib 61.8
-323.02
-Fib Zone
-321.22 - 324.81
-Swing Low
-315.51
-Swing High
-335.17
-Click chart to open full size</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_v.png</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 323.57 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Visa Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.453, "estimated_spread": 0.0971, "executable_entry": 323.57, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 323.57, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 615347255294.79, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 323.845, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 324.1201, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.275, "net_target_1_assumption": -0.1618, "net_target_2_assumption": -0.1618, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.95, "normalized_momentum_score": 60.9, "normalized_quality_score": 70.39, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 323.57, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 323.57, "ticker": "V", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-06-07T19:27:03</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>ABBV</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>No Trade</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
-        <v>227.23</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>ABBV
 No Trade
@@ -4597,19 +4298,443 @@
 Click chart to open full size</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_abbv.png</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "AbbVie Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3181, "estimated_spread": 0.0682, "executable_entry": 227.23, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 227.23, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 401468325167.28, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 227.4231, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 227.6163, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1931, "net_target_1_assumption": -0.1136, "net_target_2_assumption": -0.1136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.65, "normalized_momentum_score": 71.99, "normalized_quality_score": 69.29, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 227.23, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 227.23, "ticker": "ABBV", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>54.87</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>SLB
+No Trade
+0.00
+score
+Price
+54.87
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+54.77
+Fib Zone
+54.33 - 55.21
+Swing Low
+52.45
+Swing High
+58.51
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_slb.png</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Schlumberger Limited", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0768, "estimated_spread": 0.0165, "executable_entry": 54.87, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 54.87, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 82033812262.18, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 54.9166, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 54.9633, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0466, "net_target_1_assumption": -0.0274, "net_target_2_assumption": -0.0274, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.73, "normalized_momentum_score": 100, "normalized_quality_score": 87.02, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 54.87, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 54.87, "ticker": "SLB", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>205.1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>NVDA
+No Trade
+0.00
+score
+Price
+205.10
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+210.46
+Fib Zone
+208.33 - 212.59
+Swing Low
+194.51
+Swing High
+236.26
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_nvda.png</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 205.10 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "NVIDIA Corporation", "correlation_warning": false, "days_to_earnings": 57, "earnings_blackout": false, "earnings_date": "2026-08-26T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2871, "estimated_spread": 0.0615, "executable_entry": 205.1, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 205.1, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 4967727247833.25, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 205.2743, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 205.4487, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1743, "net_target_1_assumption": -0.1026, "net_target_2_assumption": -0.1026, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 90.08, "normalized_quality_score": 95.54, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 205.1, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 205.1, "ticker": "NVDA", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>385.73</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>AVGO
+No Trade
+0.00
+score
+Price
+385.73
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+28%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+343.19
+Fib Zone
+337.54 - 348.85
+Swing Low
+289.96
+Swing High
+429.31
+Click chart to open full size</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260607_192436_abbv.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_avgo.png</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 385.73 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "AbbVie Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3181, "estimated_spread": 0.0682, "executable_entry": 227.23, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 227.23, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 401468325167.28, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 227.4231, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 227.6163, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1931, "net_target_1_assumption": -0.1136, "net_target_2_assumption": -0.1136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.65, "normalized_momentum_score": 71.99, "normalized_quality_score": 69.29, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 227.23, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 227.23, "ticker": "ABBV", "timestamp": "2026-06-07T19:27:03", "warnings": ["Target ATR feasibility unavailable."]}</t>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Broadcom Inc.", "correlation_warning": false, "days_to_earnings": 63, "earnings_blackout": false, "earnings_date": "2026-09-03T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.54, "estimated_spread": 0.1157, "executable_entry": 385.73, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 385.73, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1826303610630.94, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 386.0579, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 386.3857, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3279, "net_target_1_assumption": -0.1929, "net_target_2_assumption": -0.1929, "normalized_atr_score": 88.92, "normalized_liquidity_score": 100, "normalized_momentum_score": 82.06, "normalized_quality_score": 89.16, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 385.73, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 385.73, "ticker": "AVGO", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:27:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>112.45</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>NOW
+No Trade
+0.00
+score
+Price
+112.45
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+95.14
+Fib Zone
+93.19 - 97.09
+Swing Low
+85.44
+Swing High
+110.83
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_002548_now.png</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 112.45 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ServiceNow, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.181, "estimated_spread": 0.0337, "executable_entry": 112.45, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 112.45, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 115970581452.7, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 112.5574, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 112.6648, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1074, "net_target_1_assumption": -0.0621, "net_target_2_assumption": -0.0621, "normalized_atr_score": 86.89, "normalized_liquidity_score": 100, "normalized_momentum_score": 57.36, "normalized_quality_score": 77.53, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 112.45, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 112.45, "ticker": "NOW", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
@@ -4972,25 +5097,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-07T19:27:03</t>
+          <t>2026-06-08T00:27:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260607_192436</t>
+          <t>20260608_002548</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMAT PANW KLAC ORCL CRWD MU MS SMCI CAT GS ASML HST LRCX TXN AMD C AAPL MPC VLO TSM BAC UPS AMH PSX LAMR UNP ANET MRK UDR JPM GE IRM V ABBV</t>
+          <t>V AMAT PANW KLAC ORCL CRWD MU UNH MS SMCI CAT GS URI ASML LRCX TXN AMD C AAPL LLY TSM BAC UPS PSX UNP ANET MRK UDR JPM GE ABBV SLB NVDA AVGO NOW</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, CRWD:SKIP, MU:SKIP, MS:SKIP, SMCI:SKIP, CAT:SKIP, GS:SKIP, ASML:SKIP, HST:SKIP, LRCX:SKIP, TXN:SKIP, AMD:SKIP, C:SKIP, AAPL:SKIP, MPC:SKIP, VLO:SKIP, TSM:SKIP, BAC:SKIP, UPS:SKIP, AMH:SKIP, PSX:SKIP, LAMR:SKIP, UNP:SKIP, ANET:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, IRM:SKIP, V:SKIP, ABBV:SKIP</t>
+          <t>V:WATCH, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, CRWD:SKIP, MU:SKIP, UNH:SKIP, MS:SKIP, SMCI:SKIP, CAT:SKIP, GS:SKIP, URI:SKIP, ASML:SKIP, LRCX:SKIP, TXN:SKIP, AMD:SKIP, C:SKIP, AAPL:SKIP, LLY:SKIP, TSM:SKIP, BAC:SKIP, UPS:SKIP, PSX:SKIP, UNP:SKIP, ANET:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, ABBV:SKIP, SLB:SKIP, NVDA:SKIP, AVGO:SKIP, NOW:SKIP</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -5007,17 +5132,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\summaries\market_lens_agent_20260607_192436.md</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\summaries\market_lens_agent_20260608_002548.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\screenshots\market_lens_agent_20260607_192436.png</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\screenshots\market_lens_agent_20260608_002548.png</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\decisions\market_lens_agent_20260607_192436.jsonl</t>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\decisions\market_lens_agent_20260608_002548.jsonl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carry forward recent watch tickers in agent scans
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -897,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -4735,6 +4735,3735 @@
       <c r="R36" t="inlineStr">
         <is>
           <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ServiceNow, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.181, "estimated_spread": 0.0337, "executable_entry": 112.45, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 112.45, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 115970581452.7, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 112.5574, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 112.6648, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1074, "net_target_1_assumption": -0.0621, "net_target_2_assumption": -0.0621, "normalized_atr_score": 86.89, "normalized_liquidity_score": 100, "normalized_momentum_score": 57.36, "normalized_quality_score": 77.53, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 112.45, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 112.45, "ticker": "NOW", "timestamp": "2026-06-08T00:27:00", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E37" t="n">
+        <v>323.57</v>
+      </c>
+      <c r="F37" t="n">
+        <v>321.22</v>
+      </c>
+      <c r="G37" t="n">
+        <v>324.81</v>
+      </c>
+      <c r="H37" t="n">
+        <v>319</v>
+      </c>
+      <c r="I37" t="n">
+        <v>325.34</v>
+      </c>
+      <c r="J37" t="n">
+        <v>338.49</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (323.02) with confluence at VWAP. Planned entry at zone low 321.22; executable entry 323.57, stop below fib 78.6% at 319.00.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>V
+Fib 61.8 Confluence Buy Zone
+0.45
+score
+Price
+323.57
+R/R
+1.39x
+Grade
+B
+Quality
+70%
+Buy Zone
+321.22 - 324.81
+Stop
+319.00
+Targets
+325.34 / 338.49
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+Trigger
+Break above prior-day high at 324.76 after holding buy zone.
+Invalidation
+Exit if price closes below 319.00 or setup support fails.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (323.02) with confluence at VWAP. Planned entry at zone low 321.22; executable entry 323.57, stop below fib 78.6% at 319.00.
+Fib 61.8
+323.02
+Fib Zone
+321.22 - 324.81
+Swing Low
+315.51
+Swing High
+335.17
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_v.png</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.45; R/R 1.39x; price 323.57 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.16; Factors: Financials | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 324.81, "buy_zone_low": 321.22, "cash_available": 100000.0, "company_name": "Visa Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.453, "estimated_spread": 0.0971, "executable_entry": 323.57, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_reward_1_per_share": 1.77, "gross_reward_2_per_share": 14.92, "gross_risk_per_share": 4.57, "gross_rr": 1.3944, "gross_rr_1": 0.3873, "gross_rr_2": 3.2648, "gross_rr_decision": 1.3944, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 615347255294.79, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 323.845, "net_reward_1_per_share": 1.3332, "net_reward_2_per_share": 14.4832, "net_risk_per_share": 5.1201, "net_rr": 1.1593, "net_rr_1": 0.2604, "net_rr_2": 2.8287, "net_stop_assumption": 318.725, "net_target_1_assumption": 325.1782, "net_target_2_assumption": 338.3282, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.95, "normalized_momentum_score": 60.9, "normalized_quality_score": 70.39, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 335.17, "price": 323.57, "prior_high_20": 335.17, "prior_high_63": 341.2725, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.45, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.45, "stop_loss": 319.0, "target_1": 325.34, "target_1_atr_distance": 0.2466, "target_2": 338.49, "target_2_atr_distance": 2.0787, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 321.22, "ticker": "V", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>453.01</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>AMAT
+No Trade
+0.00
+score
+Price
+453.01
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+403.84
+Fib Zone
+398.18 - 409.49
+Swing Low
+376.60
+Swing High
+447.89
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_amat.png</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 453.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Applied Materials, Inc.", "correlation_warning": false, "days_to_earnings": 48, "earnings_blackout": false, "earnings_date": "2026-08-13T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6342, "estimated_spread": 0.1359, "executable_entry": 453.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 453.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 359671569137.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 453.3951, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 453.7801, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3851, "net_target_1_assumption": -0.2265, "net_target_2_assumption": -0.2265, "normalized_atr_score": 98.01, "normalized_liquidity_score": 69.65, "normalized_momentum_score": 100, "normalized_quality_score": 90.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 453.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 453.01, "ticker": "AMAT", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>PANW
+No Trade
+0.00
+score
+Price
+272.05
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+157.16
+Fib Zone
+153.95 - 160.38
+Swing Low
+143.50
+Swing High
+179.27
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_panw.png</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.05 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Palo Alto Networks, Inc.", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3809, "estimated_spread": 0.0816, "executable_entry": 272.05, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.05, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 221720740051.27, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.2812, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.5125, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2312, "net_target_1_assumption": -0.136, "net_target_2_assumption": -0.136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.83, "normalized_momentum_score": 100, "normalized_quality_score": 87.95, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.05, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.05, "ticker": "PANW", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1929.2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>KLAC
+No Trade
+0.00
+score
+Price
+1929.20
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+1745.04
+Fib Zone
+1720.95 - 1769.14
+Swing Low
+1643.90
+Swing High
+1908.67
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_klac.png</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1929.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "KLA Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.7009, "estimated_spread": 0.5788, "executable_entry": 1929.2, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1929.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 252006607134.9, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1930.8398, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1932.4796, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.6398, "net_target_1_assumption": -0.9646, "net_target_2_assumption": -0.9646, "normalized_atr_score": 97.97, "normalized_liquidity_score": 51.67, "normalized_momentum_score": 100, "normalized_quality_score": 84.99, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1929.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1929.2, "ticker": "KLAC", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>213.68</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>ORCL
+No Trade
+0.00
+score
+Price
+213.68
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+175.76
+Fib Zone
+172.62 - 178.89
+Swing Low
+160.33
+Swing High
+200.71
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_orcl.png</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 213.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Oracle Corporation", "correlation_warning": false, "days_to_earnings": 2, "earnings_blackout": true, "earnings_date": "2026-06-10T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2992, "estimated_spread": 0.0641, "executable_entry": 213.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 213.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 614553488215.21, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 213.8616, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 214.0433, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1816, "net_target_1_assumption": -0.1068, "net_target_2_assumption": -0.1068, "normalized_atr_score": 88.94, "normalized_liquidity_score": 75.35, "normalized_momentum_score": 100, "normalized_quality_score": 89.84, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 213.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 213.68, "ticker": "ORCL", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable.", "Earnings blackout active."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>671.02</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>CRWD
+No Trade
+0.00
+score
+Price
+671.02
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+404.00
+Fib Zone
+395.22 - 412.77
+Swing Low
+364.47
+Swing High
+467.95
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_crwd.png</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 671.02 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "CrowdStrike Holdings, Inc.", "correlation_warning": false, "days_to_earnings": 61, "earnings_blackout": false, "earnings_date": "2026-09-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.9394, "estimated_spread": 0.2013, "executable_entry": 671.02, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 671.02, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 170818090488.37, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 671.5904, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 672.1607, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.5704, "net_target_1_assumption": -0.3355, "net_target_2_assumption": -0.3355, "normalized_atr_score": 100.0, "normalized_liquidity_score": 94.37, "normalized_momentum_score": 100, "normalized_quality_score": 98.31, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 671.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 671.02, "ticker": "CRWD", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>864.01</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>MU
+No Trade
+0.00
+score
+Price
+864.01
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+100%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+505.23
+Fib Zone
+488.78 - 521.68
+Swing Low
+311.49
+Swing High
+818.67
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_mu.png</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 864.01 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Micron Technology, Inc.", "correlation_warning": false, "days_to_earnings": 12, "earnings_blackout": false, "earnings_date": "2026-06-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3911, "estimated_spread": 0.2592, "executable_entry": 864.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 864.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 974373508417.54, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 864.8351, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 865.6603, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8251, "net_target_1_assumption": -0.4774, "net_target_2_assumption": -0.4774, "normalized_atr_score": 70.68, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 92.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 864.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 864.01, "ticker": "MU", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>399.47</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>UNH
+No Trade
+0.00
+score
+Price
+399.47
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+312.57
+Fib Zone
+310.10 - 315.05
+Swing Low
+255.97
+Swing High
+404.15
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_unh.png</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 399.47 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UnitedHealth Group Incorporated", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5593, "estimated_spread": 0.1198, "executable_entry": 399.47, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 399.47, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 362776446174.45, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 399.8095, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 400.1491, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3395, "net_target_1_assumption": -0.1997, "net_target_2_assumption": -0.1997, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.49, "normalized_momentum_score": 100, "normalized_quality_score": 88.45, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 399.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 399.47, "ticker": "UNH", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>211.93</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>MS
+No Trade
+0.00
+score
+Price
+211.93
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+167.86
+Fib Zone
+166.53 - 169.19
+Swing Low
+151.98
+Swing High
+193.55
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_ms.png</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 211.93 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Morgan Stanley", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2967, "estimated_spread": 0.0636, "executable_entry": 211.93, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 211.93, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 334273959714.43, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 212.1101, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 212.2903, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1801, "net_target_1_assumption": -0.106, "net_target_2_assumption": -0.106, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.49, "normalized_momentum_score": 100, "normalized_quality_score": 81.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 211.93, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 211.93, "ticker": "MS", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>41.64</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>SMCI
+No Trade
+0.00
+score
+Price
+41.64
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+29.63
+Fib Zone
+28.83 - 30.42
+Swing Low
+25.46
+Swing High
+36.37
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_smci.png</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 41.64 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Super Micro Computer, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.067, "estimated_spread": 0.0125, "executable_entry": 41.64, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 41.64, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 25043065223.4, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 41.6798, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 41.7195, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0398, "net_target_1_assumption": -0.023, "net_target_2_assumption": -0.023, "normalized_atr_score": 80.49, "normalized_liquidity_score": 81.49, "normalized_momentum_score": 100, "normalized_quality_score": 89.57, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 41.64, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 41.64, "ticker": "SMCI", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>904.28</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>CAT
+No Trade
+0.00
+score
+Price
+904.28
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+764.64
+Fib Zone
+757.07 - 772.21
+Swing Low
+661.59
+Swing High
+931.35
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_cat.png</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 904.28 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Caterpillar Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.266, "estimated_spread": 0.2713, "executable_entry": 904.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 904.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 416504131881.15, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 905.0486, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 905.8173, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.7686, "net_target_1_assumption": -0.4521, "net_target_2_assumption": -0.4521, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.89, "normalized_momentum_score": 100, "normalized_quality_score": 87.07, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 904.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 904.28, "ticker": "CAT", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1038.68</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>GS
+No Trade
+0.00
+score
+Price
+1038.68
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+842.30
+Fib Zone
+834.41 - 850.20
+Swing Low
+777.08
+Swing High
+947.83
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_gs.png</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1038.68 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Goldman Sachs Group, Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.4542, "estimated_spread": 0.3116, "executable_entry": 1038.68, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1038.68, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 306418323889.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1039.5629, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1040.4458, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8829, "net_target_1_assumption": -0.5193, "net_target_2_assumption": -0.5193, "normalized_atr_score": 100.0, "normalized_liquidity_score": 55.06, "normalized_momentum_score": 100, "normalized_quality_score": 86.52, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1038.68, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1038.68, "ticker": "GS", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1067.77</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>URI
+No Trade
+0.00
+score
+Price
+1067.77
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+819.18
+Fib Zone
+811.20 - 827.15
+Swing Low
+707.99
+Swing High
+999.06
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_uri.png</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1067.77 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Rentals, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 3.2033, "estimated_spread": 0.8542, "executable_entry": 1067.77, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1067.77, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 66892115391.46, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1069.7988, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1071.8275, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -2.0288, "net_target_1_assumption": -1.2279, "net_target_2_assumption": -1.2279, "normalized_atr_score": 100.0, "normalized_liquidity_score": 47.57, "normalized_momentum_score": 100, "normalized_quality_score": 84.27, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1067.77, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1067.77, "ticker": "URI", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1641.74</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>ASML
+No Trade
+0.00
+score
+Price
+1641.74
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+1455.99
+Fib Zone
+1438.81 - 1473.16
+Swing Low
+1364.81
+Swing High
+1603.49
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_asml.png</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1641.74 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ASML Holding N.V.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 2.2984, "estimated_spread": 0.4925, "executable_entry": 1641.74, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1641.74, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 632755593573.26, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1643.1355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1644.531, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -1.3955, "net_target_1_assumption": -0.8209, "net_target_2_assumption": -0.8209, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.26, "normalized_momentum_score": 100, "normalized_quality_score": 88.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1641.74, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1641.74, "ticker": "ASML", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>303.28</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>LRCX
+No Trade
+0.00
+score
+Price
+303.28
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+227.21
+Fib Zone
+223.23 - 231.20
+Swing Low
+198.60
+Swing High
+273.50
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_lrcx.png</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 303.28 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lam Research Corporation", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4246, "estimated_spread": 0.091, "executable_entry": 303.28, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 303.28, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 379263466393.46, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 303.5378, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 303.7956, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2578, "net_target_1_assumption": -0.1516, "net_target_2_assumption": -0.1516, "normalized_atr_score": 95.25, "normalized_liquidity_score": 60.92, "normalized_momentum_score": 100, "normalized_quality_score": 87.09, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 303.28, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 303.28, "ticker": "LRCX", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>285.06</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>TXN
+No Trade
+0.00
+score
+Price
+285.06
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+87%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+223.12
+Fib Zone
+220.05 - 226.19
+Swing Low
+184.01
+Swing High
+286.37
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_txn.png</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 285.06 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Texas Instruments Incorporated", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3991, "estimated_spread": 0.0855, "executable_entry": 285.06, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 285.06, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 259431048780.55, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 285.3023, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 285.5446, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2423, "net_target_1_assumption": -0.1425, "net_target_2_assumption": -0.1425, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.24, "normalized_momentum_score": 100, "normalized_quality_score": 87.47, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 285.06, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 285.06, "ticker": "TXN", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>466.38</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>AMD
+No Trade
+0.00
+score
+Price
+466.38
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+100%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+298.44
+Fib Zone
+291.08 - 305.79
+Swing Low
+192.87
+Swing High
+469.22
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_amd.png</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 466.38 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Advanced Micro Devices, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.7509, "estimated_spread": 0.1399, "executable_entry": 466.38, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 466.38, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 760479533978.74, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 466.8254, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 467.2708, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4454, "net_target_1_assumption": -0.2577, "net_target_2_assumption": -0.2577, "normalized_atr_score": 84.31, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 96.08, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 466.38, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 466.38, "ticker": "AMD", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>132.47</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>C
+No Trade
+0.00
+score
+Price
+132.47
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+114.18
+Fib Zone
+113.29 - 115.07
+Swing Low
+101.53
+Swing High
+134.65
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_c.png</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 132.47 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Citigroup Inc.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1855, "estimated_spread": 0.0397, "executable_entry": 132.47, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 132.47, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 225937781310.85, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 132.5826, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 132.6952, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1126, "net_target_1_assumption": -0.0662, "net_target_2_assumption": -0.0662, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.28, "normalized_momentum_score": 100, "normalized_quality_score": 82.68, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 132.47, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 132.47, "ticker": "C", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>307.34</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>AAPL
+No Trade
+0.00
+score
+Price
+307.34
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+257.26
+Fib Zone
+255.75 - 258.78
+Swing Low
+242.97
+Swing High
+280.39
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_aapl.png</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 307.34 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Apple Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4303, "estimated_spread": 0.0922, "executable_entry": 307.34, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 307.34, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 4514011939253.3, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 307.6012, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 307.8625, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2612, "net_target_1_assumption": -0.1537, "net_target_2_assumption": -0.1537, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 100, "normalized_quality_score": 100.0, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 307.34, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 307.34, "ticker": "AAPL", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1131.42</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>LLY
+No Trade
+0.00
+score
+Price
+1131.42
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+963.67
+Fib Zone
+954.73 - 972.61
+Swing Low
+849.05
+Swing High
+1149.10
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_lly.png</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 1131.42 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Eli Lilly and Company", "correlation_warning": false, "days_to_earnings": 42, "earnings_blackout": false, "earnings_date": "2026-08-05T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.584, "estimated_spread": 0.3394, "executable_entry": 1131.42, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 1131.42, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1008934100764.37, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 1132.3817, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 1133.3434, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.9617, "net_target_1_assumption": -0.5657, "net_target_2_assumption": -0.5657, "normalized_atr_score": 100.0, "normalized_liquidity_score": 66.54, "normalized_momentum_score": 100, "normalized_quality_score": 89.96, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 1131.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 1131.42, "ticker": "LLY", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>415.17</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>TSM
+No Trade
+0.00
+score
+Price
+415.17
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+381.16
+Fib Zone
+376.97 - 385.35
+Swing Low
+360.55
+Swing High
+414.50
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_tsm.png</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Semiconductors - Strong (79/100); SMH sector regime is strong: 44.5% 3m return, 35.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 415.17 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Semiconductors | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Taiwan Semiconductor Manufacturing Company Limited", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5812, "estimated_spread": 0.1246, "executable_entry": 415.17, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Semiconductors"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 415.17, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 2153268485619.81, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 415.5229, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 415.8758, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3529, "net_target_1_assumption": -0.2076, "net_target_2_assumption": -0.2076, "normalized_atr_score": 100.0, "normalized_liquidity_score": 80.47, "normalized_momentum_score": 100, "normalized_quality_score": 94.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 415.17, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Semiconductors", "sector_etf": "SMH", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 78.71, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 415.17, "ticker": "TSM", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>BAC
+No Trade
+0.00
+score
+Price
+53.83
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+49.41
+Fib Zone
+49.12 - 49.70
+Swing Low
+45.88
+Swing High
+55.11
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_bac.png</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 53.83 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Bank of America Corporation", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0754, "estimated_spread": 0.0161, "executable_entry": 53.83, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 53.83, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 382009487737.58, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 53.8758, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 53.9215, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0458, "net_target_1_assumption": -0.0269, "net_target_2_assumption": -0.0269, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.83, "normalized_momentum_score": 100, "normalized_quality_score": 85.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 53.83, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 53.83, "ticker": "BAC", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>108.54</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>UPS
+No Trade
+0.00
+score
+Price
+108.54
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+98.43
+Fib Zone
+97.76 - 99.10
+Swing Low
+92.50
+Swing High
+108.02
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_ups.png</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 108.54 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "United Parcel Service, Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.152, "estimated_spread": 0.0326, "executable_entry": 108.54, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 108.54, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 92259682300.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 108.6323, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 108.7245, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0923, "net_target_1_assumption": -0.0543, "net_target_2_assumption": -0.0543, "normalized_atr_score": 100.0, "normalized_liquidity_score": 51.52, "normalized_momentum_score": 99.81, "normalized_quality_score": 85.37, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 108.54, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 108.54, "ticker": "UPS", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>183.08</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>PSX
+No Trade
+0.00
+score
+Price
+183.08
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+172.07
+Fib Zone
+170.69 - 173.44
+Swing Low
+164.25
+Swing High
+184.72
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_psx.png</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 183.08 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Phillips 66", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5492, "estimated_spread": 0.1465, "executable_entry": 183.08, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 183.08, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 73403184195.73, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 183.4279, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 183.7757, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3479, "net_target_1_assumption": -0.2105, "net_target_2_assumption": -0.2105, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.74, "normalized_momentum_score": 100, "normalized_quality_score": 82.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 183.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 183.08, "ticker": "PSX", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>272.32</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>UNP
+No Trade
+0.00
+score
+Price
+272.32
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+265.53
+Fib Zone
+263.88 - 267.17
+Swing Low
+259.69
+Swing High
+274.97
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_unp.png</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 272.32 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Union Pacific Corporation", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3812, "estimated_spread": 0.0817, "executable_entry": 272.32, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 272.32, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 161679986512.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 272.5515, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 272.7829, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2315, "net_target_1_assumption": -0.1362, "net_target_2_assumption": -0.1362, "normalized_atr_score": 100.0, "normalized_liquidity_score": 61.12, "normalized_momentum_score": 80.74, "normalized_quality_score": 79.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 272.32, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 272.32, "ticker": "UNP", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>154.27</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>ANET
+No Trade
+0.00
+score
+Price
+154.27
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+140.01
+Fib Zone
+137.88 - 142.14
+Swing Low
+115.42
+Swing High
+179.80
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_anet.png</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 154.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Arista Networks, Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.216, "estimated_spread": 0.0463, "executable_entry": 154.27, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 154.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 194252074580.01, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 154.4011, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 154.5323, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1311, "net_target_1_assumption": -0.0771, "net_target_2_assumption": -0.0771, "normalized_atr_score": 99.78, "normalized_liquidity_score": 82.35, "normalized_momentum_score": 100, "normalized_quality_score": 94.65, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 154.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 154.27, "ticker": "ANET", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>120.79</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>MRK
+No Trade
+0.00
+score
+Price
+120.79
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+115.60
+Fib Zone
+114.81 - 116.39
+Swing Low
+110.94
+Swing High
+123.13
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_mrk.png</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 120.79 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Merck &amp; Co., Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1691, "estimated_spread": 0.0362, "executable_entry": 120.79, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 120.79, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 298330093349.04, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 120.8927, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 120.9953, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1027, "net_target_1_assumption": -0.0604, "net_target_2_assumption": -0.0604, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.49, "normalized_momentum_score": 76.16, "normalized_quality_score": 70.82, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 120.79, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 120.79, "ticker": "MRK", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>UDR</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>UDR
+No Trade
+0.00
+score
+Price
+39.20
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+35.12
+Fib Zone
+34.93 - 35.31
+Swing Low
+33.07
+Swing High
+38.44
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_udr.png</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 39.20 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "UDR, Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1176, "estimated_spread": 0.0314, "executable_entry": 39.2, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 39.2, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 12736693845.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 39.2745, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 39.349, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0745, "net_target_1_assumption": -0.0451, "net_target_2_assumption": -0.0451, "normalized_atr_score": 100.0, "normalized_liquidity_score": 28.69, "normalized_momentum_score": 81.18, "normalized_quality_score": 70.14, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 39.2, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 39.2, "ticker": "UDR", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>312.37</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>JPM
+No Trade
+0.00
+score
+Price
+312.37
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+299.88
+Fib Zone
+298.30 - 301.47
+Swing Low
+293.67
+Swing High
+309.93
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_jpm.png</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 312.37 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "JPMorgan Chase &amp; Co.", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4373, "estimated_spread": 0.0937, "executable_entry": 312.37, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 312.37, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 836998968557.11, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 312.6355, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 312.901, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2655, "net_target_1_assumption": -0.1562, "net_target_2_assumption": -0.1562, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.16, "normalized_momentum_score": 83.05, "normalized_quality_score": 80.42, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 312.37, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 312.37, "ticker": "JPM", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>328</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>GE
+No Trade
+0.00
+score
+Price
+328.00
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+284.61
+Fib Zone
+282.14 - 287.07
+Swing Low
+268.91
+Swing High
+310.00
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_ge.png</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 328.00 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "GE Aerospace", "correlation_warning": false, "days_to_earnings": 28, "earnings_blackout": false, "earnings_date": "2026-07-16T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4592, "estimated_spread": 0.0984, "executable_entry": 328.0, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 328.0, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 342704109784.0, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 328.2788, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 328.5576, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2788, "net_target_1_assumption": -0.164, "net_target_2_assumption": -0.164, "normalized_atr_score": 100.0, "normalized_liquidity_score": 45.05, "normalized_momentum_score": 70.2, "normalized_quality_score": 70.11, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 328.0, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 328.0, "ticker": "GE", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>227.23</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>ABBV
+No Trade
+0.00
+score
+Price
+227.23
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+207.66
+Fib Zone
+206.26 - 209.05
+Swing Low
+200.02
+Swing High
+220.01
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_abbv.png</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 227.23 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "AbbVie Inc.", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3181, "estimated_spread": 0.0682, "executable_entry": 227.23, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 227.23, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 401468325167.28, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 227.4231, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 227.6163, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1931, "net_target_1_assumption": -0.1136, "net_target_2_assumption": -0.1136, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.65, "normalized_momentum_score": 71.99, "normalized_quality_score": 69.29, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 227.23, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 227.23, "ticker": "ABBV", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>54.87</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>SLB
+No Trade
+0.00
+score
+Price
+54.87
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+54.77
+Fib Zone
+54.33 - 55.21
+Swing Low
+52.45
+Swing High
+58.51
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_slb.png</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 54.87 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Schlumberger Limited", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0768, "estimated_spread": 0.0165, "executable_entry": 54.87, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 54.87, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 82033812262.18, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 54.9166, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 54.9633, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0466, "net_target_1_assumption": -0.0274, "net_target_2_assumption": -0.0274, "normalized_atr_score": 100.0, "normalized_liquidity_score": 56.73, "normalized_momentum_score": 100, "normalized_quality_score": 87.02, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 54.87, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 54.87, "ticker": "SLB", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>205.1</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>NVDA
+No Trade
+0.00
+score
+Price
+205.10
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+210.46
+Fib Zone
+208.33 - 212.59
+Swing Low
+194.51
+Swing High
+236.26
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_nvda.png</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 205.10 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, High Beta Growth, Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "NVIDIA Corporation", "correlation_warning": false, "days_to_earnings": 57, "earnings_blackout": false, "earnings_date": "2026-08-26T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2871, "estimated_spread": 0.0615, "executable_entry": 205.1, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "High Beta Growth", "Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 205.1, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 4967727247833.25, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 205.2743, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 205.4487, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1743, "net_target_1_assumption": -0.1026, "net_target_2_assumption": -0.1026, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 90.08, "normalized_quality_score": 95.54, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 205.1, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 205.1, "ticker": "NVDA", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>385.73</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>AVGO
+No Trade
+0.00
+score
+Price
+385.73
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+28%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+343.19
+Fib Zone
+337.54 - 348.85
+Swing Low
+289.96
+Swing High
+429.31
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_avgo.png</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 385.73 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: AI / Semiconductors, Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Broadcom Inc.", "correlation_warning": false, "days_to_earnings": 63, "earnings_blackout": false, "earnings_date": "2026-09-03T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.54, "estimated_spread": 0.1157, "executable_entry": 385.73, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["AI / Semiconductors", "Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 385.73, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1826303610630.94, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 386.0579, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 386.3857, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3279, "net_target_1_assumption": -0.1929, "net_target_2_assumption": -0.1929, "normalized_atr_score": 88.92, "normalized_liquidity_score": 100, "normalized_momentum_score": 82.06, "normalized_quality_score": 89.16, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 385.73, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 385.73, "ticker": "AVGO", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
+        <v>112.45</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>NOW
+No Trade
+0.00
+score
+Price
+112.45
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+95.14
+Fib Zone
+93.19 - 97.09
+Swing Low
+85.44
+Swing High
+110.83
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\charts\market_lens_agent_20260608_010748_now.png</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 112.45 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: High Beta Growth, Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ServiceNow, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.181, "estimated_spread": 0.0337, "executable_entry": 112.45, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 112.45, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 115970581452.7, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 112.5574, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 112.6648, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1074, "net_target_1_assumption": -0.0621, "net_target_2_assumption": -0.0621, "normalized_atr_score": 86.89, "normalized_liquidity_score": 100, "normalized_momentum_score": 57.36, "normalized_quality_score": 77.53, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 112.45, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 112.45, "ticker": "NOW", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
@@ -5016,7 +8745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="52" min="1" max="1"/>
@@ -5143,6 +8872,58 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\decisions\market_lens_agent_20260608_002548.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:09:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>20260608_010748</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>V AMAT PANW KLAC ORCL CRWD MU UNH MS SMCI CAT GS URI ASML LRCX TXN AMD C AAPL LLY TSM BAC UPS PSX UNP ANET MRK UDR JPM GE ABBV SLB NVDA AVGO NOW</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>V:WATCH, AMAT:SKIP, PANW:SKIP, KLAC:SKIP, ORCL:SKIP, CRWD:SKIP, MU:SKIP, UNH:SKIP, MS:SKIP, SMCI:SKIP, CAT:SKIP, GS:SKIP, URI:SKIP, ASML:SKIP, LRCX:SKIP, TXN:SKIP, AMD:SKIP, C:SKIP, AAPL:SKIP, LLY:SKIP, TSM:SKIP, BAC:SKIP, UPS:SKIP, PSX:SKIP, UNP:SKIP, ANET:SKIP, MRK:SKIP, UDR:SKIP, JPM:SKIP, GE:SKIP, ABBV:SKIP, SLB:SKIP, NVDA:SKIP, AVGO:SKIP, NOW:SKIP</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\summaries\market_lens_agent_20260608_010748.md</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\screenshots\market_lens_agent_20260608_010748.png</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\decisions\market_lens_agent_20260608_010748.jsonl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Avoid repeated skip scans and collapse agent actions
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -563,6 +563,7 @@
       <c r="G1" s="21" t="n"/>
       <c r="H1" s="21" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -897,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -8464,6 +8465,3961 @@
       <c r="R71" t="inlineStr">
         <is>
           <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "ServiceNow, Inc.", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.181, "estimated_spread": 0.0337, "executable_entry": 112.45, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["High Beta Growth", "Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 112.45, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 115970581452.7, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.1331, "ema200": 98.7805, "ema50": 98.9067, "price": 100.07, "return_1m": 1.85, "return_3m": 0.9, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 112.5574, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 112.6648, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1074, "net_target_1_assumption": -0.0621, "net_target_2_assumption": -0.0621, "normalized_atr_score": 86.89, "normalized_liquidity_score": 100, "normalized_momentum_score": 57.36, "normalized_quality_score": 77.53, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 112.45, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 112.45, "ticker": "NOW", "timestamp": "2026-06-08T01:09:18", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>OKE</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E72" t="n">
+        <v>88.25</v>
+      </c>
+      <c r="F72" t="n">
+        <v>87.78</v>
+      </c>
+      <c r="G72" t="n">
+        <v>89.02</v>
+      </c>
+      <c r="H72" t="n">
+        <v>86.06999999999999</v>
+      </c>
+      <c r="I72" t="n">
+        <v>88.7</v>
+      </c>
+      <c r="J72" t="n">
+        <v>96.06999999999999</v>
+      </c>
+      <c r="K72" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (88.40) with confluence at VWAP. Planned entry at zone low 87.78; executable entry 88.25, stop below fib 78.6% at 86.07. Structural confluence: swing low at 83.66 aligns with VAL (83.81).</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.10.</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>OKE
+Fib 61.8 Confluence Buy Zone
+0.49
+score
+Price
+88.25
+R/R
+1.39x
+Grade
+B
+Quality
+73%
+Buy Zone
+87.78 - 89.02
+Stop
+86.07
+Targets
+88.70 / 96.07
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Break above prior-day high at 89.52 after holding buy zone.
+Invalidation
+Exit if price closes below 86.07 or setup support fails.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (88.40) with confluence at VWAP. Planned entry at zone low 87.78; executable entry 88.25, stop below fib 78.6% at 86.07. Structural confluence: swing low at 83.66 aligns with VAL (83.81).
+Fib 61.8
+88.40
+Fib Zone
+87.78 - 89.02
+Swing Low
+83.66
+Swing High
+96.07
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_oke.png</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.49; R/R 1.39x; price 88.25 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.10; Factors: Energy | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.10.</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 89.02, "buy_zone_low": 87.78, "cash_available": 100000.0, "company_name": "ONEOK, Inc.", "correlation_warning": false, "days_to_earnings": -28, "earnings_blackout": false, "earnings_date": "2026-04-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2647, "estimated_spread": 0.0706, "executable_entry": 88.25, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_reward_1_per_share": 0.45, "gross_reward_2_per_share": 7.82, "gross_risk_per_share": 2.18, "gross_rr": 1.3897, "gross_rr_1": 0.2064, "gross_rr_2": 3.5872, "gross_rr_decision": 1.3897, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 55600399189.0, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 88.4177, "net_reward_1_per_share": 0.1808, "net_reward_2_per_share": 7.5508, "net_risk_per_share": 2.5154, "net_rr": 1.0974, "net_rr_1": 0.0719, "net_rr_2": 3.0019, "net_stop_assumption": 85.9023, "net_target_1_assumption": 88.5985, "net_target_2_assumption": 95.9685, "normalized_atr_score": 100.0, "normalized_liquidity_score": 38.57, "normalized_momentum_score": 66.9, "normalized_quality_score": 66.68, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 96.07, "price": 88.25, "prior_high_20": 96.07, "prior_high_63": 96.07, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.10.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.49, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.49, "stop_loss": 86.07, "target_1": 88.7, "target_1_atr_distance": 0.1827, "target_2": 96.07, "target_2_atr_distance": 3.1745, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 87.78, "ticker": "OKE", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E73" t="n">
+        <v>149.92</v>
+      </c>
+      <c r="F73" t="n">
+        <v>149.87</v>
+      </c>
+      <c r="G73" t="n">
+        <v>151.87</v>
+      </c>
+      <c r="H73" t="n">
+        <v>146.99</v>
+      </c>
+      <c r="I73" t="n">
+        <v>150.49</v>
+      </c>
+      <c r="J73" t="n">
+        <v>173.86</v>
+      </c>
+      <c r="K73" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (150.87) with confluence at VWAP. Planned entry at zone low 149.87; executable entry 149.92, stop below fib 78.6% at 146.99.</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>WATCH: Target 1 is too close versus daily ATR.</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>XOM
+Fib 61.8 Confluence Buy Zone
+0.49
+score
+Price
+149.92
+R/R
+2.98x
+Grade
+C
+Quality
+64%
+Buy Zone
+149.87 - 151.87
+Stop
+146.99
+Targets
+150.49 / 173.86
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Break above prior-day high at 153.43 after holding buy zone.
+Invalidation
+Exit if price closes below 146.99 or setup support fails.
+Trend quality is not clean.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (150.87) with confluence at VWAP. Planned entry at zone low 149.87; executable entry 149.92, stop below fib 78.6% at 146.99.
+Fib 61.8
+150.87
+Fib Zone
+149.87 - 151.87
+Swing Low
+142.95
+Swing High
+163.68
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_xom.png</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.49; R/R 2.98x; price 149.92 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.68; Factors: Energy | Agent action: WATCH - WATCH: Target 1 is too close versus daily ATR.</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 5996.8, "adjusted_position_size": 40, "adjusted_risk_amount": 117.2, "ask": 0.0, "bid": 0.0, "buy_zone_high": 151.87, "buy_zone_low": 149.87, "cash_available": 100000.0, "company_name": "Exxon Mobil Corporation", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-07-31T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2099, "estimated_spread": 0.045, "executable_entry": 149.92, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {"Energy": 5996.8}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_reward_1_per_share": 0.57, "gross_reward_2_per_share": 23.94, "gross_risk_per_share": 2.93, "gross_rr": 2.9862, "gross_rr_1": 0.1945, "gross_rr_2": 8.1706, "gross_rr_decision": 2.9862, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 621410470937.42, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 150.0474, "net_reward_1_per_share": 0.3676, "net_reward_2_per_share": 23.7376, "net_risk_per_share": 3.1849, "net_rr": 2.6837, "net_rr_1": 0.1154, "net_rr_2": 7.4533, "net_stop_assumption": 146.8626, "net_target_1_assumption": 150.415, "net_target_2_assumption": 173.785, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.97, "normalized_momentum_score": 55.95, "normalized_quality_score": 67.87, "original_cash_out": 9894.72, "original_position_size": 66, "original_risk_amount": 193.38, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": true, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 40 shares, cash 5996.80, risk 117.20.", "previous_resistance": 163.68, "price": 149.92, "prior_high_20": 163.68, "prior_high_63": 175.2207, "reason": "WATCH: Target 1 is too close versus daily ATR.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 5996.8, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.49, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "Position size reduced by Energy sector exposure cap (66 -&gt; 40 shares).", "spread_source": "liquidity_fallback", "stock_score": 0.49, "stop_loss": 146.99, "target_1": 150.49, "target_1_atr_distance": 0.1428, "target_2": 173.86, "target_2_atr_distance": 5.9956, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 149.87, "ticker": "XOM", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR.", "Position size reduced by Energy sector exposure cap (66 -&gt; 40 shares)."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E74" t="n">
+        <v>323.57</v>
+      </c>
+      <c r="F74" t="n">
+        <v>321.22</v>
+      </c>
+      <c r="G74" t="n">
+        <v>324.81</v>
+      </c>
+      <c r="H74" t="n">
+        <v>319</v>
+      </c>
+      <c r="I74" t="n">
+        <v>325.34</v>
+      </c>
+      <c r="J74" t="n">
+        <v>338.49</v>
+      </c>
+      <c r="K74" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (323.02) with confluence at VWAP. Planned entry at zone low 321.22; executable entry 323.57, stop below fib 78.6% at 319.00.</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>V
+Fib 61.8 Confluence Buy Zone
+0.45
+score
+Price
+323.57
+R/R
+1.39x
+Grade
+B
+Quality
+70%
+Buy Zone
+321.22 - 324.81
+Stop
+319.00
+Targets
+325.34 / 338.49
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+Trigger
+Break above prior-day high at 324.76 after holding buy zone.
+Invalidation
+Exit if price closes below 319.00 or setup support fails.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (323.02) with confluence at VWAP. Planned entry at zone low 321.22; executable entry 323.57, stop below fib 78.6% at 319.00.
+Fib 61.8
+323.02
+Fib Zone
+321.22 - 324.81
+Swing Low
+315.51
+Swing High
+335.17
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_v.png</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.45; R/R 1.39x; price 323.57 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.16; Factors: Financials | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 324.81, "buy_zone_low": 321.22, "cash_available": 100000.0, "company_name": "Visa Inc.", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.453, "estimated_spread": 0.0971, "executable_entry": 323.57, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_reward_1_per_share": 1.77, "gross_reward_2_per_share": 14.92, "gross_risk_per_share": 4.57, "gross_rr": 1.3944, "gross_rr_1": 0.3873, "gross_rr_2": 3.2648, "gross_rr_decision": 1.3944, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 615347255294.79, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 323.845, "net_reward_1_per_share": 1.3332, "net_reward_2_per_share": 14.4832, "net_risk_per_share": 5.1201, "net_rr": 1.1593, "net_rr_1": 0.2604, "net_rr_2": 2.8287, "net_stop_assumption": 318.725, "net_target_1_assumption": 325.1782, "net_target_2_assumption": 338.3282, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.95, "normalized_momentum_score": 60.9, "normalized_quality_score": 70.39, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 335.17, "price": 323.57, "prior_high_20": 335.17, "prior_high_63": 341.2725, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.39 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.16.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.45, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.45, "stop_loss": 319.0, "target_1": 325.34, "target_1_atr_distance": 0.2466, "target_2": 338.49, "target_2_atr_distance": 2.0787, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 321.22, "ticker": "V", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>VWAP Reclaim Setup</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E75" t="n">
+        <v>187.31</v>
+      </c>
+      <c r="F75" t="n">
+        <v>186.04</v>
+      </c>
+      <c r="G75" t="n">
+        <v>188.58</v>
+      </c>
+      <c r="H75" t="n">
+        <v>182.39</v>
+      </c>
+      <c r="I75" t="n">
+        <v>189.98</v>
+      </c>
+      <c r="J75" t="n">
+        <v>204.51</v>
+      </c>
+      <c r="K75" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Price (187.31) reclaiming VWAP (187.85) after trading below it. Volume confirming. Anchored VWAP context 186.37 is supportive. Entry at 187.31, stop at 182.39.</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.58 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.43.</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>CVX
+VWAP Reclaim Setup
+0.45
+score
+Price
+187.31
+R/R
+1.58x
+Grade
+C
+Quality
+64%
+Buy Zone
+186.04 - 188.58
+Stop
+182.39
+Targets
+189.98 / 204.51
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Hold VWAP and break above 190.10.
+Invalidation
+Exit if price closes below 182.39 or setup support fails.
+Trend quality is not clean.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (187.31) reclaiming VWAP (187.85) after trading below it. Volume confirming. Anchored VWAP context 186.37 is supportive. Entry at 187.31, stop at 182.39.
+Fib 61.8
+185.91
+Fib Zone
+184.85 - 186.97
+Swing Low
+177.90
+Swing High
+198.87
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_cvx.png</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: VWAP Reclaim Setup; score 0.45; R/R 1.58x; price 187.31 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.43; Factors: Energy | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.58 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.43.</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 188.58, "buy_zone_low": 186.04, "cash_available": 100000.0, "company_name": "Chevron Corporation", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-07-31T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2622, "estimated_spread": 0.0562, "executable_entry": 187.31, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_reward_1_per_share": 2.67, "gross_reward_2_per_share": 17.2, "gross_risk_per_share": 4.92, "gross_rr": 1.5763, "gross_rr_1": 0.5427, "gross_rr_2": 3.4959, "gross_rr_decision": 1.5763, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 373046166318.62, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 187.4692, "net_reward_1_per_share": 2.4171, "net_reward_2_per_share": 16.9471, "net_risk_per_share": 5.2384, "net_rr": 1.4322, "net_rr_1": 0.4614, "net_rr_2": 3.2352, "net_stop_assumption": 182.2308, "net_target_1_assumption": 189.8863, "net_target_2_assumption": 204.4163, "normalized_atr_score": 100.0, "normalized_liquidity_score": 49.74, "normalized_momentum_score": 54.93, "normalized_quality_score": 64.64, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 198.87, "price": 187.31, "prior_high_20": 198.87, "prior_high_63": 212.7613, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.58 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.43.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.45, "setup_type": "VWAP Reclaim Setup", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.45, "stop_loss": 182.39, "target_1": 189.98, "target_1_atr_distance": 0.6284, "target_2": 204.51, "target_2_atr_distance": 4.0483, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 186.04, "ticker": "CVX", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ELAN</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E76" t="n">
+        <v>23.63</v>
+      </c>
+      <c r="F76" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="G76" t="n">
+        <v>23.69</v>
+      </c>
+      <c r="H76" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="I76" t="n">
+        <v>23.94</v>
+      </c>
+      <c r="J76" t="n">
+        <v>26.29</v>
+      </c>
+      <c r="K76" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (23.40) with confluence at POC, VWAP. Planned entry at zone low 23.11; executable entry 23.63, stop below fib 78.6% at 22.50.</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.01 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.87.</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>ELAN
+Fib 61.8 Confluence Buy Zone
+0.44
+score
+Price
+23.63
+R/R
+1.01x
+Grade
+C
+Quality
+65%
+Buy Zone
+23.11 - 23.69
+Stop
+22.50
+Targets
+23.94 / 26.29
+Watch only; needs confirmation
+Mixed
+Relative Strength
+In line
+50%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+Trigger
+Break above prior-day high at 26.23 after holding buy zone.
+Invalidation
+Exit if price closes below 22.50 or setup support fails.
+Market regime: Mixed.
+Relative strength: In line.
+Price at 61.8% fib retracement (23.40) with confluence at POC, VWAP. Planned entry at zone low 23.11; executable entry 23.63, stop below fib 78.6% at 22.50.
+Fib 61.8
+23.40
+Fib Zone
+23.11 - 23.69
+Swing Low
+21.62
+Swing High
+26.29
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_elan.png</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.44; R/R 1.01x; price 23.63 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.87; Factors: Defensive, Healthcare | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.01 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.87.</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 23.69, "buy_zone_low": 23.11, "cash_available": 100000.0, "company_name": "Elanco Animal Health Incorporated", "correlation_warning": false, "days_to_earnings": 43, "earnings_blackout": false, "earnings_date": "2026-08-06T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0709, "estimated_spread": 0.0189, "executable_entry": 23.63, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "WATCH", "gross_reward_1_per_share": 0.31, "gross_reward_2_per_share": 2.66, "gross_risk_per_share": 1.13, "gross_rr": 1.0022, "gross_rr_1": 0.2743, "gross_rr_2": 2.354, "gross_rr_decision": 1.0022, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 11801993227.14, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 23.6749, "net_reward_1_per_share": 0.2379, "net_reward_2_per_share": 2.5879, "net_risk_per_share": 1.2198, "net_rr": 0.8694, "net_rr_1": 0.1951, "net_rr_2": 2.1216, "net_stop_assumption": 22.4551, "net_target_1_assumption": 23.9128, "net_target_2_assumption": 26.2628, "normalized_atr_score": 100.0, "normalized_liquidity_score": 23.93, "normalized_momentum_score": 43.32, "normalized_quality_score": 51.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 26.23, "price": 23.63, "prior_high_20": 26.23, "prior_high_63": 26.29, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.01 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.87.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.44, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.44, "stop_loss": 22.5, "target_1": 23.94, "target_1_atr_distance": 0.268, "target_2": 26.29, "target_2_atr_distance": 2.2992, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 23.11, "ticker": "ELAN", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E77" t="n">
+        <v>416.67</v>
+      </c>
+      <c r="F77" t="n">
+        <v>414.17</v>
+      </c>
+      <c r="G77" t="n">
+        <v>427.06</v>
+      </c>
+      <c r="H77" t="n">
+        <v>407.73</v>
+      </c>
+      <c r="I77" t="n">
+        <v>426.34</v>
+      </c>
+      <c r="J77" t="n">
+        <v>444.49</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Price (416.67) retesting broken resistance (427.06) as support. Breakout on 2026-05-29 with 2.3× avg volume. Volume confirmed breakout. Entry at 416.67, stop at 407.73.</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.79 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.42.</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>MSFT
+Breakout + Retest
+0.43
+score
+Price
+416.67
+R/R
+1.79x
+Grade
+B
+Quality
+76%
+Buy Zone
+414.17 - 427.06
+Stop
+407.73
+Targets
+426.34 / 444.49
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Close above 436.15 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 407.73 or setup support fails.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (416.67) retesting broken resistance (427.06) as support. Breakout on 2026-05-29 with 2.3× avg volume. Volume confirmed breakout. Entry at 416.67, stop at 407.73.
+Fib 61.8
+412.14
+Fib Zone
+408.92 - 415.36
+Swing Low
+400.01
+Swing High
+431.76
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_msft.png</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: Breakout + Retest; score 0.43; R/R 1.79x; price 416.67 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.42; Factors: Mega Cap Tech, Rates-sensitive Growth, Technology | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.79 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.42.</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 427.06, "buy_zone_low": 414.17, "cash_available": 100000.0, "company_name": "Microsoft Corporation", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.4167, "estimated_spread": 0.125, "executable_entry": 416.67, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Mega Cap Tech", "Rates-sensitive Growth", "Technology"], "final_action": "WATCH", "gross_reward_1_per_share": 9.67, "gross_reward_2_per_share": 27.82, "gross_risk_per_share": 8.94, "gross_rr": 1.7922, "gross_rr_1": 1.0817, "gross_rr_2": 3.1119, "gross_rr_decision": 1.7922, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 3095205987862.73, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 417.4408, "net_reward_1_per_share": 8.4825, "net_reward_2_per_share": 26.6325, "net_risk_per_share": 10.4817, "net_rr": 1.4153, "net_rr_1": 0.8093, "net_rr_2": 2.5409, "net_stop_assumption": 406.9592, "net_target_1_assumption": 425.9233, "net_target_2_assumption": 444.0733, "normalized_atr_score": 100.0, "normalized_liquidity_score": 100, "normalized_momentum_score": 55.96, "normalized_quality_score": 80.18, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 466.32, "price": 416.67, "prior_high_20": 466.32, "prior_high_63": 466.32, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.79 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.42.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.43, "setup_type": "Breakout + Retest", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.43, "stop_loss": 407.73, "target_1": 426.34, "target_1_atr_distance": 0.7507, "target_2": 444.49, "target_2_atr_distance": 2.1598, "target_feasibility_status": "OK", "theoretical_entry": 414.17, "ticker": "MSFT", "timestamp": "2026-06-08T01:37:33", "warnings": []}</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>AIG</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E78" t="n">
+        <v>75.48999999999999</v>
+      </c>
+      <c r="F78" t="n">
+        <v>75.13</v>
+      </c>
+      <c r="G78" t="n">
+        <v>76.02</v>
+      </c>
+      <c r="H78" t="n">
+        <v>74.26000000000001</v>
+      </c>
+      <c r="I78" t="n">
+        <v>76.38</v>
+      </c>
+      <c r="J78" t="n">
+        <v>79.77</v>
+      </c>
+      <c r="K78" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (75.57) with confluence at VWAP. Planned entry at zone low 75.13; executable entry 75.49, stop below fib 78.6% at 74.26.</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.68 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.22.</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>AIG
+Fib 61.8 Confluence Buy Zone
+0.43
+score
+Price
+75.49
+R/R
+1.68x
+Grade
+C
+Quality
+59%
+Buy Zone
+75.13 - 76.02
+Stop
+74.26
+Targets
+76.38 / 79.77
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+94%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Break above prior-day high at 75.49 after holding buy zone.
+Invalidation
+Exit if price closes below 74.26 or setup support fails.
+Trend quality is not clean.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (75.57) with confluence at VWAP. Planned entry at zone low 75.13; executable entry 75.49, stop below fib 78.6% at 74.26.
+Fib 61.8
+75.57
+Fib Zone
+75.13 - 76.02
+Swing Low
+72.98
+Swing High
+79.77
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_aig.png</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.43; R/R 1.68x; price 75.49 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.22; Factors: Financials | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.68 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.22.</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 76.02, "buy_zone_low": 75.13, "cash_available": 100000.0, "company_name": "American International Group, Inc.", "correlation_warning": false, "days_to_earnings": -26, "earnings_blackout": false, "earnings_date": "2026-04-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2265, "estimated_spread": 0.0604, "executable_entry": 75.49, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_reward_1_per_share": 0.89, "gross_reward_2_per_share": 4.28, "gross_risk_per_share": 1.23, "gross_rr": 1.6882, "gross_rr_1": 0.7236, "gross_rr_2": 3.4797, "gross_rr_decision": 1.6882, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 40025266490.65, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 75.6334, "net_reward_1_per_share": 0.6598, "net_reward_2_per_share": 4.0498, "net_risk_per_share": 1.5169, "net_rr": 1.2172, "net_rr_1": 0.4349, "net_rr_2": 2.6698, "net_stop_assumption": 74.1166, "net_target_1_assumption": 76.2932, "net_target_2_assumption": 79.6832, "normalized_atr_score": 100.0, "normalized_liquidity_score": 33.59, "normalized_momentum_score": 41.09, "normalized_quality_score": 53.57, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 78.92, "price": 75.49, "prior_high_20": 78.92, "prior_high_63": 79.77, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.68 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.22.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.43, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.43, "stop_loss": 74.26, "target_1": 76.38, "target_1_atr_distance": 0.5033, "target_2": 79.77, "target_2_atr_distance": 2.4203, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 75.13, "ticker": "AIG", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Breakout + Retest</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E79" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="F79" t="n">
+        <v>62.05</v>
+      </c>
+      <c r="G79" t="n">
+        <v>64.13</v>
+      </c>
+      <c r="H79" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="I79" t="n">
+        <v>64.56999999999999</v>
+      </c>
+      <c r="J79" t="n">
+        <v>69.36</v>
+      </c>
+      <c r="K79" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Price (62.59) retesting broken resistance (64.13) as support. Breakout on 2026-04-23 with 1.5× avg volume. Volume confirmed breakout. Entry at 62.59, stop at 61.01.</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>WATCH: Neutral market requires stronger setup score (0.41 &lt; 0.45).</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>BKR
+Breakout + Retest
+0.41
+score
+Price
+62.59
+R/R
+2.31x
+Grade
+C
+Quality
+63%
+Buy Zone
+62.05 - 64.13
+Stop
+61.01
+Targets
+64.57 / 69.36
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+45%
+Trigger
+Close above 66.24 or reclaim of broken resistance.
+Invalidation
+Exit if price closes below 61.01 or setup support fails.
+Trend quality is not clean.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (62.59) retesting broken resistance (64.13) as support. Breakout on 2026-04-23 with 1.5× avg volume. Volume confirmed breakout. Entry at 62.59, stop at 61.01.
+Fib 61.8
+64.55
+Fib Zone
+64.03 - 65.07
+Swing Low
+62.46
+Swing High
+67.92
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_bkr.png</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Breakout + Retest; score 0.41; R/R 2.31x; price 62.59 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.74; Factors: Energy | Agent action: WATCH - WATCH: Neutral market requires stronger setup score (0.41 &lt; 0.45).</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 5946.05, "adjusted_position_size": 95, "adjusted_risk_amount": 150.1, "ask": 0.0, "bid": 0.0, "buy_zone_high": 64.13, "buy_zone_low": 62.05, "cash_available": 100000.0, "company_name": "Baker Hughes Company", "correlation_warning": false, "days_to_earnings": 31, "earnings_blackout": false, "earnings_date": "2026-07-21T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.313, "estimated_spread": 0.0501, "executable_entry": 62.59, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {"Energy": 5946.05}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_reward_1_per_share": 1.98, "gross_reward_2_per_share": 6.77, "gross_risk_per_share": 1.58, "gross_rr": 2.3142, "gross_rr_1": 1.2532, "gross_rr_2": 4.2848, "gross_rr_decision": 2.3142, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 62093579896.61, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 62.7715, "net_reward_1_per_share": 1.6952, "net_reward_2_per_share": 6.4852, "net_risk_per_share": 1.943, "net_rr": 1.7353, "net_rr_1": 0.8725, "net_rr_2": 3.3377, "net_stop_assumption": 60.8285, "net_target_1_assumption": 64.4667, "net_target_2_assumption": 69.2567, "normalized_atr_score": 100.0, "normalized_liquidity_score": 47.52, "normalized_momentum_score": 62.0, "normalized_quality_score": 67.16, "original_cash_out": 9951.81, "original_position_size": 159, "original_risk_amount": 251.22, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": true, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 95 shares, cash 5946.05, risk 150.10.", "previous_resistance": 67.92, "price": 62.59, "prior_high_20": 67.92, "prior_high_63": 70.1753, "reason": "WATCH: Neutral market requires stronger setup score (0.41 &lt; 0.45).", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 5946.05, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.41, "setup_type": "Breakout + Retest", "sizing_adjustment_reason": "Position size reduced by Energy sector exposure cap (159 -&gt; 95 shares).", "spread_source": "liquidity_fallback", "stock_score": 0.41, "stop_loss": 61.01, "target_1": 64.57, "target_1_atr_distance": 0.953, "target_2": 69.36, "target_2_atr_distance": 3.2586, "target_feasibility_status": "OK", "theoretical_entry": 62.05, "ticker": "BKR", "timestamp": "2026-06-08T01:37:33", "warnings": ["Position size reduced by Energy sector exposure cap (159 -&gt; 95 shares).", "WATCH: Gross R/R is valid, but Net R/R 1.74 failed after slippage/spread adjustment."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="E80" t="n">
+        <v>117.14</v>
+      </c>
+      <c r="F80" t="n">
+        <v>116.7</v>
+      </c>
+      <c r="G80" t="n">
+        <v>118.25</v>
+      </c>
+      <c r="H80" t="n">
+        <v>114.49</v>
+      </c>
+      <c r="I80" t="n">
+        <v>117.87</v>
+      </c>
+      <c r="J80" t="n">
+        <v>134.17</v>
+      </c>
+      <c r="K80" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (117.48) with confluence at VWAP. Planned entry at zone low 116.70; executable entry 117.14, stop below fib 78.6% at 114.49.</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>WATCH: Neutral market requires stronger setup score (0.39 &lt; 0.45).</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>COP
+Fib 61.8 Confluence Buy Zone
+0.39
+score
+Price
+117.14
+R/R
+2.43x
+Grade
+C
+Quality
+63%
+Buy Zone
+116.70 - 118.25
+Stop
+114.49
+Targets
+117.87 / 134.17
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Break above prior-day high at 119.58 after holding buy zone.
+Invalidation
+Exit if price closes below 114.49 or setup support fails.
+Trend quality is not clean.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (117.48) with confluence at VWAP. Planned entry at zone low 116.70; executable entry 117.14, stop below fib 78.6% at 114.49.
+Fib 61.8
+117.48
+Fib Zone
+116.70 - 118.25
+Swing Low
+111.38
+Swing High
+127.33
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_cop.png</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.39; R/R 2.43x; price 117.14 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.20; Factors: Energy | Agent action: WATCH - WATCH: Neutral market requires stronger setup score (0.39 &lt; 0.45).</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 5974.14, "adjusted_position_size": 51, "adjusted_risk_amount": 135.15, "ask": 0.0, "bid": 0.0, "buy_zone_high": 118.25, "buy_zone_low": 116.7, "cash_available": 100000.0, "company_name": "ConocoPhillips", "correlation_warning": false, "days_to_earnings": 43, "earnings_blackout": false, "earnings_date": "2026-08-06T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.164, "estimated_spread": 0.0351, "executable_entry": 117.14, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {"Energy": 5974.14}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "WATCH", "gross_reward_1_per_share": 0.73, "gross_reward_2_per_share": 17.03, "gross_risk_per_share": 2.65, "gross_rr": 2.4283, "gross_rr_1": 0.2755, "gross_rr_2": 6.4264, "gross_rr_decision": 2.4283, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "BUY_SIMULATED", "market_cap": 142710959236.39, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 117.2396, "net_reward_1_per_share": 0.5719, "net_reward_2_per_share": 16.8719, "net_risk_per_share": 2.8491, "net_rr": 2.2031, "net_rr_1": 0.2007, "net_rr_2": 5.9217, "net_stop_assumption": 114.3904, "net_target_1_assumption": 117.8114, "net_target_2_assumption": 134.1114, "normalized_atr_score": 100.0, "normalized_liquidity_score": 59.07, "normalized_momentum_score": 57.04, "normalized_quality_score": 68.39, "original_cash_out": 9956.9, "original_position_size": 85, "original_risk_amount": 225.25, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": true, "position_sizing_explanation": "Base position sizing produced a candidate trade, but the risk transparency layer blocked the new buy. Candidate size: 51 shares, cash 5974.14, risk 135.15.", "previous_resistance": 126.0, "price": 117.14, "prior_high_20": 126.0, "prior_high_63": 134.8677, "reason": "WATCH: Neutral market requires stronger setup score (0.39 &lt; 0.45).", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 5974.14, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.39, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "Position size reduced by Energy sector exposure cap (85 -&gt; 51 shares).", "spread_source": "liquidity_fallback", "stock_score": 0.39, "stop_loss": 114.49, "target_1": 117.87, "target_1_atr_distance": 0.2365, "target_2": 134.17, "target_2_atr_distance": 5.5183, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 116.7, "ticker": "COP", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR.", "Position size reduced by Energy sector exposure cap (85 -&gt; 51 shares).", "WATCH: Neutral sector requires a cleaner setup score.", "WATCH: Gross R/R is valid, but Net R/R 2.20 failed after slippage/spread adjustment.", "WATCH: Target 1 is too close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>AXP</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E81" t="n">
+        <v>310.66</v>
+      </c>
+      <c r="F81" t="n">
+        <v>307.44</v>
+      </c>
+      <c r="G81" t="n">
+        <v>311.01</v>
+      </c>
+      <c r="H81" t="n">
+        <v>305.79</v>
+      </c>
+      <c r="I81" t="n">
+        <v>311.14</v>
+      </c>
+      <c r="J81" t="n">
+        <v>333.13</v>
+      </c>
+      <c r="K81" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (309.23) with confluence at POC, VWAP. Planned entry at zone low 307.44; executable entry 310.66, stop below fib 78.6% at 305.79. Structural confluence: swing low at 303.04 aligns with HVN (302.06).</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.68 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.44.</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>AXP
+Fib 61.8 Confluence Buy Zone
+0.34
+score
+Price
+310.66
+R/R
+1.68x
+Grade
+C
+Quality
+63%
+Buy Zone
+307.44 - 311.01
+Stop
+305.79
+Targets
+311.14 / 333.13
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+Trigger
+Break above prior-day high at 314.96 after holding buy zone.
+Invalidation
+Exit if price closes below 305.79 or setup support fails.
+Trend quality is not clean.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (309.23) with confluence at POC, VWAP. Planned entry at zone low 307.44; executable entry 310.66, stop below fib 78.6% at 305.79. Structural confluence: swing low at 303.04 aligns with HVN (302.06).
+Fib 61.8
+309.23
+Fib Zone
+307.44 - 311.01
+Swing Low
+303.04
+Swing High
+319.24
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_axp.png</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.34; R/R 1.68x; price 310.66 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.44; Factors: Financials | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.68 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.44.</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 311.01, "buy_zone_low": 307.44, "cash_available": 100000.0, "company_name": "American Express Company", "correlation_warning": false, "days_to_earnings": 34, "earnings_blackout": false, "earnings_date": "2026-07-24T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4349, "estimated_spread": 0.0932, "executable_entry": 310.66, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "WATCH", "gross_reward_1_per_share": 0.48, "gross_reward_2_per_share": 22.47, "gross_risk_per_share": 4.87, "gross_rr": 1.679, "gross_rr_1": 0.0986, "gross_rr_2": 4.614, "gross_rr_decision": 1.679, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 211971535281.13, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 310.9241, "net_reward_1_per_share": 0.0606, "net_reward_2_per_share": 22.0506, "net_risk_per_share": 5.3981, "net_rr": 1.437, "net_rr_1": 0.0112, "net_rr_2": 4.0849, "net_stop_assumption": 305.5259, "net_target_1_assumption": 310.9847, "net_target_2_assumption": 332.9747, "normalized_atr_score": 100.0, "normalized_liquidity_score": 35.29, "normalized_momentum_score": 53.35, "normalized_quality_score": 59.59, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 324.54, "price": 310.66, "prior_high_20": 324.54, "prior_high_63": 339.98, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.68 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.44.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.34, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.34, "stop_loss": 305.79, "target_1": 311.14, "target_1_atr_distance": 0.0672, "target_2": 333.13, "target_2_atr_distance": 3.1456, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 307.44, "ticker": "AXP", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>DHR</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>VWAP Reclaim Setup</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E82" t="n">
+        <v>184.3</v>
+      </c>
+      <c r="F82" t="n">
+        <v>182.7</v>
+      </c>
+      <c r="G82" t="n">
+        <v>185.9</v>
+      </c>
+      <c r="H82" t="n">
+        <v>178.98</v>
+      </c>
+      <c r="I82" t="n">
+        <v>187.66</v>
+      </c>
+      <c r="J82" t="n">
+        <v>196.09</v>
+      </c>
+      <c r="K82" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Price (184.30) reclaiming VWAP (185.00) after trading below it. Volume confirming. Anchored VWAP context 175.57 is supportive. Entry at 184.30, stop at 178.98.</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.19 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.08.</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>DHR
+VWAP Reclaim Setup
+0.33
+score
+Price
+184.30
+R/R
+1.19x
+Grade
+B
+Quality
+74%
+Buy Zone
+182.70 - 185.90
+Stop
+178.98
+Targets
+187.66 / 196.09
+Tradable if trigger confirms
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Hold VWAP and break above 187.79.
+Invalidation
+Exit if price closes below 178.98 or setup support fails.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (184.30) reclaiming VWAP (185.00) after trading below it. Volume confirming. Anchored VWAP context 175.57 is supportive. Entry at 184.30, stop at 178.98.
+Fib 61.8
+188.46
+Fib Zone
+187.12 - 189.79
+Swing Low
+181.01
+Swing High
+200.50
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_dhr.png</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: VWAP Reclaim Setup; score 0.33; R/R 1.19x; price 184.30 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.08; Factors: Defensive, Healthcare | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.19 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.08.</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 185.9, "buy_zone_low": 182.7, "cash_available": 100000.0, "company_name": "Danaher Corporation", "correlation_warning": false, "days_to_earnings": 31, "earnings_blackout": false, "earnings_date": "2026-07-21T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.258, "estimated_spread": 0.0553, "executable_entry": 184.3, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "WATCH", "gross_reward_1_per_share": 3.36, "gross_reward_2_per_share": 11.79, "gross_risk_per_share": 5.32, "gross_rr": 1.1862, "gross_rr_1": 0.6316, "gross_rr_2": 2.2162, "gross_rr_decision": 1.1862, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 130442128716.04, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 184.4567, "net_reward_1_per_share": 3.1112, "net_reward_2_per_share": 11.5412, "net_risk_per_share": 5.6333, "net_rr": 1.076, "net_rr_1": 0.5523, "net_rr_2": 2.0487, "net_stop_assumption": 178.8233, "net_target_1_assumption": 187.5678, "net_target_2_assumption": 195.9978, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.96, "normalized_momentum_score": 35.16, "normalized_quality_score": 59.11, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 187.79, "price": 184.3, "prior_high_20": 187.79, "prior_high_63": 200.5, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.19 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.08.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.33, "setup_type": "VWAP Reclaim Setup", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.33, "stop_loss": 178.98, "target_1": 187.66, "target_1_atr_distance": 0.631, "target_2": 196.09, "target_2_atr_distance": 2.2142, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 182.7, "ticker": "DHR", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>VWAP Reclaim Setup</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E83" t="n">
+        <v>26.04</v>
+      </c>
+      <c r="F83" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="G83" t="n">
+        <v>26.19</v>
+      </c>
+      <c r="H83" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="I83" t="n">
+        <v>26.28</v>
+      </c>
+      <c r="J83" t="n">
+        <v>27.57</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Price (26.04) reclaiming VWAP (26.04) after trading below it. Volume confirming. Anchored VWAP context 25.81 is supportive. Entry at 26.04, stop at 25.48.</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.24 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.09.</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>PFE
+VWAP Reclaim Setup
+0.32
+score
+Price
+26.04
+R/R
+1.24x
+Grade
+C
+Quality
+63%
+Buy Zone
+25.89 - 26.19
+Stop
+25.48
+Targets
+26.28 / 27.57
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+Trigger
+Hold VWAP and break above 26.04.
+Invalidation
+Exit if price closes below 25.48 or setup support fails.
+Trend quality is not clean.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price (26.04) reclaiming VWAP (26.04) after trading below it. Volume confirming. Anchored VWAP context 25.81 is supportive. Entry at 26.04, stop at 25.48.
+Fib 61.8
+25.71
+Fib Zone
+25.58 - 25.83
+Swing Low
+25.19
+Swing High
+26.54
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_pfe.png</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: VWAP Reclaim Setup; score 0.32; R/R 1.24x; price 26.04 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 1.09; Factors: Defensive, Healthcare | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.24 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.09.</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 26.19, "buy_zone_low": 25.89, "cash_available": 100000.0, "company_name": "Pfizer Inc.", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0365, "estimated_spread": 0.0078, "executable_entry": 26.04, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "WATCH", "gross_reward_1_per_share": 0.24, "gross_reward_2_per_share": 1.53, "gross_risk_per_share": 0.56, "gross_rr": 1.2348, "gross_rr_1": 0.4286, "gross_rr_2": 2.7321, "gross_rr_decision": 1.2348, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 148413531378.76, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 26.0621, "net_reward_1_per_share": 0.2048, "net_reward_2_per_share": 1.4948, "net_risk_per_share": 0.6043, "net_rr": 1.0862, "net_rr_1": 0.339, "net_rr_2": 2.4738, "net_stop_assumption": 25.4579, "net_target_1_assumption": 26.267, "net_target_2_assumption": 27.557, "normalized_atr_score": 100.0, "normalized_liquidity_score": 62.09, "normalized_momentum_score": 45.88, "normalized_quality_score": 64.27, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 26.54, "price": 26.04, "prior_high_20": 26.54, "prior_high_63": 28.2831, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.24 is below minimum 2.00. Market regime NEUTRAL; sector NEUTRAL; net R/R 1.09.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.32, "setup_type": "VWAP Reclaim Setup", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.32, "stop_loss": 25.48, "target_1": 26.28, "target_1_atr_distance": 0.496, "target_2": 27.57, "target_2_atr_distance": 3.1618, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 25.89, "ticker": "PFE", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>DLR</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Fib 61.8 Confluence Buy Zone</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E84" t="n">
+        <v>186.79</v>
+      </c>
+      <c r="F84" t="n">
+        <v>185.45</v>
+      </c>
+      <c r="G84" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="H84" t="n">
+        <v>180.17</v>
+      </c>
+      <c r="I84" t="n">
+        <v>187.64</v>
+      </c>
+      <c r="J84" t="n">
+        <v>208.14</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Price at 61.8% fib retracement (186.47) with confluence at VWAP. Planned entry at zone low 185.45; executable entry 186.79, stop below fib 78.6% at 180.17.</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>WATCH: Technical setup detected, but weighted risk/reward 1.21 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.02.</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>DLR
+Fib 61.8 Confluence Buy Zone
+0.24
+score
+Price
+186.79
+R/R
+1.21x
+Grade
+C
+Quality
+54%
+Buy Zone
+185.45 - 187.50
+Stop
+180.17
+Targets
+187.64 / 208.14
+Watch only; needs confirmation
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+Trigger
+Break above prior-day high at 189.25 after holding buy zone.
+Invalidation
+Exit if price closes below 180.17 or setup support fails.
+Trend quality is not clean.
+Recent volume shows distribution risk.
+Market regime: Mixed.
+Relative strength: Leadership.
+Price at 61.8% fib retracement (186.47) with confluence at VWAP. Planned entry at zone low 185.45; executable entry 186.79, stop below fib 78.6% at 180.17.
+Fib 61.8
+186.47
+Fib Zone
+185.45 - 187.50
+Swing Low
+173.08
+Swing High
+208.14
+Save setup
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_dlr.png</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.24; R/R 1.21x; price 186.79 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 1.02; Factors: Real Estate | Agent action: WATCH - WATCH: Technical setup detected, but weighted risk/reward 1.21 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.02.</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 187.5, "buy_zone_low": 185.45, "cash_available": 100000.0, "company_name": "Digital Realty", "correlation_warning": false, "days_to_earnings": 33, "earnings_blackout": false, "earnings_date": "2026-07-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5604, "estimated_spread": 0.1494, "executable_entry": 186.79, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "WATCH", "gross_reward_1_per_share": 0.85, "gross_reward_2_per_share": 21.35, "gross_risk_per_share": 6.62, "gross_rr": 1.2122, "gross_rr_1": 0.1284, "gross_rr_2": 3.2251, "gross_rr_decision": 1.2122, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "WATCH", "market_cap": 65639137456.01, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "net_entry": 187.1449, "net_reward_1_per_share": 0.2803, "net_reward_2_per_share": 20.7803, "net_risk_per_share": 7.3298, "net_rr": 1.0171, "net_rr_1": 0.0382, "net_rr_2": 2.835, "net_stop_assumption": 179.8151, "net_target_1_assumption": 187.4252, "net_target_2_assumption": 207.9252, "normalized_atr_score": 100.0, "normalized_liquidity_score": 40.59, "normalized_momentum_score": 58.42, "normalized_quality_score": 63.47, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 199.2, "price": 186.79, "prior_high_20": 199.2, "prior_high_63": 208.14, "reason": "WATCH: Technical setup detected, but weighted risk/reward 1.21 is below minimum 2.00. Market regime NEUTRAL; sector STRONG; net R/R 1.02.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.24, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.24, "stop_loss": 180.17, "target_1": 187.64, "target_1_atr_distance": 0.207, "target_2": 208.14, "target_2_atr_distance": 5.1987, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 185.45, "ticker": "DLR", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>HST
+No Trade
+0.00
+score
+Price
+24.62
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+21.35
+Fib Zone
+21.22 - 21.48
+Swing Low
+20.71
+Swing High
+22.39
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_hst.png</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 24.62 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Host Hotels &amp; Resorts", "correlation_warning": false, "days_to_earnings": 37, "earnings_blackout": false, "earnings_date": "2026-07-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0739, "estimated_spread": 0.0197, "executable_entry": 24.62, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 24.62, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 16861728472.99, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 24.6668, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 24.7136, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0468, "net_target_1_assumption": -0.0283, "net_target_2_assumption": -0.0283, "normalized_atr_score": 100.0, "normalized_liquidity_score": 26.55, "normalized_momentum_score": 100, "normalized_quality_score": 77.97, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 24.62, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 24.62, "ticker": "HST", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>262.01</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>MPC
+No Trade
+0.00
+score
+Price
+262.01
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+245.05
+Fib Zone
+242.88 - 247.22
+Swing Low
+233.25
+Swing High
+264.14
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_mpc.png</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 262.01 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Marathon Petroleum Corporation", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3668, "estimated_spread": 0.0786, "executable_entry": 262.01, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 262.01, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 76490320587.29, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 262.2327, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 262.4554, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2227, "net_target_1_assumption": -0.131, "net_target_2_assumption": -0.131, "normalized_atr_score": 100.0, "normalized_liquidity_score": 52.86, "normalized_momentum_score": 100, "normalized_quality_score": 85.86, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 262.01, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 262.01, "ticker": "MPC", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" t="n">
+        <v>255.82</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>VLO
+No Trade
+0.00
+score
+Price
+255.82
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+240.05
+Fib Zone
+237.85 - 242.25
+Swing Low
+226.18
+Swing High
+262.50
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_vlo.png</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 255.82 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Energy | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Valero Energy Corporation", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3581, "estimated_spread": 0.0767, "executable_entry": 255.82, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 255.82, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 75961346466.04, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 256.0374, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 256.2549, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2174, "net_target_1_assumption": -0.1279, "net_target_2_assumption": -0.1279, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.08, "normalized_momentum_score": 100, "normalized_quality_score": 87.12, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 255.82, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 255.82, "ticker": "VLO", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>AMH</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" t="n">
+        <v>33.27</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>AMH
+No Trade
+0.00
+score
+Price
+33.27
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+28.73
+Fib Zone
+28.57 - 28.89
+Swing Low
+27.22
+Swing High
+31.18
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_amh.png</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 33.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "American Homes 4 Rent Common Shares of Beneficial Interest", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.0998, "estimated_spread": 0.0266, "executable_entry": 33.27, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 33.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 11997015510.91, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 33.3332, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 33.3964, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0632, "net_target_1_assumption": -0.0383, "net_target_2_assumption": -0.0383, "normalized_atr_score": 100.0, "normalized_liquidity_score": 17.57, "normalized_momentum_score": 99.67, "normalized_quality_score": 75.12, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 33.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 33.27, "ticker": "AMH", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>LAMR</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
+        <v>151.42</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>LAMR
+No Trade
+0.00
+score
+Price
+151.42
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+148.26
+Fib Zone
+147.52 - 149.00
+Swing Low
+144.11
+Swing High
+154.97
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_lamr.png</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 151.42 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Lamar Advertising Company", "correlation_warning": false, "days_to_earnings": 44, "earnings_blackout": false, "earnings_date": "2026-08-07T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4543, "estimated_spread": 0.1211, "executable_entry": 151.42, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 151.42, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 15365359607.61, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 151.7077, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 151.9954, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2877, "net_target_1_assumption": -0.1741, "net_target_2_assumption": -0.1741, "normalized_atr_score": 100.0, "normalized_liquidity_score": 16.68, "normalized_momentum_score": 90.76, "normalized_quality_score": 70.85, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 151.42, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 151.42, "ticker": "LAMR", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>IRM</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>124.66</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>IRM
+No Trade
+0.00
+score
+Price
+124.66
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+119.20
+Fib Zone
+118.31 - 120.10
+Swing Low
+110.00
+Swing High
+134.09
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_irm.png</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 124.66 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Iron Mountain", "correlation_warning": false, "days_to_earnings": -26, "earnings_blackout": false, "earnings_date": "2026-04-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.374, "estimated_spread": 0.0997, "executable_entry": 124.66, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 124.66, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 37089427823.03, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 124.8969, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 125.1337, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2369, "net_target_1_assumption": -0.1434, "net_target_2_assumption": -0.1434, "normalized_atr_score": 100.0, "normalized_liquidity_score": 24.67, "normalized_momentum_score": 100, "normalized_quality_score": 77.4, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 124.66, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 124.66, "ticker": "IRM", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ETN</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" t="n">
+        <v>395.94</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>ETN
+No Trade
+0.00
+score
+Price
+395.94
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+376.65
+Fib Zone
+372.93 - 380.37
+Swing Low
+341.06
+Swing High
+434.23
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_etn.png</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 395.94 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Eaton Corporation plc", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.5543, "estimated_spread": 0.1188, "executable_entry": 395.94, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 395.94, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 153743502948.0, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 396.2765, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 396.6131, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3365, "net_target_1_assumption": -0.198, "net_target_2_assumption": -0.198, "normalized_atr_score": 100.0, "normalized_liquidity_score": 67.34, "normalized_momentum_score": 89.3, "normalized_quality_score": 85.39, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 395.94, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 395.94, "ticker": "ETN", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SBAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>208.02</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>SBAC
+No Trade
+0.00
+score
+Price
+208.02
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+185.00
+Fib Zone
+183.45 - 186.54
+Swing Low
+161.43
+Swing High
+223.11
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_sbac.png</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Real Estate - Strong (70/100); XLRE sector regime is strong: 4.7% 3m return, -4.3% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 208.02 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Real Estate | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "SBA Communications", "correlation_warning": false, "days_to_earnings": -27, "earnings_blackout": false, "earnings_date": "2026-04-29T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6241, "estimated_spread": 0.1664, "executable_entry": 208.02, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Real Estate"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 208.02, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 22063229249.49, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 208.4152, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 208.8105, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3952, "net_target_1_assumption": -0.2392, "net_target_2_assumption": -0.2392, "normalized_atr_score": 100.0, "normalized_liquidity_score": 25.07, "normalized_momentum_score": 67.29, "normalized_quality_score": 62.8, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 208.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Real Estate", "sector_etf": "XLRE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.63, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 208.02, "ticker": "SBAC", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>326.27</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>CB
+No Trade
+0.00
+score
+Price
+326.27
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+50%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+325.36
+Fib Zone
+323.74 - 326.98
+Swing Low
+320.00
+Swing High
+334.03
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_cb.png</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 326.27 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Chubb Limited", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4568, "estimated_spread": 0.0979, "executable_entry": 326.27, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 326.27, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 126547112523.46, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 326.5473, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 326.8247, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2773, "net_target_1_assumption": -0.1631, "net_target_2_assumption": -0.1631, "normalized_atr_score": 100.0, "normalized_liquidity_score": 49.77, "normalized_momentum_score": 55.28, "normalized_quality_score": 64.81, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 326.27, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 326.27, "ticker": "CB", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BRK-B</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>488.13</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>BRK-B
+No Trade
+0.00
+score
+Price
+488.13
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+473.72
+Fib Zone
+471.94 - 475.50
+Swing Low
+464.01
+Swing High
+489.42
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_brk-b.png</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 488.13 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Berkshire Hathaway Inc.", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-08-01T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6834, "estimated_spread": 0.1464, "executable_entry": 488.13, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 488.13, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 1052825054461.12, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 488.5449, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 488.9598, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4149, "net_target_1_assumption": -0.2441, "net_target_2_assumption": -0.2441, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.88, "normalized_momentum_score": 47.83, "normalized_quality_score": 63.89, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 488.13, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 488.13, "ticker": "BRK-B", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>164.02</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>IT
+No Trade
+0.00
+score
+Price
+164.02
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+149.73
+Fib Zone
+147.69 - 151.76
+Swing Low
+140.56
+Swing High
+164.56
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_it.png</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 164.02 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Gartner", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4921, "estimated_spread": 0.1312, "executable_entry": 164.02, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 164.02, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 10981449119.83, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 164.3316, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 164.6433, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.3116, "net_target_1_assumption": -0.1886, "net_target_2_assumption": -0.1886, "normalized_atr_score": 100.0, "normalized_liquidity_score": 34.64, "normalized_momentum_score": 51.77, "normalized_quality_score": 58.69, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 164.02, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 164.02, "ticker": "IT", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="n">
+        <v>232.77</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>JNJ
+No Trade
+0.00
+score
+Price
+232.77
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+224.86
+Fib Zone
+223.76 - 225.95
+Swing Low
+219.11
+Swing High
+234.15
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_jnj.png</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 232.77 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Johnson &amp; Johnson", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3259, "estimated_spread": 0.0698, "executable_entry": 232.77, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 232.77, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 560327904624.41, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 232.9679, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 233.1657, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1979, "net_target_1_assumption": -0.1164, "net_target_2_assumption": -0.1164, "normalized_atr_score": 100.0, "normalized_liquidity_score": 48.96, "normalized_momentum_score": 45.75, "normalized_quality_score": 60.28, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 232.77, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 232.77, "ticker": "JNJ", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" t="n">
+        <v>346.44</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>GD
+No Trade
+0.00
+score
+Price
+346.44
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+In line
+47%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+340.19
+Fib Zone
+338.55 - 341.84
+Swing Low
+333.29
+Swing High
+351.36
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_gd.png</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 346.44 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "General Dynamics Corporation", "correlation_warning": false, "days_to_earnings": 32, "earnings_blackout": false, "earnings_date": "2026-07-22T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.0393, "estimated_spread": 0.2772, "executable_entry": 346.44, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 346.44, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 93687834644.51, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 347.0982, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 347.7565, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.6582, "net_target_1_assumption": -0.3984, "net_target_2_assumption": -0.3984, "normalized_atr_score": 100.0, "normalized_liquidity_score": 39.95, "normalized_momentum_score": 37.08, "normalized_quality_score": 53.67, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 346.44, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 346.44, "ticker": "GD", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
+        <v>583.4400000000001</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>DE
+No Trade
+0.00
+score
+Price
+583.44
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+571.60
+Fib Zone
+567.30 - 575.90
+Swing Low
+557.76
+Swing High
+593.98
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_de.png</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 583.44 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Deere &amp; Company", "correlation_warning": false, "days_to_earnings": 53, "earnings_blackout": false, "earnings_date": "2026-08-20T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.8168, "estimated_spread": 0.175, "executable_entry": 583.44, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 583.44, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 157492291901.03, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 583.9359, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 584.4318, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4959, "net_target_1_assumption": -0.2917, "net_target_2_assumption": -0.2917, "normalized_atr_score": 100.0, "normalized_liquidity_score": 62.19, "normalized_momentum_score": 43.15, "normalized_quality_score": 63.07, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 583.44, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 583.44, "ticker": "DE", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>WFC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" t="n">
+        <v>81.94</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>WFC
+No Trade
+0.00
+score
+Price
+81.94
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Neutral
+65%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+78.42
+Fib Zone
+77.95 - 78.90
+Swing Low
+73.61
+Swing High
+86.21
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_wfc.png</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 81.94 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Wells Fargo &amp; Company", "correlation_warning": false, "days_to_earnings": 26, "earnings_blackout": false, "earnings_date": "2026-07-14T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1147, "estimated_spread": 0.0246, "executable_entry": 81.94, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 81.94, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 250751934609.53, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 82.0096, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 82.0793, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0696, "net_target_1_assumption": -0.041, "net_target_2_assumption": -0.041, "normalized_atr_score": 100.0, "normalized_liquidity_score": 42.84, "normalized_momentum_score": 72.91, "normalized_quality_score": 70.66, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 81.94, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 81.94, "ticker": "WFC", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>349.58</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>AMGN
+No Trade
+0.00
+score
+Price
+349.58
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+327.93
+Fib Zone
+325.90 - 329.96
+Swing Low
+318.12
+Swing High
+343.80
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_amgn.png</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 349.58 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Amgen Inc.", "correlation_warning": false, "days_to_earnings": 41, "earnings_blackout": false, "earnings_date": "2026-08-04T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4894, "estimated_spread": 0.1049, "executable_entry": 349.58, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 349.58, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 188671211177.86, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 349.8771, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 350.1743, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2971, "net_target_1_assumption": -0.1748, "net_target_2_assumption": -0.1748, "normalized_atr_score": 100.0, "normalized_liquidity_score": 60.83, "normalized_momentum_score": 40.24, "normalized_quality_score": 61.36, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 349.58, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 349.58, "ticker": "AMGN", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" t="n">
+        <v>185.66</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>CRM
+No Trade
+0.00
+score
+Price
+185.66
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Clean uptrend
+86%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+173.16
+Fib Zone
+170.76 - 175.56
+Swing Low
+164.33
+Swing High
+187.44
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_crm.png</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Technology - Strong (76/100); XLK sector regime is strong: 29.2% 3m return, 20.1% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 185.66 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Technology | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Salesforce, Inc.", "correlation_warning": false, "days_to_earnings": 62, "earnings_blackout": false, "earnings_date": "2026-09-02T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2599, "estimated_spread": 0.0557, "executable_entry": 185.66, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Technology"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 185.66, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 152055542999.27, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 185.8178, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 185.9756, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1578, "net_target_1_assumption": -0.0928, "net_target_2_assumption": -0.0928, "normalized_atr_score": 100.0, "normalized_liquidity_score": 98.07, "normalized_momentum_score": 29.03, "normalized_quality_score": 67.48, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 185.66, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Technology", "sector_etf": "XLK", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 76.23, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 185.66, "ticker": "CRM", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>BLK</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" t="n">
+        <v>995.6</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>BLK
+No Trade
+0.00
+score
+Price
+995.60
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+30%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+1045.24
+Fib Zone
+1038.79 - 1051.69
+Swing Low
+1024.42
+Swing High
+1078.92
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_blk.png</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 995.60 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "BlackRock, Inc.", "correlation_warning": false, "days_to_earnings": 27, "earnings_blackout": false, "earnings_date": "2026-07-15T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 1.3938, "estimated_spread": 0.2987, "executable_entry": 995.6, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 995.6, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 154550955658.51, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 996.4463, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 997.2925, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.8463, "net_target_1_assumption": -0.4978, "net_target_2_assumption": -0.4978, "normalized_atr_score": 100.0, "normalized_liquidity_score": 57.27, "normalized_momentum_score": 54.58, "normalized_quality_score": 66.74, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 995.6, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 995.6, "ticker": "BLK", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" t="n">
+        <v>81.67</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>MDT
+No Trade
+0.00
+score
+Price
+81.67
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+58%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+76.25
+Fib Zone
+75.75 - 76.75
+Swing Low
+74.40
+Swing High
+79.25
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_mdt.png</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Healthcare - Neutral (66/100); XLV sector regime is neutral: -0.4% 3m return, -9.4% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 81.67 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Defensive, Healthcare | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Medtronic plc", "correlation_warning": false, "days_to_earnings": 51, "earnings_blackout": false, "earnings_date": "2026-08-18T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.1143, "estimated_spread": 0.0245, "executable_entry": 81.67, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Defensive", "Healthcare"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 81.67, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 104854882659.02, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 81.7394, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 81.8088, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.0694, "net_target_1_assumption": -0.0408, "net_target_2_assumption": -0.0408, "normalized_atr_score": 100.0, "normalized_liquidity_score": 64.58, "normalized_momentum_score": 26.07, "normalized_quality_score": 56.11, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 81.67, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Healthcare", "sector_etf": "XLV", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 65.79, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 81.67, "ticker": "MDT", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" t="n">
+        <v>491.08</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>MA
+No Trade
+0.00
+score
+Price
+491.08
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+84%
+Trend Quality
+Messy
+0%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+85%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+497.52
+Fib Zone
+494.61 - 500.43
+Swing Low
+488.01
+Swing High
+512.90
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_ma.png</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 491.08 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 0.00; Factors: Financials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Mastercard Incorporated", "correlation_warning": false, "days_to_earnings": 38, "earnings_blackout": false, "earnings_date": "2026-07-30T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.6875, "estimated_spread": 0.1473, "executable_entry": 491.08, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 491.08, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 433910347648.87, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 491.4974, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 491.9148, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.4174, "net_target_1_assumption": -0.2455, "net_target_2_assumption": -0.2455, "normalized_atr_score": 100.0, "normalized_liquidity_score": 49.93, "normalized_momentum_score": 28.91, "normalized_quality_score": 52.99, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 491.08, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector STRONG; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 491.08, "ticker": "MA", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>EMR</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" t="n">
+        <v>138.12</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>EMR
+No Trade
+0.00
+score
+Price
+138.12
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Constructive
+68%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Confirmed
+80%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+134.79
+Fib Zone
+133.80 - 135.78
+Swing Low
+128.13
+Swing High
+145.57
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_emr.png</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 138.12 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Emerson Electric Co.", "correlation_warning": false, "days_to_earnings": 42, "earnings_blackout": false, "earnings_date": "2026-08-05T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.4144, "estimated_spread": 0.1105, "executable_entry": 138.12, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 138.12, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 77361009265.14, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 138.3824, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 138.6449, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.2624, "net_target_1_assumption": -0.1588, "net_target_2_assumption": -0.1588, "normalized_atr_score": 100.0, "normalized_liquidity_score": 41.05, "normalized_momentum_score": 41.73, "normalized_quality_score": 56.09, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 138.12, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 138.12, "ticker": "EMR", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>No Trade</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" t="n">
+        <v>215.45</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>No clean technical setup detected. Price in middle of value area or poor risk/reward.</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>BA
+No Trade
+0.00
+score
+Price
+215.45
+R/R
+0.00x
+Grade
+No Trade
+Quality
+0%
+Buy Zone
+-
+Stop
+0.00
+Targets
+-
+Skip
+Mixed
+Relative Strength
+Leadership
+100%
+Trend Quality
+Messy
+18%
+Liquidity
+Institutional liquidity
+100%
+Volume
+Distribution risk
+45%
+No actionable setup detected.
+No clean technical setup detected. Price in middle of value area or poor risk/reward.
+Fib 61.8
+220.99
+Fib Zone
+219.16 - 222.82
+Swing Low
+214.00
+Swing High
+232.30
+Click chart to open full size</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_013140_ba.png</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Industrials - Neutral (67/100); XLI sector regime is neutral: 2.2% 3m return, -6.9% vs SPY | Setup: No Trade; score 0.00; R/R 0.00x; price 215.45 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 0.00; Factors: Industrials | Agent action: SKIP - SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": null, "buy_zone_low": null, "cash_available": 100000.0, "company_name": "Boeing Company", "correlation_warning": false, "days_to_earnings": 36, "earnings_blackout": false, "earnings_date": "2026-07-28T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3016, "estimated_spread": 0.0646, "executable_entry": 215.45, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {}, "factor_exposure_before": {}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Industrials"], "final_action": "SKIP", "gross_reward_1_per_share": 0.0, "gross_reward_2_per_share": 0.0, "gross_risk_per_share": 215.45, "gross_rr": 0.0, "gross_rr_1": 0.0, "gross_rr_2": 0.0, "gross_rr_decision": 0.0, "highest_correlation_ticker": "", "highest_correlation_value": null, "initial_action": "SKIP", "market_cap": 169839734808.24, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2284, "ema200": 98.8017, "ema50": 98.9549, "price": 100.134, "return_1m": 2.34, "return_3m": 1.32, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "UNKNOWN", "net_entry": 215.6331, "net_reward_1_per_share": 0.0, "net_reward_2_per_share": 0.0, "net_risk_per_share": 215.8163, "net_rr": 0.0, "net_rr_1": 0.0, "net_rr_2": 0.0, "net_stop_assumption": -0.1831, "net_target_1_assumption": -0.1077, "net_target_2_assumption": -0.1077, "normalized_atr_score": 100.0, "normalized_liquidity_score": 82.1, "normalized_momentum_score": 25.63, "normalized_quality_score": 61.16, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 0, "portfolio_exposure_before": 0, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 0.0, "price": 215.45, "prior_high_20": 0.0, "prior_high_63": 0.0, "reason": "SKIP: No Trade result. Market regime NEUTRAL; sector NEUTRAL; net R/R 0.00.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Industrials", "sector_etf": "XLI", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 66.69, "setup_score": 0.0, "setup_type": "No Trade", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.0, "stop_loss": 0.0, "target_1": null, "target_1_atr_distance": 0.0, "target_2": null, "target_2_atr_distance": 0.0, "target_feasibility_status": "UNKNOWN", "theoretical_entry": 215.45, "ticker": "BA", "timestamp": "2026-06-08T01:37:33", "warnings": ["Target ATR feasibility unavailable."]}</t>
         </is>
       </c>
     </row>
@@ -8745,7 +12701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="52" min="1" max="1"/>
@@ -8924,6 +12880,58 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>C:\Users\User\Documents\Codex\2026-05-29\adva-mo-project-orion-https-github\work\market-lens-scanner\agent_results\decisions\market_lens_agent_20260608_010748.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:37:33</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>20260608_013140</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OKE XOM V CVX ELAN MSFT AIG BKR COP AXP DHR PFE DLR HST MPC VLO AMH LAMR IRM ETN SBAC CB BRK-B IT JNJ GD DE WFC AMGN CRM BLK MDT MA EMR BA</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OKE:WATCH, XOM:WATCH, V:WATCH, CVX:WATCH, ELAN:WATCH, MSFT:WATCH, AIG:WATCH, BKR:WATCH, COP:WATCH, AXP:WATCH, DHR:WATCH, PFE:WATCH, DLR:WATCH, HST:SKIP, MPC:SKIP, VLO:SKIP, AMH:SKIP, LAMR:SKIP, IRM:SKIP, ETN:SKIP, SBAC:SKIP, CB:SKIP, BRK-B:SKIP, IT:SKIP, JNJ:SKIP, GD:SKIP, DE:SKIP, WFC:SKIP, AMGN:SKIP, CRM:SKIP, BLK:SKIP, MDT:SKIP, MA:SKIP, EMR:SKIP, BA:SKIP</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>agent_results\summaries\market_lens_agent_20260608_013140.md</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260608_013140.png</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>agent_results\decisions\market_lens_agent_20260608_013140.jsonl</t>
         </is>
       </c>
     </row>
@@ -9401,6 +13409,7 @@
       <c r="C1" s="21" t="n"/>
       <c r="D1" s="21" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="55" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Harden market lens automations
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -22804,7 +22804,7 @@
         <v>149.92</v>
       </c>
       <c r="D2" t="n">
-        <v>149.92</v>
+        <v>150.02</v>
       </c>
       <c r="E2" t="n">
         <v>40</v>
@@ -22824,16 +22824,16 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>5996.8</v>
+        <v>6000.8</v>
       </c>
       <c r="M2" t="n">
-        <v>117.2</v>
+        <v>121.2</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -22876,7 +22876,7 @@
         <v>132.14</v>
       </c>
       <c r="D3" t="n">
-        <v>132.14</v>
+        <v>132.12</v>
       </c>
       <c r="E3" t="n">
         <v>45</v>
@@ -22896,16 +22896,16 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>-0.9</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>-0.9</v>
       </c>
       <c r="L3" t="n">
-        <v>5946.3</v>
+        <v>5945.4</v>
       </c>
       <c r="M3" t="n">
-        <v>29.7</v>
+        <v>28.8</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -22947,7 +22947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="52" min="1" max="1"/>
@@ -23284,6 +23284,49 @@
           <t>agent_results\decisions\market_lens_agent_20260608_092643.jsonl</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:45:35+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>monitor_20260608_064535</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>XOM HIG</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MONITOR:HOLD</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>88056.89999999999</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11946.2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>150</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>agent_results\position_monitor\position_monitor_20260608_064535.md</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Market Lens position monitor
</commit_message>
<xml_diff>
--- a/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
+++ b/agent_tracker/market_lens_agent_portfolio_budget_100k.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Position Events" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Setup Watchlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Trade Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Open Positions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Update Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Agent Control" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Position Events" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -22389,7 +22389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -22663,6 +22663,156 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-08T14:04:49+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TAKE_PARTIAL_PROFIT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>150.49</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3009.8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>3009.8</v>
+      </c>
+      <c r="L4" t="n">
+        <v>146.99</v>
+      </c>
+      <c r="M4" t="n">
+        <v>150.49</v>
+      </c>
+      <c r="N4" t="n">
+        <v>173.86</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Target 1 touched by intraday high; taking partial profit and moving stop to breakeven.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260608_091643.png</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_092643_xom.png</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Energy - Neutral (48/100); XLE sector regime is neutral: 3.1% 3m return, -6.0% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.49; R/R 2.98x; price 149.92 | Market: NEUTRAL; Sector regime: NEUTRAL; Net R/R: 2.68; Factors: Energy | Agent action: HOLD - HOLD: Existing simulated position remains open. NEUTRAL regime recorded.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 151.87, "buy_zone_low": 149.87, "cash_available": 88056.9, "company_name": "Exxon Mobil Corporation", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-07-31T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2099, "estimated_spread": 0.045, "executable_entry": 149.92, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {"Financials": 5946.3}, "factor_exposure_before": {"Financials": 5946.3}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "HOLD", "gross_reward_1_per_share": 0.57, "gross_reward_2_per_share": 23.94, "gross_risk_per_share": 2.93, "gross_rr": 2.9862, "gross_rr_1": 0.1945, "gross_rr_2": 8.1706, "gross_rr_decision": 2.9862, "highest_correlation_ticker": "HIG", "highest_correlation_value": -0.0856, "initial_action": "HOLD", "market_cap": 621410470937.42, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2236, "ema200": 98.8009, "ema50": 98.9529, "price": 100.084, "return_1m": 2.29, "return_3m": 1.27, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "minimum_net_rr_required": 2.5, "net_entry": 150.0474, "net_reward_1_per_share": 0.3676, "net_reward_2_per_share": 23.7376, "net_risk_per_share": 3.1849, "net_rr": 2.6837, "net_rr_1": 0.1154, "net_rr_2": 7.4533, "net_stop_assumption": 146.8626, "net_target_1_assumption": 150.415, "net_target_2_assumption": 173.785, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.97, "normalized_momentum_score": 55.95, "normalized_quality_score": 67.87, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 11943.1, "portfolio_exposure_before": 11943.1, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 163.68, "price": 149.92, "prior_high_20": 163.68, "prior_high_63": 175.2207, "reason": "HOLD: Existing simulated position remains open. NEUTRAL regime recorded.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.49, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.49, "stop_loss": 146.99, "target_1": 150.49, "target_1_atr_distance": 0.1428, "target_2": 173.86, "target_2_atr_distance": 5.9956, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 149.87, "ticker": "XOM", "timestamp": "2026-06-08T09:33:45", "warnings": ["Target 1 is close versus daily ATR."]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-08T14:04:49+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EXIT_STOP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HIG</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>131.48</v>
+      </c>
+      <c r="F5" t="n">
+        <v>45</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5916.6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5916.6</v>
+      </c>
+      <c r="L5" t="n">
+        <v>131.48</v>
+      </c>
+      <c r="M5" t="n">
+        <v>133.49</v>
+      </c>
+      <c r="N5" t="n">
+        <v>139.89</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Stop loss touched by intraday low.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>agent_results\screenshots\market_lens_agent_20260608_092643.png</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>agent_results\charts\market_lens_agent_20260608_092643_hig.png</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.51; R/R 5.41x; price 132.14 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 2.74; Factors: Financials | Agent action: BUY_SIMULATED - BUY_SIMULATED: NEUTRAL market regime, STRONG sector, valid setup, net R/R 2.74, no earnings blackout, correlation acceptable, and risk limits allow entry. Position size reduced to 45 shares to fit exposure caps.</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>{"adjusted_cash_out": 5946.3, "adjusted_position_size": 45, "adjusted_risk_amount": 29.7, "ask": 0.0, "bid": 0.0, "buy_zone_high": 133.48, "buy_zone_low": 132.07, "cash_available": 94003.2, "company_name": "Hartford (The)", "correlation_warning": false, "days_to_earnings": -32, "earnings_blackout": false, "earnings_date": "2026-04-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3964, "estimated_spread": 0.1057, "executable_entry": 132.14, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {"Energy": 5996.8, "Financials": 5946.3}, "factor_exposure_before": {"Energy": 5996.8}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "BUY_SIMULATED", "gross_reward_1_per_share": 1.35, "gross_reward_2_per_share": 7.75, "gross_risk_per_share": 0.66, "gross_rr": 5.4394, "gross_rr_1": 2.0455, "gross_rr_2": 11.7424, "gross_rr_decision": 5.4394, "highest_correlation_ticker": "XOM", "highest_correlation_value": -0.0856, "initial_action": "BUY_SIMULATED", "market_cap": 36223646387.48, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2236, "ema200": 98.8009, "ema50": 98.9529, "price": 100.084, "return_1m": 2.29, "return_3m": 1.27, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "minimum_net_rr_required": 2.2, "net_entry": 132.3911, "net_reward_1_per_share": 0.947, "net_reward_2_per_share": 7.347, "net_risk_per_share": 1.1621, "net_rr": 2.7424, "net_rr_1": 0.8149, "net_rr_2": 6.322, "net_stop_assumption": 131.2289, "net_target_1_assumption": 133.338, "net_target_2_assumption": 139.738, "normalized_atr_score": 100.0, "normalized_liquidity_score": 31.03, "normalized_momentum_score": 38.09, "normalized_quality_score": 51.45, "original_cash_out": 9910.5, "original_position_size": 75, "original_risk_amount": 49.5, "portfolio_exposure_after": 11943.1, "portfolio_exposure_before": 5996.8, "position_size": 45, "position_size_adjusted": true, "position_sizing_explanation": "Position size reduced from 75 to 45 shares. Accepted cash out 5946.30, risk 29.70. Reason: Position size reduced by Financials sector exposure cap (75 -&gt; 45 shares).", "previous_resistance": 136.5226, "price": 132.14, "prior_high_20": 136.5226, "prior_high_63": 140.9417, "reason": "BUY_SIMULATED: NEUTRAL market regime, STRONG sector, valid setup, net R/R 2.74, no earnings blackout, correlation acceptable, and risk limits allow entry. Position size reduced to 45 shares to fit exposure caps.", "risk_amount": 29.7, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 5946.3, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.51, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "Position size reduced by Financials sector exposure cap (75 -&gt; 45 shares).", "spread_source": "liquidity_fallback", "stock_score": 0.51, "stop_loss": 131.48, "target_1": 133.49, "target_1_atr_distance": 0.478, "target_2": 139.89, "target_2_atr_distance": 2.7441, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 132.07, "ticker": "HIG", "timestamp": "2026-06-08T09:33:45", "warnings": ["Target 1 is close versus daily ATR.", "Position size reduced by Financials sector exposure cap (75 -&gt; 45 shares)."]}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -22677,7 +22827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="52" min="1" max="1"/>
@@ -22804,13 +22954,13 @@
         <v>149.92</v>
       </c>
       <c r="D2" t="n">
-        <v>150.02</v>
+        <v>150.49</v>
       </c>
       <c r="E2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F2" t="n">
-        <v>146.99</v>
+        <v>149.92</v>
       </c>
       <c r="G2" t="n">
         <v>150.49</v>
@@ -22824,20 +22974,20 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>4</v>
+        <v>11.4</v>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>11.4</v>
       </c>
       <c r="L2" t="n">
-        <v>6000.8</v>
+        <v>3009.8</v>
       </c>
       <c r="M2" t="n">
-        <v>121.2</v>
+        <v>11.4</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY_SIMULATED: NEUTRAL market regime, NEUTRAL sector, valid setup, net R/R 2.68, no earnings blackout, correlation acceptable, and risk limits allow entry. Position size reduced to 40 shares to fit exposure caps.</t>
+          <t>Partial profit taken; stop moved to breakeven.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -22858,78 +23008,6 @@
       <c r="R2" t="inlineStr">
         <is>
           <t>{"adjusted_cash_out": 0.0, "adjusted_position_size": 0, "adjusted_risk_amount": 0.0, "ask": 0.0, "bid": 0.0, "buy_zone_high": 151.87, "buy_zone_low": 149.87, "cash_available": 88056.9, "company_name": "Exxon Mobil Corporation", "correlation_warning": false, "days_to_earnings": 39, "earnings_blackout": false, "earnings_date": "2026-07-31T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.2099, "estimated_spread": 0.045, "executable_entry": 149.92, "execution_liquidity_bucket": "large_liquid", "factor_exposure_after": {"Financials": 5946.3}, "factor_exposure_before": {"Financials": 5946.3}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Energy"], "final_action": "HOLD", "gross_reward_1_per_share": 0.57, "gross_reward_2_per_share": 23.94, "gross_risk_per_share": 2.93, "gross_rr": 2.9862, "gross_rr_1": 0.1945, "gross_rr_2": 8.1706, "gross_rr_decision": 2.9862, "highest_correlation_ticker": "HIG", "highest_correlation_value": -0.0856, "initial_action": "HOLD", "market_cap": 621410470937.42, "market_cap_bucket": "Mega Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2236, "ema200": 98.8009, "ema50": 98.9529, "price": 100.084, "return_1m": 2.29, "return_3m": 1.27, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "minimum_net_rr_required": 2.5, "net_entry": 150.0474, "net_reward_1_per_share": 0.3676, "net_reward_2_per_share": 23.7376, "net_risk_per_share": 3.1849, "net_rr": 2.6837, "net_rr_1": 0.1154, "net_rr_2": 7.4533, "net_stop_assumption": 146.8626, "net_target_1_assumption": 150.415, "net_target_2_assumption": 173.785, "normalized_atr_score": 100.0, "normalized_liquidity_score": 58.97, "normalized_momentum_score": 55.95, "normalized_quality_score": 67.87, "original_cash_out": 0.0, "original_position_size": 0, "original_risk_amount": 0.0, "portfolio_exposure_after": 11943.1, "portfolio_exposure_before": 11943.1, "position_size": 0, "position_size_adjusted": false, "position_sizing_explanation": "No new position size was calculated because the base decision did not open a simulated buy.", "previous_resistance": 163.68, "price": 149.92, "prior_high_20": 163.68, "prior_high_63": 175.2207, "reason": "HOLD: Existing simulated position remains open. NEUTRAL regime recorded.", "risk_amount": 0.0, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Energy", "sector_etf": "XLE", "sector_exposure_after": 0.0, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "NEUTRAL", "sector_score": 47.51, "setup_score": 0.49, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "", "spread_source": "liquidity_fallback", "stock_score": 0.49, "stop_loss": 146.99, "target_1": 150.49, "target_1_atr_distance": 0.1428, "target_2": 173.86, "target_2_atr_distance": 5.9956, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 149.87, "ticker": "XOM", "timestamp": "2026-06-08T09:33:45", "warnings": ["Target 1 is close versus daily ATR."]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HIG</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-08T09:33:45</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>132.14</v>
-      </c>
-      <c r="D3" t="n">
-        <v>132.12</v>
-      </c>
-      <c r="E3" t="n">
-        <v>45</v>
-      </c>
-      <c r="F3" t="n">
-        <v>131.48</v>
-      </c>
-      <c r="G3" t="n">
-        <v>133.49</v>
-      </c>
-      <c r="H3" t="n">
-        <v>139.89</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>-0.9</v>
-      </c>
-      <c r="K3" t="n">
-        <v>-0.9</v>
-      </c>
-      <c r="L3" t="n">
-        <v>5945.4</v>
-      </c>
-      <c r="M3" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>BUY_SIMULATED: NEUTRAL market regime, STRONG sector, valid setup, net R/R 2.74, no earnings blackout, correlation acceptable, and risk limits allow entry. Position size reduced to 45 shares to fit exposure caps.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>agent_results\screenshots\market_lens_agent_20260608_092643.png</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>agent_results\charts\market_lens_agent_20260608_092643_hig.png</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Smart Universe: broad liquid US universe, diversified by sector | Sector: Financials - Strong (70/100); XLF sector regime is strong: 4.4% 3m return, -4.6% vs SPY | Setup: Fib 61.8 Confluence Buy Zone; score 0.51; R/R 5.41x; price 132.14 | Market: NEUTRAL; Sector regime: STRONG; Net R/R: 2.74; Factors: Financials | Agent action: BUY_SIMULATED - BUY_SIMULATED: NEUTRAL market regime, STRONG sector, valid setup, net R/R 2.74, no earnings blackout, correlation acceptable, and risk limits allow entry. Position size reduced to 45 shares to fit exposure caps.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>{"adjusted_cash_out": 5946.3, "adjusted_position_size": 45, "adjusted_risk_amount": 29.7, "ask": 0.0, "bid": 0.0, "buy_zone_high": 133.48, "buy_zone_low": 132.07, "cash_available": 94003.2, "company_name": "Hartford (The)", "correlation_warning": false, "days_to_earnings": -32, "earnings_blackout": false, "earnings_date": "2026-04-23T00:00:00", "estimated_fees": 0.0, "estimated_slippage": 0.3964, "estimated_spread": 0.1057, "executable_entry": 132.14, "execution_liquidity_bucket": "mid_liquid", "factor_exposure_after": {"Energy": 5996.8, "Financials": 5946.3}, "factor_exposure_before": {"Energy": 5996.8}, "factor_exposure_cap": 7000.0, "factor_exposure_limit_exceeded": false, "factor_tags": ["Financials"], "final_action": "BUY_SIMULATED", "gross_reward_1_per_share": 1.35, "gross_reward_2_per_share": 7.75, "gross_risk_per_share": 0.66, "gross_rr": 5.4394, "gross_rr_1": 2.0455, "gross_rr_2": 11.7424, "gross_rr_decision": 5.4394, "highest_correlation_ticker": "XOM", "highest_correlation_value": -0.0856, "initial_action": "BUY_SIMULATED", "market_cap": 36223646387.48, "market_cap_bucket": "Large Cap", "market_regime": "NEUTRAL", "market_regime_indicators": {"DXY": {"ema20": 99.2236, "ema200": 98.8009, "ema50": 98.9529, "price": 100.084, "return_1m": 2.29, "return_3m": 1.27, "trend": "bullish"}, "IWM": {"ema20": 284.8339, "ema200": 266.8273, "ema50": 276.8465, "price": 281.65, "return_1m": -0.22, "return_3m": 11.25, "trend": "mixed"}, "QQQ": {"ema20": 717.5737, "ema200": 649.8326, "ema50": 683.0818, "price": 705.06, "return_1m": 1.46, "return_3m": 16.16, "trend": "mixed"}, "SPY": {"ema20": 743.679, "ema200": 702.3249, "ema50": 723.0899, "price": 737.55, "return_1m": 0.82, "return_3m": 9.04, "trend": "mixed"}, "US10Y": {"ema20": 4.482, "ema200": 4.307, "ema50": 4.4111, "price": 4.536, "return_1m": 3.28, "return_3m": 9.67, "trend": "bullish"}, "VIX": {"ema20": 17.2086, "ema200": 18.6108, "ema50": 18.3779, "price": 21.51, "return_1m": 25.13, "return_3m": -13.72, "trend": "mixed"}}, "market_regime_reason": "Market regime is mixed; use lower exposure and higher net R/R.", "market_regime_score": 0.52, "market_structure_status": "SUPPORTED_BY_20D_RESISTANCE", "minimum_net_rr_required": 2.2, "net_entry": 132.3911, "net_reward_1_per_share": 0.947, "net_reward_2_per_share": 7.347, "net_risk_per_share": 1.1621, "net_rr": 2.7424, "net_rr_1": 0.8149, "net_rr_2": 6.322, "net_stop_assumption": 131.2289, "net_target_1_assumption": 133.338, "net_target_2_assumption": 139.738, "normalized_atr_score": 100.0, "normalized_liquidity_score": 31.03, "normalized_momentum_score": 38.09, "normalized_quality_score": 51.45, "original_cash_out": 9910.5, "original_position_size": 75, "original_risk_amount": 49.5, "portfolio_exposure_after": 11943.1, "portfolio_exposure_before": 5996.8, "position_size": 45, "position_size_adjusted": true, "position_sizing_explanation": "Position size reduced from 75 to 45 shares. Accepted cash out 5946.30, risk 29.70. Reason: Position size reduced by Financials sector exposure cap (75 -&gt; 45 shares).", "previous_resistance": 136.5226, "price": 132.14, "prior_high_20": 136.5226, "prior_high_63": 140.9417, "reason": "BUY_SIMULATED: NEUTRAL market regime, STRONG sector, valid setup, net R/R 2.74, no earnings blackout, correlation acceptable, and risk limits allow entry. Position size reduced to 45 shares to fit exposure caps.", "risk_amount": 29.7, "scan_source": "Smart Universe: broad liquid US universe filtered and diversified by the Market Lens UI.", "sector": "Financials", "sector_etf": "XLF", "sector_exposure_after": 5946.3, "sector_exposure_before": 0.0, "sector_exposure_cap": 6000.0, "sector_exposure_limit_exceeded": false, "sector_regime": "STRONG", "sector_score": 69.62, "setup_score": 0.51, "setup_type": "Fib 61.8 Confluence Buy Zone", "sizing_adjustment_reason": "Position size reduced by Financials sector exposure cap (75 -&gt; 45 shares).", "spread_source": "liquidity_fallback", "stock_score": 0.51, "stop_loss": 131.48, "target_1": 133.49, "target_1_atr_distance": 0.478, "target_2": 139.89, "target_2_atr_distance": 2.7441, "target_feasibility_status": "LOW_REWARD_DISTANCE", "theoretical_entry": 132.07, "ticker": "HIG", "timestamp": "2026-06-08T09:33:45", "warnings": ["Target 1 is close versus daily ATR.", "Position size reduced by Financials sector exposure cap (75 -&gt; 45 shares)."]}</t>
         </is>
       </c>
     </row>
@@ -22947,7 +23025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="52" min="1" max="1"/>
@@ -23326,7 +23404,49 @@
           <t>agent_results\position_monitor\position_monitor_20260608_064535.md</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-08T14:04:49+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>monitor_20260608_140449</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>XOM:TAKE_PARTIAL_PROFIT, HIG:EXIT_STOP</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>96983.3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3009.8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>agent_results/position_monitor/position_monitor_20260608_140449.md</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24034,7 +24154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24114,6 +24234,124 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-08T14:04:49+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>20260608_140449</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TAKE_PARTIAL_PROFIT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-06-08T13:30:00+00:00</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>150.49</v>
+      </c>
+      <c r="G2" t="n">
+        <v>151.345</v>
+      </c>
+      <c r="H2" t="n">
+        <v>151.11</v>
+      </c>
+      <c r="I2" t="n">
+        <v>151.11</v>
+      </c>
+      <c r="J2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K2" t="n">
+        <v>3009.8</v>
+      </c>
+      <c r="L2" t="n">
+        <v>146.99</v>
+      </c>
+      <c r="M2" t="n">
+        <v>150.49</v>
+      </c>
+      <c r="N2" t="n">
+        <v>173.86</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Target 1 touched by intraday high; taking partial profit and moving stop to breakeven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-08T14:04:49+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>20260608_140449</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>HIG</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EXIT_STOP</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-06-08T13:30:00+00:00</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>131.48</v>
+      </c>
+      <c r="G3" t="n">
+        <v>130.75</v>
+      </c>
+      <c r="H3" t="n">
+        <v>130.385</v>
+      </c>
+      <c r="I3" t="n">
+        <v>130.53</v>
+      </c>
+      <c r="J3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5916.6</v>
+      </c>
+      <c r="L3" t="n">
+        <v>131.48</v>
+      </c>
+      <c r="M3" t="n">
+        <v>133.49</v>
+      </c>
+      <c r="N3" t="n">
+        <v>139.89</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Stop loss touched by intraday low.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>